<commit_message>
feat(arquitectura): estructurar Resumen de Arquitectura y Fichas con Que es, Lead text y Base juridica formal
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa de Navegación" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descripciones y Base Legal" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Arquitectura" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapa de Navegación" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas por Rol y Categoría" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Descripciones y Base Legal'!$A$6:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fichas por Rol y Categoría'!$A$6:$H$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,13 +33,49 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <i val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -56,18 +93,8 @@
       <color rgb="00475569"/>
       <sz val="8"/>
     </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="001E293B"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +111,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="0014649B"/>
         <bgColor rgb="0014649B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000284C7"/>
+        <bgColor rgb="000284C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00059669"/>
+        <bgColor rgb="00059669"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007C3AED"/>
+        <bgColor rgb="007C3AED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -115,6 +166,20 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="00FFFFFF"/>
       </left>
       <right style="thin">
@@ -127,25 +192,11 @@
         <color rgb="00FFFFFF"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -153,41 +204,88 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -555,6 +653,330 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>SUPERINTENDENCIA DE ADMINISTRACIÓN TRIBUTARIA — SAT GUATEMALA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>RESUMEN EJECUTIVO DE ARQUITECTURA DE INFORMACIÓN — DEFINICIÓN DE SEGMENTOS, LEAD TEXT Y BASE JURÍDICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL DEL PORTAL
+739 Trámites</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>CONTRIBUYENTES
+413 Trámites</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>COMERCIO EXTERIOR
+202 Trámites</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>PROFESIONALES
+45 Trámites</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>ENTES EXENTOS
+79 Trámites</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="9">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>1. RESUMEN ESTRUCTURAL POR SEGMENTO (NIVEL 1) — DEFINICIONES INSTITUCIONALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OPERADORES DE COMERCIO EXTERIOR  (202 Trámites — 27.3% del Portal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Qué es:</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Son todas las personas individuales o jurídicas que intervienen en el ingreso, permanencia, traslado y salida de mercancías del territorio aduanero nacional. Comprende tanto a los dueños de las mercancías (importadores y exportadores) como a los prestadores de servicios logísticos autorizados (auxiliares de la función pública, transportistas, depósitos) y empresas que operan bajo regímenes territoriales especiales.</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Lead text:</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Gestiona tus trámites aduaneros, consulta requisitos y haz seguimiento a tus operaciones según tu rol en la cadena logística.</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Base jurídica:</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>Código Tributario (Dto. 6-91), CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA (Resolución 224-2008 COMIECO).</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CONTRIBUYENTES  (413 Trámites — 55.9% del Portal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Qué es:</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Son las personas individuales, jurídicas, patrimonios o entes afectos al cumplimiento de obligaciones tributarias internas en el territorio guatemalteco. Abarca a ciudadanos sin actividad económica activa, asalariados en relación de dependencia, pequeños contribuyentes, contribuyentes del régimen general del IVA e ISR, propietarios de vehículos y grandes/medianos contribuyentes especiales calificados.</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Lead text:</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Cumple con tus obligaciones tributarias, emite tus facturas, actualiza tu RTU y gestiona tus trámites de vehículos e impuestos internos de forma ágil y 100% digital.</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Base jurídica:</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>Constitución Política (Art. 135d), Código Tributario (Dto. 6-91), Ley del IVA (Dto. 27-92), Ley de Actualización Tributaria (Dto. 10-2012), Ley del ISCV (Dto. 70-94) y Ley de Simplificación Tributaria (Dto. 7-2019 / Dto. 31-2024).</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PROFESIONALES  (45 Trámites — 6.1% del Portal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Qué es:</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Son las personas individuales colegiadas activas o técnicos acreditados ante la SAT que ejercen liberalmente su profesión o actúan como auxiliares técnicos en materia tributaria, mercantil y notarial. Comprende a abogados y notarios (traspasos vehiculares electrónicos y fe pública), peritos contadores, contadores públicos y auditores (CPA) y gestores tributarios acreditados.</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Lead text:</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Accede a herramientas especializadas de fe pública, autorización de libros contables, presentación de dictámenes fiscales y gestión de trámites profesionales.</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Base jurídica:</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>Código de Notariado (Dto. 314), Ley de Colegiación Profesional Obligatoria (Dto. 72-2001), Decreto 2450 (Normas de la Profesión Contable), Ley de Timbres Fiscales (Dto. 37-92) y Código Tributario (Art. 57 "A" y 112).</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENTES EXENTOS  (79 Trámites — 10.7% del Portal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Qué es:</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Son las personas jurídicas, entidades del sector público, organismos diplomáticos y organizaciones de la sociedad civil que, por mandato constitucional o ley específica ordinaria, gozan de exención total o parcial de tributos y aranceles en el territorio nacional. Incluye centros educativos, universidades, comunidades religiosas, ONGs, fundaciones sin fines de lucro, municipalidades y ministerios de Estado.</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Lead text:</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Solicita y gestiona tus resoluciones de exención, emite constancias tributarias electrónicas y administra las obligaciones formales de tu entidad.</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Base jurídica:</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Constitución Política (Arts. 37, 73, 88 y 257), Ley de ONGs (Dto. 02-2003), Ley del IVA (Dto. 27-92, Art. 8), Ley de Actualización Tributaria (Dto. 10-2012, Art. 11), Código Municipal (Dto. 12-2002) y Ley Orgánica del Presupuesto (Dto. 101-97).</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="B2:H3"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="F6:G7"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="B11:G11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -583,1084 +1005,1084 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Nivel 1: Segmento Oficial</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>Nivel 2: Categoría / Área</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Nivel 3: Grupo / Actor Específico</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>Nivel 4: Tema / Especialidad</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="18" t="inlineStr">
         <is>
           <t>Trámites Contenidos</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>Ruta de Navegación de Entrada (Miga de Pan)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>NIT sin Obligaciones</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>Personas Individuales</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>RTU Digital y Solicitud de NIT</t>
         </is>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; NIT sin Obligaciones &gt; RTU Digital y Solicitud de NIT</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="25" t="inlineStr">
         <is>
           <t>Pequeño Contribuyente General</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="25" t="inlineStr">
         <is>
           <t>Régimen de 5% y Facturación FEL</t>
         </is>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="26" t="n">
         <v>22</v>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="25" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Régimen de 5% y Facturación FEL</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>Sector Primario y Agropecuario</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>Regímenes Especiales Decreto 31-2024 / 7-2019</t>
         </is>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Regímenes Especiales Decreto 31-2024 / 7-2019</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="25" t="inlineStr">
         <is>
           <t>Personas y Empresas en Régimen General</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="25" t="inlineStr">
         <is>
           <t>IVA General e Impuesto Sobre la Renta (ISR)</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="25" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; IVA General e Impuesto Sobre la Renta (ISR)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Asalariados</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>Trabajadores en Relación de Dependencia</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>Retenciones de ISR y Planilla del IVA</t>
         </is>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Asalariados &gt; Retenciones de ISR y Planilla del IVA</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="25" t="inlineStr">
         <is>
           <t>Propietarios y Compradores de Vehículos</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr">
+      <c r="F12" s="25" t="inlineStr">
         <is>
           <t>Registro Fiscal de Vehículos (RFV)</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="26" t="n">
         <v>72</v>
       </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="H12" s="25" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Vehículos &gt; Registro Fiscal de Vehículos (RFV)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes Especiales</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>Grandes y Medianos Contribuyentes</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="21" t="inlineStr">
         <is>
           <t>Gerencias Especializadas de Fiscalización</t>
         </is>
       </c>
-      <c r="G13" s="7" t="n">
+      <c r="G13" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyentes Especiales &gt; Gerencias Especializadas de Fiscalización</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr">
         <is>
           <t>Facturación Electrónica</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="25" t="inlineStr">
         <is>
           <t>Emisores de DTE</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F14" s="25" t="inlineStr">
         <is>
           <t>Sistema FEL y Agencia Virtual</t>
         </is>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H14" s="25" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Facturación Electrónica &gt; Sistema FEL y Agencia Virtual</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>Servicios al Contribuyente</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>Ciudadanía y Usuarios de Agencia Virtual</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="21" t="inlineStr">
         <is>
           <t>Plataforma Digital, Citas y Solvencias</t>
         </is>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G15" s="22" t="n">
         <v>67</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Servicios al Contribuyente &gt; Plataforma Digital, Citas y Solvencias</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="24" t="inlineStr">
         <is>
           <t>Importadores y Exportadores (Compartido)</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="25" t="inlineStr">
         <is>
           <t>Operadores Comerciales Generales</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F16" s="25" t="inlineStr">
         <is>
           <t>Gestiones Aduaneras Comunes y Arancel</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="H16" s="25" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Importadores y Exportadores (Compartido) &gt; Gestiones Aduaneras Comunes y Arancel</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>Importadores</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>Importadores Registrados</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="21" t="inlineStr">
         <is>
           <t>Padrón de Importadores y DUCA-D</t>
         </is>
       </c>
-      <c r="G17" s="7" t="n">
+      <c r="G17" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Importadores &gt; Padrón de Importadores y DUCA-D</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>Exportadores</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>Exportadores Habituales y Ocasionales</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F18" s="25" t="inlineStr">
         <is>
           <t>Padrón de Exportadores y Devolución IVA</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
+      <c r="G18" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H18" s="25" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Exportadores &gt; Padrón de Exportadores y Devolución IVA</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="20" t="inlineStr">
         <is>
           <t>Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>Operadores Certificados en Seguridad</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>Cadena Logística Segura y Carril Exprés</t>
         </is>
       </c>
-      <c r="G19" s="7" t="n">
+      <c r="G19" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Operador Económico Autorizado (OEA) &gt; Cadena Logística Segura y Carril Exprés</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="24" t="inlineStr">
         <is>
           <t>Agentes Aduaneros</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="25" t="inlineStr">
         <is>
           <t>Auxiliares de la Función Pública Aduanera</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F20" s="25" t="inlineStr">
         <is>
           <t>Despacho Aduanero Oficial y Representación</t>
         </is>
       </c>
-      <c r="G20" s="11" t="n">
+      <c r="G20" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="H20" s="25" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Agentes Aduaneros &gt; Despacho Aduanero Oficial y Representación</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="20" t="inlineStr">
         <is>
           <t>Apoderados Especiales Aduaneros</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>Representantes Legales Exclusivos</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="21" t="inlineStr">
         <is>
           <t>Despacho Aduanero por Cuenta Propia</t>
         </is>
       </c>
-      <c r="G21" s="7" t="n">
+      <c r="G21" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="21" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Apoderados Especiales Aduaneros &gt; Despacho Aduanero por Cuenta Propia</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="8" t="n">
+      <c r="B22" s="23" t="n">
         <v>16</v>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="24" t="inlineStr">
         <is>
           <t>Empresas de Entrega Rápida o Courier</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E22" s="25" t="inlineStr">
         <is>
           <t>Mensajería y Envíos Expresos</t>
         </is>
       </c>
-      <c r="F22" s="10" t="inlineStr">
+      <c r="F22" s="25" t="inlineStr">
         <is>
           <t>Paquetería Internacional y Franquicias</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
+      <c r="G22" s="26" t="n">
         <v>13</v>
       </c>
-      <c r="H22" s="10" t="inlineStr">
+      <c r="H22" s="25" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Empresas de Entrega Rápida o Courier &gt; Paquetería Internacional y Franquicias</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="20" t="inlineStr">
         <is>
           <t>Consolidadores y Desconsolidadores de Carga</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>Operadores Logísticos y de Carga</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="21" t="inlineStr">
         <is>
           <t>Manifiestos CUSCAR y Guías Hijas</t>
         </is>
       </c>
-      <c r="G23" s="7" t="n">
+      <c r="G23" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="21" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Consolidadores y Desconsolidadores de Carga &gt; Manifiestos CUSCAR y Guías Hijas</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="8" t="n">
+      <c r="B24" s="23" t="n">
         <v>18</v>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" s="24" t="inlineStr">
         <is>
           <t>Transportistas Aduaneros</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E24" s="25" t="inlineStr">
         <is>
           <t>Transporte Internacional Terrestre y Carga</t>
         </is>
       </c>
-      <c r="F24" s="10" t="inlineStr">
+      <c r="F24" s="25" t="inlineStr">
         <is>
           <t>Tránsito Aduanero Internacional y Marchamo</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
+      <c r="G24" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="H24" s="10" t="inlineStr">
+      <c r="H24" s="25" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Transportistas Aduaneros &gt; Tránsito Aduanero Internacional y Marchamo</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="4" t="n">
+      <c r="B25" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="20" t="inlineStr">
         <is>
           <t>Depósitos Aduaneros</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>Almacenes Fiscales, AGD y DAT</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="21" t="inlineStr">
         <is>
           <t>Custodia de Mercancías y Títulos de Crédito</t>
         </is>
       </c>
-      <c r="G25" s="7" t="n">
+      <c r="G25" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Depósitos Aduaneros &gt; Custodia de Mercancías y Títulos de Crédito</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="8" t="n">
+      <c r="B26" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C26" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" s="24" t="inlineStr">
         <is>
           <t>ZDEEP - Entidades Administradoras</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E26" s="25" t="inlineStr">
         <is>
           <t>Polígonos ZDEEP</t>
         </is>
       </c>
-      <c r="F26" s="10" t="inlineStr">
+      <c r="F26" s="25" t="inlineStr">
         <is>
           <t>Administración de Zonas Especiales Públicas</t>
         </is>
       </c>
-      <c r="G26" s="11" t="n">
+      <c r="G26" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="H26" s="25" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; ZDEEP - Entidades Administradoras &gt; Administración de Zonas Especiales Públicas</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="4" t="n">
+      <c r="B27" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>ZDEEP - Empresas Usuarias</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="21" t="inlineStr">
         <is>
           <t>Empresas Instaladas en ZDEEP</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="21" t="inlineStr">
         <is>
           <t>Transformación, Servicios y Exenciones</t>
         </is>
       </c>
-      <c r="G27" s="7" t="n">
+      <c r="G27" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; ZDEEP - Empresas Usuarias &gt; Transformación, Servicios y Exenciones</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="8" t="n">
+      <c r="B28" s="23" t="n">
         <v>22</v>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C28" s="24" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D28" s="24" t="inlineStr">
         <is>
           <t>Abogados y Notarios</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="E28" s="25" t="inlineStr">
         <is>
           <t>Notarios en Ejercicio</t>
         </is>
       </c>
-      <c r="F28" s="10" t="inlineStr">
+      <c r="F28" s="25" t="inlineStr">
         <is>
           <t>Papel Sellado de Protocolo y Avisos</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
+      <c r="G28" s="26" t="n">
         <v>17</v>
       </c>
-      <c r="H28" s="10" t="inlineStr">
+      <c r="H28" s="25" t="inlineStr">
         <is>
           <t>Profesionales &gt; Abogados y Notarios &gt; Papel Sellado de Protocolo y Avisos</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>Peritos Contadores</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="21" t="inlineStr">
         <is>
           <t>Contadores Registrados</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="F29" s="21" t="inlineStr">
         <is>
           <t>Libros Contables y Declaraciones</t>
         </is>
       </c>
-      <c r="G29" s="7" t="n">
+      <c r="G29" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>Profesionales &gt; Peritos Contadores &gt; Libros Contables y Declaraciones</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="23" t="n">
         <v>24</v>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C30" s="24" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D30" s="24" t="inlineStr">
         <is>
           <t>Auditores</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E30" s="25" t="inlineStr">
         <is>
           <t>Contadores Públicos y Auditores (CPA)</t>
         </is>
       </c>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="F30" s="25" t="inlineStr">
         <is>
           <t>Dictámenes Tributarios y Devolución IVA</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
+      <c r="G30" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="H30" s="10" t="inlineStr">
+      <c r="H30" s="25" t="inlineStr">
         <is>
           <t>Profesionales &gt; Auditores &gt; Dictámenes Tributarios y Devolución IVA</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="4" t="n">
+      <c r="B31" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>Gestores Tributarios</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="21" t="inlineStr">
         <is>
           <t>Gestores Acreditados SAT</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" s="21" t="inlineStr">
         <is>
           <t>Gafetes y Trámites Presenciales</t>
         </is>
       </c>
-      <c r="G31" s="7" t="n">
+      <c r="G31" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="H31" s="21" t="inlineStr">
         <is>
           <t>Profesionales &gt; Gestores Tributarios &gt; Gafetes y Trámites Presenciales</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="8" t="n">
+      <c r="B32" s="23" t="n">
         <v>26</v>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D32" s="24" t="inlineStr">
         <is>
           <t>Servicios Profesionales</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E32" s="25" t="inlineStr">
         <is>
           <t>Profesionales Liberales Independientes</t>
         </is>
       </c>
-      <c r="F32" s="10" t="inlineStr">
+      <c r="F32" s="25" t="inlineStr">
         <is>
           <t>Facturación por Honorarios y Retenciones</t>
         </is>
       </c>
-      <c r="G32" s="11" t="n">
+      <c r="G32" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="H32" s="10" t="inlineStr">
+      <c r="H32" s="25" t="inlineStr">
         <is>
           <t>Profesionales &gt; Servicios Profesionales &gt; Facturación por Honorarios y Retenciones</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="4" t="n">
+      <c r="B33" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="20" t="inlineStr">
         <is>
           <t>Constitucionales</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E33" s="21" t="inlineStr">
         <is>
           <t>Universidades, Colegios e Iglesias</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="F33" s="21" t="inlineStr">
         <is>
           <t>Exenciones Tributarias de Rango Constitucional</t>
         </is>
       </c>
-      <c r="G33" s="7" t="n">
+      <c r="G33" s="22" t="n">
         <v>18</v>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="H33" s="21" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Constitucionales &gt; Exenciones Tributarias de Rango Constitucional</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="8" t="n">
+      <c r="B34" s="23" t="n">
         <v>28</v>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="24" t="inlineStr">
         <is>
           <t>No Lucrativos</t>
         </is>
       </c>
-      <c r="E34" s="10" t="inlineStr">
+      <c r="E34" s="25" t="inlineStr">
         <is>
           <t>ONGs, Fundaciones y Cooperativas</t>
         </is>
       </c>
-      <c r="F34" s="10" t="inlineStr">
+      <c r="F34" s="25" t="inlineStr">
         <is>
           <t>Reconocimiento de Exención de ISR e IVA</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
+      <c r="G34" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="H34" s="10" t="inlineStr">
+      <c r="H34" s="25" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; No Lucrativos &gt; Reconocimiento de Exención de ISR e IVA</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="4" t="n">
+      <c r="B35" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="20" t="inlineStr">
         <is>
           <t>Municipalidades</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>Gobiernos Locales y Empresas Municipales</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F35" s="21" t="inlineStr">
         <is>
           <t>Autonomía Municipal y Régimen Exento</t>
         </is>
       </c>
-      <c r="G35" s="7" t="n">
+      <c r="G35" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="H35" s="21" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Municipalidades &gt; Autonomía Municipal y Régimen Exento</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="8" t="n">
+      <c r="B36" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="24" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D36" s="24" t="inlineStr">
         <is>
           <t>Entidades del Estado</t>
         </is>
       </c>
-      <c r="E36" s="10" t="inlineStr">
+      <c r="E36" s="25" t="inlineStr">
         <is>
           <t>Ministerios, Secretarías y Organismos del Estado</t>
         </is>
       </c>
-      <c r="F36" s="10" t="inlineStr">
+      <c r="F36" s="25" t="inlineStr">
         <is>
           <t>Compras Públicas y Agentes de Retención</t>
         </is>
       </c>
-      <c r="G36" s="11" t="n">
+      <c r="G36" s="26" t="n">
         <v>26</v>
       </c>
-      <c r="H36" s="10" t="inlineStr">
+      <c r="H36" s="25" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Entidades del Estado &gt; Compras Públicas y Agentes de Retención</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="4" t="n">
+      <c r="B37" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="20" t="inlineStr">
         <is>
           <t>Decreto</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>Entidades con Incentivos Especiales</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F37" s="21" t="inlineStr">
         <is>
           <t>Exenciones y Fomento por Decreto Legislativo</t>
         </is>
       </c>
-      <c r="G37" s="7" t="n">
+      <c r="G37" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="H37" s="21" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Decreto &gt; Exenciones y Fomento por Decreto Legislativo</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="12" t="inlineStr"/>
-      <c r="C38" s="13" t="inlineStr">
+      <c r="B38" s="27" t="inlineStr"/>
+      <c r="C38" s="28" t="inlineStr">
         <is>
           <t>TOTAL DEL PORTAL</t>
         </is>
       </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="D38" s="29" t="inlineStr">
         <is>
           <t>4 Segmentos y 31 Categorías Principales</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr"/>
-      <c r="F38" s="12" t="inlineStr"/>
-      <c r="G38" s="15">
+      <c r="E38" s="27" t="inlineStr"/>
+      <c r="F38" s="27" t="inlineStr"/>
+      <c r="G38" s="30">
         <f>SUM(G7:G37)</f>
         <v/>
       </c>
-      <c r="H38" s="13" t="inlineStr">
+      <c r="H38" s="28" t="inlineStr">
         <is>
           <t>739 Trámites Oficiales Integrados</t>
         </is>
@@ -1675,7 +2097,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1686,18 +2108,18 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>MATRIZ DE DESCRIPCIONES FUNCIONALES Y FUNDAMENTO JURÍDICO — PORTAL SAT</t>
+          <t>FICHAS TÉCNICAS DE ARQUITECTURA: DEFINICIÓN, LEAD TEXT Y BASE JURÍDICA POR ROL</t>
         </is>
       </c>
     </row>
@@ -1705,1227 +2127,1227 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DEFINICIÓN OPERATIVA: PARA QUIÉN ES, ALCANCE FUNCIONAL Y EN BASE A QUÉ NORMATIVA OPERA CADA CATEGORÍA</t>
+          <t>MATRIZ COMPLETA DE LAS 31 CATEGORÍAS DEL PORTAL CON SUS TEXTOS ORIENTADORES Y MARCO NORMATIVO OFICIAL</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Segmento (L1)</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Categoría / Actor (L2/L3)</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Especialidad / Tema (L4)</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>¿Para quién es? (Audiencia Destinataria en Lenguaje Ciudadano)</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>¿Qué se puede hacer aquí? (Alcance y Gestiones Clave)</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Base Legal de Referencia (En base a qué: CAUCA, RECAUCA, Leyes, Decretos)</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Total Fichas</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Segmento (Nivel 1)</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Categoría / Rol (Nivel 2/3)</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Tema / Especialidad (Nivel 4)</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Qué es: (Definición Operativa de la Figura)</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Lead text: (Texto Orientador de Interfaz)</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Base jurídica: (Fundamento Legal Oficial: CAUCA, RECAUCA, Leyes)</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Trámites</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>NIT sin Obligaciones</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>RTU Digital y Solicitud de NIT</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>Personas individuales, estudiantes, asalariados y personas en el extranjero que no realizan actividad económica pero requieren NIT para trámites civiles, herencias, cuentas bancarias o compra de bienes.</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>Inscripción de primer NIT en línea, actualización de datos de residencia, solicitud de solvencia fiscal y consultas ciudadanas.</t>
-        </is>
-      </c>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="E7" s="31" t="inlineStr">
+        <is>
+          <t>Categoría destinada a personas individuales (estudiantes, personas en relación de dependencia sin renta afecta o ciudadanos en el extranjero) que requieren un Número de Identificación Tributaria únicamente para actos civiles, contractuales, bancarios o de registro público, sin realizar actividades mercantiles ni prestación de servicios técnicos afectos.</t>
+        </is>
+      </c>
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>Inscribe tu primer NIT en línea, actualiza tus datos de residencia y obtén tu constancia de solvencia fiscal sin necesidad de acudir a una agencia.</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
         <is>
           <t>Código Tributario (Decreto 6-91, Arts. 112 y 120), Ley de Actualización Tributaria (Decreto 10-2012) y Acuerdo de Directorio SAT 08-2020.</t>
         </is>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="22" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="8" t="n">
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="25" t="inlineStr">
         <is>
           <t>Régimen de 5% y Facturación FEL</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>Personas individuales o jurídicas con ventas o servicios de hasta Q150,000 en el año calendario que tributan con una tarifa definitiva del 5% sin derecho a crédito fiscal.</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>Inscripción y cambio de régimen, habilitación de factura electrónica FEL, declaración mensual en Declaraguate (SAT-2046) y cierre o suspensión de actividades.</t>
-        </is>
-      </c>
-      <c r="G8" s="19" t="inlineStr">
+      <c r="E8" s="34" t="inlineStr">
+        <is>
+          <t>Régimen simplificado para personas individuales o jurídicas cuyas ventas de bienes o prestación de servicios no superan el monto de Q150,000 en el año calendario, tributando bajo una tarifa definitiva del 5% sobre ingresos brutos mensuales sin derecho a crédito fiscal.</t>
+        </is>
+      </c>
+      <c r="F8" s="35" t="inlineStr">
+        <is>
+          <t>Emite tus facturas electrónicas FEL de pequeño contribuyente, declara mensualmente el 5% en Declaraguate y mantén tus libros al día.</t>
+        </is>
+      </c>
+      <c r="G8" s="36" t="inlineStr">
         <is>
           <t>Ley del IVA (Decreto 27-92, Arts. 45 al 50) y Ley de Simplificación Tributaria (Decreto 7-2019, Régimen Electrónico de Pequeño Contribuyente).</t>
         </is>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="H8" s="26" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="4" t="n">
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Regímenes Especiales Decreto 31-2024 / 7-2019</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
-        <is>
-          <t>Productores y comercializadores artesanales, agrícolas y ganaderos que operan en los regímenes simplificados del sector primario y pecuario.</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>Inscripción en padrón agropecuario, liquidación y pago del Impuesto a la Confianza Tributaria (ICT) y emisión de documentos tributarios autorizados.</t>
-        </is>
-      </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>Decreto 7-2019 y Decreto 31-2024 (Ley para la Integración del Sector Productivo Primario y Agropecuario).</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="n">
+      <c r="E9" s="31" t="inlineStr">
+        <is>
+          <t>Regímenes tributarios especiales creados para productores, ganaderos y comercializadores del sector agropecuario, artesanal y primario que comercializan productos no transformados.</t>
+        </is>
+      </c>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>Inscríbete en el régimen especial agropecuario, liquida tu Impuesto a la Confianza Tributaria y emite comprobantes oficiales simplificados.</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>Ley de Simplificación Tributaria (Decreto 7-2019) y Ley para la Integración del Sector Productivo Primario y Agropecuario (Decreto 31-2024).</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="8" t="n">
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="25" t="inlineStr">
         <is>
           <t>IVA General e Impuesto Sobre la Renta (ISR)</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>Empresas individuales, sociedades mercantiles y profesionales con ingresos mayores a Q150,000 o afiliados al Régimen General del IVA y del ISR (Opcional Simplificado o Sobre Utilidades).</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>Declaración y pago mensual de IVA (SAT-2237), pagos trimestrales o mensuales de ISR (SAT-1311/SAT-1411), liquidación de ISO y emisión obligatoria de FEL.</t>
-        </is>
-      </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="E10" s="34" t="inlineStr">
+        <is>
+          <t>Régimen aplicable a personas individuales y sociedades mercantiles con ingresos superiores a Q150,000 o afiliados voluntariamente al Régimen General del IVA (12%) y regímenes del ISR (Opcional Simplificado 5%/7% o Sobre Utilidades de Actividades Lucrativas 25%).</t>
+        </is>
+      </c>
+      <c r="F10" s="35" t="inlineStr">
+        <is>
+          <t>Declara y paga tu IVA mensual, liquida tus pagos trimestrales o retenciones de ISR, gestiona tu crédito fiscal y factura mediante FEL.</t>
+        </is>
+      </c>
+      <c r="G10" s="36" t="inlineStr">
         <is>
           <t>Ley del IVA (Decreto 27-92), Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del Impuesto de Solidaridad (Decreto 73-2008).</t>
         </is>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="26" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="4" t="n">
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Asalariados</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>Retenciones de ISR y Planilla del IVA</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>Trabajadores contratados por patronos públicos o privados que perciben sueldos, salarios o bonificaciones sujetos a retención del Impuesto Sobre la Renta.</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>Proyección anual de ISR, presentación de la planilla electrónica del IVA con comprobantes FEL y solicitud de devolución de retenciones practicadas en exceso.</t>
-        </is>
-      </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="E11" s="31" t="inlineStr">
+        <is>
+          <t>Régimen tributario de rentas del trabajo en relación de dependencia aplicable a trabajadores contratados por patronos públicos o privados que perciben ingresos salariales sujetos a retención del ISR.</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>Consulta tus retenciones de ISR practicadas por tu patrono, ingresa tu planilla del IVA con facturas FEL y solicita devolución de retenciones en exceso.</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
         <is>
           <t>Ley de Actualización Tributaria (Decreto 10-2012, Arts. 68 al 82 - Rentas del Trabajo en Relación de Dependencia).</t>
         </is>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="22" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="8" t="n">
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="25" t="inlineStr">
         <is>
           <t>Registro Fiscal de Vehículos (RFV)</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
-        <is>
-          <t>Personas y empresas propietarias de automotores, importadores de vehículos y ciudadanos que compran o venden automóviles terrestres, motos o unidades marítimas.</t>
-        </is>
-      </c>
-      <c r="F12" s="18" t="inlineStr">
-        <is>
-          <t>Pago del Impuesto sobre Circulación (ISCV - Calcomanía), primeras placas, traspaso electrónico con notario, reposición de tarjeta y distintivos, y baja o inactivación.</t>
-        </is>
-      </c>
-      <c r="G12" s="19" t="inlineStr">
+      <c r="E12" s="34" t="inlineStr">
+        <is>
+          <t>Registro Fiscal de Vehículos (RFV) que administra el parque vehicular nacional, altas, bajas, modificaciones y el impuesto anual de circulación para propietarios y compradores de automotores terrestres, marítimos y aéreos.</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>Paga tu calcomanía anual de circulación (ISCV), tramita primeras placas, realiza traspasos vehiculares y repón distintivos extraviados.</t>
+        </is>
+      </c>
+      <c r="G12" s="36" t="inlineStr">
         <is>
           <t>Ley del Impuesto sobre Circulación de Vehículos Terrestres, Marítimos y Aéreos (Decreto 70-94) y Código Tributario (Decreto 6-91).</t>
         </is>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="26" t="n">
         <v>72</v>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="4" t="n">
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes Especiales</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>Gerencias Especializadas de Fiscalización</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>Contribuyentes calificados por resolución de la SAT en función de su representatividad fiscal, nivel de facturación y sector económico.</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>Atención en gerencias diferenciadas, presentación de estados financieros auditados, precios de transferencia y control intensivo de solvencia.</t>
-        </is>
-      </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Segmento de control fiscal diferenciado conformado por grandes y medianos contribuyentes calificados por resolución de la SAT en función de su representatividad en la recaudación, facturación y relevancia sectorial.</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>Gestiona tus obligaciones en agencias especializadas, presenta estados financieros auditados y cumple con estudios de precios de transferencia.</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
         <is>
           <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3) y Resoluciones de Directorio de Calificación de Contribuyentes Especiales.</t>
         </is>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="22" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="8" t="n">
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>Facturación Electrónica</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="25" t="inlineStr">
         <is>
           <t>Sistema FEL y Agencia Virtual</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
-        <is>
-          <t>Todos los contribuyentes afiliados al régimen tributario nacional obligados a emitir facturas, notas de crédito, notas de débito y recibos digitales.</t>
-        </is>
-      </c>
-      <c r="F14" s="18" t="inlineStr">
-        <is>
-          <t>Habilitación como emisor FEL, emisión gratuita desde la Agencia Virtual, anulación de DTE, consulta de facturas recibidas y acreditación de certificadores.</t>
-        </is>
-      </c>
-      <c r="G14" s="19" t="inlineStr">
+      <c r="E14" s="34" t="inlineStr">
+        <is>
+          <t>Régimen obligatorio de emisión, transmisión y certificación de Documentos Tributarios Electrónicos (DTE) a través del sistema FEL y certificadores autorizados para todos los contribuyentes afiliados al régimen tributario nacional.</t>
+        </is>
+      </c>
+      <c r="F14" s="35" t="inlineStr">
+        <is>
+          <t>Habilítate como emisor de factura electrónica FEL, emite facturas gratuitas desde la Agencia Virtual y administra tus documentos emitidos y recibidos.</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
         <is>
           <t>Ley del IVA (Decreto 27-92, Arts. 29 y 29 "A") y Acuerdo de Directorio SAT 13-2018 (Régimen FEL).</t>
         </is>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="26" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="4" t="n">
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>Servicios al Contribuyente</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>Plataforma Digital, Citas y Solvencias</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>Cualquier persona individual o jurídica que necesita gestionar claves de acceso, citas presenciales, solvencias fiscales o presentar consultas.</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>Creación y reseteo de usuario en Agencia Virtual, emisión de solvencia fiscal inmediata, programación de citas presenciales y consulta de NIT.</t>
-        </is>
-      </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
+        <is>
+          <t>Plataforma de servicios transversales de atención ciudadana, autenticación digital, expedición de solvencias fiscales, agendamiento de citas presenciales y consultas públicas en bases de datos de la SAT.</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>Crea o desbloquea tu Agencia Virtual, genera tu solvencia fiscal con código QR, agenda citas presenciales y consulta el estado de tus gestiones.</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
         <is>
           <t>Código Tributario (Decreto 6-91, Art. 57 "A" y Art. 120) y Acuerdos de Directorio de Servicios Electrónicos.</t>
         </is>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="22" t="n">
         <v>67</v>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="8" t="n">
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>Importadores y Exportadores (Compartido)</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="25" t="inlineStr">
         <is>
           <t>Gestiones Aduaneras Comunes y Arancel</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
-        <is>
-          <t>Empresas y personas que realizan operaciones transfronterizas de entrada y salida de mercancías.</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>Consulta del Arancel Integrado Centroamericano (SAC), pago electrónico por BancaSAT, DUCA general, solvencia aduanera y permisos no arancelarios.</t>
-        </is>
-      </c>
-      <c r="G16" s="19" t="inlineStr">
-        <is>
-          <t>Código Aduanero Uniforme Centroamericano (CAUCA IV), Reglamento (RECAUCA IV) y Convenio Arancelario Centroamericano.</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="n">
+      <c r="E16" s="34" t="inlineStr">
+        <is>
+          <t>Operadores comerciales que realizan indistintamente gestiones transversales de entrada y salida de mercancías, consultas arancelarias y pagos tributarios aduaneros en las aduanas de la República.</t>
+        </is>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>Consulta el Arancel Integrado Centroamericano (SAC), realiza pagos por BancaSAT y tramita solvencias aduaneras unificadas.</t>
+        </is>
+      </c>
+      <c r="G16" s="36" t="inlineStr">
+        <is>
+          <t>Convenio sobre el Régimen Arancelario y Aduanero Centroamericano, CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA IV (Resolución 224-2008 COMIECO).</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1">
-      <c r="A17" s="4" t="n">
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>Importadores</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>Padrón de Importadores y DUCA-D</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
-        <is>
-          <t>Empresas y personas individuales autorizadas en el padrón aduanero de la SAT para introducir mercancías al territorio nacional.</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>Inscripción en el padrón de importadores, liquidación de DUCA-D de importación, declaración del valor aduanero, rescate de mercancías en abandono e IPRIMA.</t>
-        </is>
-      </c>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>CAUCA IV, RECAUCA IV (Despacho Aduanero de Importación) y Acuerdo Relativo a la Aplicación del Artículo VII del GATT (Valoración OMC).</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="n">
+      <c r="E17" s="31" t="inlineStr">
+        <is>
+          <t>Personas individuales o jurídicas autorizadas en el padrón aduanero de la SAT para introducir legalmente mercancías extranjeras al territorio aduanero nacional para su consumo, uso o transformación.</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>Inscríbete en el padrón de importadores, liquida tus declaraciones aduaneras DUCA-D, consulta aranceles y rescata mercancías en aduana.</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Acuerdo Relativo a la Aplicación del Artículo VII del GATT (Valoración OMC).</t>
+        </is>
+      </c>
+      <c r="H17" s="22" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="8" t="n">
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>Exportadores</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="25" t="inlineStr">
         <is>
           <t>Padrón de Exportadores y Devolución IVA</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
-        <is>
-          <t>Personas y empresas inscritas en el Registro de Exportadores de la SAT que despachan productos nacionales hacia mercados internacionales.</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Inscripción en Agencia Virtual con código VUPE, autorización de listas de embarque, declaraciones simplificadas y solicitud de devolución de crédito fiscal del IVA.</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>Ley de Fomento y Maquila (Decreto 29-89), Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis) y CAUCA/RECAUCA.</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="n">
+      <c r="E18" s="34" t="inlineStr">
+        <is>
+          <t>Personas individuales o jurídicas inscritas en el Registro de Exportadores de la SAT que despachan mercancías de origen nacional o nacionalizadas hacia mercados del exterior.</t>
+        </is>
+      </c>
+      <c r="F18" s="35" t="inlineStr">
+        <is>
+          <t>Registra tus exportaciones con código VUPE, emite facturas con régimen especial y gestiona la devolución de crédito fiscal del IVA.</t>
+        </is>
+      </c>
+      <c r="G18" s="36" t="inlineStr">
+        <is>
+          <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Ley de Fomento y Maquila (Decreto 29-89) y CAUCA/RECAUCA IV.</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="4" t="n">
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>Cadena Logística Segura y Carril Exprés</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>Empresas calificadas por la Intendencia de Aduanas que garantizan altos estándares de seguridad en la cadena logística internacional.</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>Acceso a carriles preferenciales en puestos fronterizos y puertos, atención prioritaria en contingencias, reducción de selectivo rojo y despacho ágil.</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>Marco Normativo SAFE de la Organización Mundial de Aduanas (OMA), CAUCA IV y Acuerdos de Directorio SAT.</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="n">
+      <c r="E19" s="31" t="inlineStr">
+        <is>
+          <t>Operadores de la cadena logística internacional certificados por la Intendencia de Aduanas por mantener rigurosos estándares de seguridad y confiabilidad en sus operaciones transfronterizas.</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>Accede a carriles exprés preferenciales, prioridad en contingencias y despacho ágil con selectivo rojo reducido.</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio de la SAT sobre el Programa OEA-Guatemala.</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="8" t="n">
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>Agentes Aduaneros</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="25" t="inlineStr">
         <is>
           <t>Despacho Aduanero Oficial y Representación</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>Profesionales autorizados por el Directorio de la SAT para prestar servicios a terceros en el despacho de mercancías ante la aduana.</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>Habilitación de carné oficial, constitución de seguro de caución, transmisión de DUCAs con firma electrónica, acreditación de asistentes y recursos legales.</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="inlineStr">
+      <c r="E20" s="34" t="inlineStr">
+        <is>
+          <t>Profesionales auxiliares de la función pública aduanera autorizados para actuar por cuenta de terceros en los trámites y operaciones de desaduanamiento ante la SAT.</t>
+        </is>
+      </c>
+      <c r="F20" s="35" t="inlineStr">
+        <is>
+          <t>Gestiona tu carné y habilitación oficial, presenta pólizas de seguro de caución y transmite declaraciones con firma electrónica.</t>
+        </is>
+      </c>
+      <c r="G20" s="36" t="inlineStr">
         <is>
           <t>CAUCA IV (Arts. 22 al 28), RECAUCA IV (Arts. 74 al 85) y Ley Nacional de Aduanas.</t>
         </is>
       </c>
-      <c r="H20" s="11" t="n">
+      <c r="H20" s="26" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1">
-      <c r="A21" s="4" t="n">
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>Apoderados Especiales Aduaneros</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="21" t="inlineStr">
         <is>
           <t>Despacho Aduanero por Cuenta Propia</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
-        <is>
-          <t>Personas individuales designadas mediante mandato por una persona jurídica para representarla exclusivamente en sus despachos aduaneros.</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>Registro de mandato legal, renovación anual de autorización, carné de apoderado, presentación de fianzas operativas y gestión de DUCAs corporativas.</t>
-        </is>
-      </c>
-      <c r="G21" s="17" t="inlineStr">
-        <is>
-          <t>CAUCA IV (Art. 21), RECAUCA IV (Arts. 86 al 90) y Ley Nacional de Aduanas.</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="n">
+      <c r="E21" s="31" t="inlineStr">
+        <is>
+          <t>Personas individuales mandatarias designadas exclusivamente por una persona jurídica para representarla formalmente en sus despachos aduaneros propios.</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>Registra tu mandato legal, actualiza tu carné de apoderado y tramita declaraciones DUCA corporativas.</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Art. 21), RECAUCA IV (Arts. 86 al 90) y Código de Notariado.</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="22" ht="42" customHeight="1">
-      <c r="A22" s="8" t="n">
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="23" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>Empresas de Entrega Rápida o Courier</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="25" t="inlineStr">
         <is>
           <t>Paquetería Internacional y Franquicias</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Empresas de paquetería urgente que transportan y desaduanan envíos postales no comerciales y encomiendas internacionales.</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="inlineStr">
-        <is>
-          <t>Transmisión de manifiestos courier, despacho simplificado oficioso (Categorías A, B y C), habilitación de recintos desconsolidadores y franquicias.</t>
-        </is>
-      </c>
-      <c r="G22" s="19" t="inlineStr">
+      <c r="E22" s="34" t="inlineStr">
+        <is>
+          <t>Empresas de mensajería y paquetería urgente autorizadas para transportar y desaduanar envíos postales exprés y encomiendas internacionales no comerciales.</t>
+        </is>
+      </c>
+      <c r="F22" s="35" t="inlineStr">
+        <is>
+          <t>Transmite manifiestos courier, aplica franquicias simplificadas y habilita recintos desconsolidadores de paquetería.</t>
+        </is>
+      </c>
+      <c r="G22" s="36" t="inlineStr">
         <is>
           <t>CAUCA IV y RECAUCA IV (Arts. 574 al 596 - Régimen de Envíos de Entrega Rápida o Courier).</t>
         </is>
       </c>
-      <c r="H22" s="11" t="n">
+      <c r="H22" s="26" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="4" t="n">
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>Consolidadores y Desconsolidadores de Carga</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>Manifiestos CUSCAR y Guías Hijas</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
-        <is>
-          <t>Empresas autorizadas para agrupar o desagrupar mercancías de diferentes consignatarios en una sola unidad de carga.</t>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>Transmisión electrónica del mensaje CUSCAR, desconsolidación de conocimientos de embarque (B/L, AWB) y reporte de faltantes, sobrantes o averías.</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>CAUCA IV y RECAUCA IV (Arts. 102 al 109 - Empresas Consolidadoras y Desconsolidadoras de Carga).</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="n">
+      <c r="E23" s="31" t="inlineStr">
+        <is>
+          <t>Operadores logísticos autorizados para agrupar o separar mercancías pertenecientes a distintos consignatarios bajo un solo documento matriz de transporte.</t>
+        </is>
+      </c>
+      <c r="F23" s="32" t="inlineStr">
+        <is>
+          <t>Transmite manifiestos CUSCAR, emite guías hijas y reporta inconsistencias o averías de carga ante la aduana.</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="inlineStr">
+        <is>
+          <t>CAUCA IV y RECAUCA IV (Arts. 102 al 109 - Auxiliares Consolidador y Desconsolidador de Carga).</t>
+        </is>
+      </c>
+      <c r="H23" s="22" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="8" t="n">
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="23" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>Transportistas Aduaneros</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="25" t="inlineStr">
         <is>
           <t>Tránsito Aduanero Internacional y Marchamo</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Empresas y conductores de transporte internacional de carga terrestre, aéreo y marítimo autorizados ante la SAT.</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>Registro de medios de transporte, admisión temporal de equipo (ATC), colocación de marchamo electrónico RFID, transmisión de DUCA-T y cartas de ingreso.</t>
-        </is>
-      </c>
-      <c r="G24" s="19" t="inlineStr">
-        <is>
-          <t>CAUCA IV (Arts. 18 al 20), RECAUCA IV (Tránsito Aduanero Terrestre) y Reglamentos de Transporte Centroamericano.</t>
-        </is>
-      </c>
-      <c r="H24" s="11" t="n">
+      <c r="E24" s="34" t="inlineStr">
+        <is>
+          <t>Empresas y conductores autorizados para realizar el traslado de mercancías bajo control aduanero dentro del territorio nacional o en tránsito internacional centroamericano.</t>
+        </is>
+      </c>
+      <c r="F24" s="35" t="inlineStr">
+        <is>
+          <t>Registra medios de transporte, activa marchamos electrónicos RFID y transmite declaraciones de tránsito DUCA-T.</t>
+        </is>
+      </c>
+      <c r="G24" s="36" t="inlineStr">
+        <is>
+          <t>CAUCA IV (Arts. 18 al 20), RECAUCA IV (Tránsito Aduanero Internacional Terrestre) y Reglamentos de Transporte Centroamericano.</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="4" t="n">
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>Depósitos Aduaneros</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Custodia de Mercancías y Títulos de Crédito</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
-        <is>
-          <t>Entidades públicas y privadas autorizadas para custodiar mercancías extranjeras bajo control aduanero con suspensión de tributos.</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>Recepción de mercancías, control de permanencia y cobro SCP, emisión de certificados de depósito y bonos de prenda (AGD), actas DAT y reporte de inventarios.</t>
-        </is>
-      </c>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="E25" s="31" t="inlineStr">
+        <is>
+          <t>Recintos públicos o privados (Almacenes Fiscales, Almacenes Generales de Depósito y Depósitos Aduaneros Temporales DAT) autorizados para custodiar mercancías con suspensión de tributos aduaneros.</t>
+        </is>
+      </c>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>Controla inventarios de custodia, gestiona actas de recepción, emite certificados de depósito (AGD) y tramita prórrogas de permanencia.</t>
+        </is>
+      </c>
+      <c r="G25" s="33" t="inlineStr">
         <is>
           <t>Decreto 1236 (Ley de Almacenes Generales de Depósito), CAUCA IV y RECAUCA IV (Arts. 119 al 129 - Régimen de Depósito Aduanero).</t>
         </is>
       </c>
-      <c r="H25" s="7" t="n">
+      <c r="H25" s="22" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="8" t="n">
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="24" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C26" s="24" t="inlineStr">
         <is>
           <t>ZDEEP - Entidades Administradoras</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="25" t="inlineStr">
         <is>
           <t>Administración de Zonas Especiales Públicas</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Personas jurídicas públicas o privadas autorizadas por ZOLIC y SAT para desarrollar y administrar polígonos industriales y logísticos ZDEEP.</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>Delimitación perimetral de polígonos, registro y control de garitas aduaneras, fiscalización de infraestructura física y control de accesos.</t>
-        </is>
-      </c>
-      <c r="G26" s="19" t="inlineStr">
+      <c r="E26" s="34" t="inlineStr">
+        <is>
+          <t>Personas jurídicas públicas o privadas autorizadas por ZOLIC y SAT para desarrollar, operar y vigilar la infraestructura de polígonos industriales y logísticos ZDEEP.</t>
+        </is>
+      </c>
+      <c r="F26" s="35" t="inlineStr">
+        <is>
+          <t>Delimita polígonos aduaneros, administra garitas de control y supervisa el perímetro de seguridad de la zona especial.</t>
+        </is>
+      </c>
+      <c r="G26" s="36" t="inlineStr">
         <is>
           <t>Decreto 22-73 (Ley Orgánica de ZOLIC reformada), CAUCA IV, RECAUCA IV y Resoluciones Conjuntas SAT-ZOLIC.</t>
         </is>
       </c>
-      <c r="H26" s="11" t="n">
+      <c r="H26" s="26" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="27" ht="42" customHeight="1">
-      <c r="A27" s="4" t="n">
+    <row r="27" ht="50" customHeight="1">
+      <c r="A27" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="20" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>ZDEEP - Empresas Usuarias</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>Transformación, Servicios y Exenciones</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>Empresas industriales, comerciales o de servicios instaladas y operando dentro de los recintos calificados como ZDEEP.</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>Ingreso y egreso de materias primas con suspensión de DAI/IVA, descargo de inventarios de transformación, goce de exenciones y traslados fiscales.</t>
-        </is>
-      </c>
-      <c r="G27" s="17" t="inlineStr">
-        <is>
-          <t>Decreto 22-73 (Régimen Fiscal ZDEEP), Ley de Actualización Tributaria y CAUCA/RECAUCA.</t>
-        </is>
-      </c>
-      <c r="H27" s="7" t="n">
+      <c r="E27" s="31" t="inlineStr">
+        <is>
+          <t>Empresas industriales, comerciales o de servicios instaladas y operando dentro de los recintos calificados como ZDEEP para producir o transformar con beneficios fiscales.</t>
+        </is>
+      </c>
+      <c r="F27" s="32" t="inlineStr">
+        <is>
+          <t>Ingresa materias primas con suspensión de DAI e IVA, realiza descargos de producción y goza de exenciones tributarias.</t>
+        </is>
+      </c>
+      <c r="G27" s="33" t="inlineStr">
+        <is>
+          <t>Decreto 22-73 (Régimen Fiscal ZDEEP), Ley de Actualización Tributaria (Decreto 10-2012) y CAUCA/RECAUCA IV.</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="28" ht="42" customHeight="1">
-      <c r="A28" s="8" t="n">
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="23" t="n">
         <v>22</v>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C28" s="24" t="inlineStr">
         <is>
           <t>Abogados y Notarios</t>
         </is>
       </c>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="D28" s="25" t="inlineStr">
         <is>
           <t>Papel Sellado de Protocolo y Avisos</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr">
-        <is>
-          <t>Abogados y notarios colegiados activos autorizados para dar fe pública en actos civiles y mercantiles ante la SAT.</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>Compra de Papel Sellado Especial para Protocolos (SAT-7130), timbres fiscales, traspasos electrónicos vehiculares (TEV) y avisos notariales obligatorios.</t>
-        </is>
-      </c>
-      <c r="G28" s="19" t="inlineStr">
-        <is>
-          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales (Decreto 37-92) y Código Tributario (Art. 57 "A").</t>
-        </is>
-      </c>
-      <c r="H28" s="11" t="n">
+      <c r="E28" s="34" t="inlineStr">
+        <is>
+          <t>Profesionales del derecho colegiados activos autorizados para ejercer la fe pública notarial, redactar instrumentos públicos y autorizar traspasos electrónicos de vehículos ante la SAT.</t>
+        </is>
+      </c>
+      <c r="F28" s="35" t="inlineStr">
+        <is>
+          <t>Compra papel sellado especial para protocolos, adquiere timbres fiscales, realiza traspasos vehiculares electrónicos (TEV) y presenta avisos notariales.</t>
+        </is>
+      </c>
+      <c r="G28" s="36" t="inlineStr">
+        <is>
+          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales y de Papel Sellado Especial para Protocolos (Decreto 37-92) y Código Tributario.</t>
+        </is>
+      </c>
+      <c r="H28" s="26" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="29" ht="42" customHeight="1">
-      <c r="A29" s="4" t="n">
+    <row r="29" ht="50" customHeight="1">
+      <c r="A29" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>Peritos Contadores</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D29" s="21" t="inlineStr">
         <is>
           <t>Libros Contables y Declaraciones</t>
         </is>
       </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>Peritos contadores habilitados ante la SAT para firmar balances, registrar contabilidades y asesorar contribuyentes.</t>
-        </is>
-      </c>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>Inscripción y actualización en el Registro de Contadores, autorización de libros contables digitales, presentación de balances y retenciones.</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>Decreto 2450 (Normas de la Profesión Contable), Código de Comercio y Código Tributario (Arts. 112 y 120).</t>
-        </is>
-      </c>
-      <c r="H29" s="7" t="n">
+      <c r="E29" s="31" t="inlineStr">
+        <is>
+          <t>Técnicos y profesionales contables inscritos y autorizados ante la SAT para llevar y firmar registros contables de contribuyentes, certificar estados financieros y realizar gestiones tributarias.</t>
+        </is>
+      </c>
+      <c r="F29" s="32" t="inlineStr">
+        <is>
+          <t>Inscríbete y actualiza tus datos en el Registro de Contadores, autoriza libros contables computarizados y asocia contribuyentes a tu perfil.</t>
+        </is>
+      </c>
+      <c r="G29" s="33" t="inlineStr">
+        <is>
+          <t>Decreto 2450 (Normas que Regulan el Ejercicio de la Profesión de Contador), Código de Comercio (Decreto 2-70) y Código Tributario (Arts. 112 y 120).</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="30" ht="42" customHeight="1">
-      <c r="A30" s="8" t="n">
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="23" t="n">
         <v>24</v>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="24" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C30" s="24" t="inlineStr">
         <is>
           <t>Auditores</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D30" s="25" t="inlineStr">
         <is>
           <t>Dictámenes Tributarios y Devolución IVA</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>Auditores y firmas contables independientes colegiadas encargadas de dictaminar estados financieros e informes fiscales.</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="inlineStr">
-        <is>
-          <t>Emisión de dictámenes de crédito fiscal para exportadores, dictámenes de precios de transferencia y auditorías requeridas por SAT.</t>
-        </is>
-      </c>
-      <c r="G30" s="19" t="inlineStr">
-        <is>
-          <t>Ley del IVA (Decreto 27-92, Art. 23 bis), Decreto 10-2012 y Ley de Colegiación Profesional Obligatoria (Decreto 72-2001).</t>
-        </is>
-      </c>
-      <c r="H30" s="11" t="n">
+      <c r="E30" s="34" t="inlineStr">
+        <is>
+          <t>Contadores Públicos y Auditores (CPA) colegiados activos y firmas de auditoría facultados para emitir dictámenes sobre estados financieros, devolución de crédito fiscal e informes de precios de transferencia.</t>
+        </is>
+      </c>
+      <c r="F30" s="35" t="inlineStr">
+        <is>
+          <t>Emite dictámenes de crédito fiscal para exportadores, dictámenes de estados financieros para licitaciones y presenta informes tributarios requeridos por SAT.</t>
+        </is>
+      </c>
+      <c r="G30" s="36" t="inlineStr">
+        <is>
+          <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001), Ley del IVA (Decreto 27-92, Art. 23 bis) y Ley de Actualización Tributaria (Decreto 10-2012).</t>
+        </is>
+      </c>
+      <c r="H30" s="26" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="31" ht="42" customHeight="1">
-      <c r="A31" s="4" t="n">
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="20" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>Gestores Tributarios</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>Gafetes y Trámites Presenciales</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
-        <is>
-          <t>Personas autorizadas formalmente para representar y gestionar trámites administrativos de terceros ante las oficinas y agencias de la SAT.</t>
-        </is>
-      </c>
-      <c r="F31" s="16" t="inlineStr">
-        <is>
-          <t>Acreditación oficial, renovación anual de gafetes, registro de huella biométrica y gestión presencial en ventanillas de atención.</t>
-        </is>
-      </c>
-      <c r="G31" s="17" t="inlineStr">
-        <is>
-          <t>Acuerdos de Directorio de la SAT sobre Acreditación y Regulación de Gestores Tributarios y Código Tributario.</t>
-        </is>
-      </c>
-      <c r="H31" s="7" t="n">
+      <c r="E31" s="31" t="inlineStr">
+        <is>
+          <t>Personas individuales autorizadas y acreditadas formalmente ante la SAT para representar a terceros en la tramitación presencial de gestiones administrativas tributarias y aduaneras.</t>
+        </is>
+      </c>
+      <c r="F31" s="32" t="inlineStr">
+        <is>
+          <t>Tramita y renueva tu carné oficial de gestor tributario, registra tus datos biométricos y gestiona expedientes autorizados en agencias tributarias.</t>
+        </is>
+      </c>
+      <c r="G31" s="33" t="inlineStr">
+        <is>
+          <t>Acuerdos de Directorio de la SAT sobre Regulación y Acreditación de Gestores Tributarios y Código Tributario.</t>
+        </is>
+      </c>
+      <c r="H31" s="22" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="32" ht="42" customHeight="1">
-      <c r="A32" s="8" t="n">
+    <row r="32" ht="50" customHeight="1">
+      <c r="A32" s="23" t="n">
         <v>26</v>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="24" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C32" s="24" t="inlineStr">
         <is>
           <t>Servicios Profesionales</t>
         </is>
       </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D32" s="25" t="inlineStr">
         <is>
           <t>Facturación por Honorarios y Retenciones</t>
         </is>
       </c>
-      <c r="E32" s="18" t="inlineStr">
-        <is>
-          <t>Médicos, ingenieros, arquitectos, consultores y profesionales que ejercen de forma independiente prestando servicios técnicos.</t>
-        </is>
-      </c>
-      <c r="F32" s="18" t="inlineStr">
-        <is>
-          <t>Facturación electrónica FEL por honorarios, pago de retenciones de ISR, actualización de colegiado activo y solvencia fiscal.</t>
-        </is>
-      </c>
-      <c r="G32" s="19" t="inlineStr">
+      <c r="E32" s="34" t="inlineStr">
+        <is>
+          <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de consultoría por honorarios profesionales.</t>
+        </is>
+      </c>
+      <c r="F32" s="35" t="inlineStr">
+        <is>
+          <t>Emite facturas electrónicas FEL por honorarios, liquida retenciones de ISR, actualiza tu colegiado activo y consulta tu solvencia fiscal.</t>
+        </is>
+      </c>
+      <c r="G32" s="36" t="inlineStr">
         <is>
           <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del IVA (Decreto 27-92).</t>
         </is>
       </c>
-      <c r="H32" s="11" t="n">
+      <c r="H32" s="26" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="33" ht="42" customHeight="1">
-      <c r="A33" s="4" t="n">
+    <row r="33" ht="50" customHeight="1">
+      <c r="A33" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>Constitucionales</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="21" t="inlineStr">
         <is>
           <t>Exenciones Tributarias de Rango Constitucional</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
-        <is>
-          <t>Centros educativos, universidades, misiones diplomáticas, comunidades religiosas e iglesias con exención expresa en la Carta Magna.</t>
-        </is>
-      </c>
-      <c r="F33" s="16" t="inlineStr">
-        <is>
-          <t>Registro de personería exenta en RTU, emisión de constancias de exención del IVA y timbres, y acreditación de representación legal.</t>
-        </is>
-      </c>
-      <c r="G33" s="17" t="inlineStr">
+      <c r="E33" s="31" t="inlineStr">
+        <is>
+          <t>Instituciones educativas, universidades, comunidades religiosas, misiones diplomáticas y cuerpos consulares que gozan de exención de impuestos por mandato directo de la Carta Magna.</t>
+        </is>
+      </c>
+      <c r="F33" s="32" t="inlineStr">
+        <is>
+          <t>Inscribe tu personería jurídica exenta en el RTU, emite constancias electrónicas de exención de IVA y timbres, y acredita representación legal.</t>
+        </is>
+      </c>
+      <c r="G33" s="33" t="inlineStr">
         <is>
           <t>Constitución Política de la República de Guatemala (Arts. 37, 73, 88), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
         </is>
       </c>
-      <c r="H33" s="7" t="n">
+      <c r="H33" s="22" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="34" ht="42" customHeight="1">
-      <c r="A34" s="8" t="n">
+    <row r="34" ht="50" customHeight="1">
+      <c r="A34" s="23" t="n">
         <v>28</v>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="24" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C34" s="24" t="inlineStr">
         <is>
           <t>No Lucrativos</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D34" s="25" t="inlineStr">
         <is>
           <t>Reconocimiento de Exención de ISR e IVA</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
-        <is>
-          <t>Asociaciones civiles, fundaciones benéficas, cooperativas de ahorro y gremiales legalmente constituidas sin fines de lucro.</t>
-        </is>
-      </c>
-      <c r="F34" s="18" t="inlineStr">
-        <is>
-          <t>Trámite de resolución de exención de ISR, actualización de estatutos, retenciones a terceros y presentación de informes anuales.</t>
-        </is>
-      </c>
-      <c r="G34" s="19" t="inlineStr">
-        <is>
-          <t>Decreto 02-2003 (Ley de ONGs), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
-        </is>
-      </c>
-      <c r="H34" s="11" t="n">
+      <c r="E34" s="34" t="inlineStr">
+        <is>
+          <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas, asociaciones civiles sin fines de lucro y cooperativas que solicitan reconocimiento administrativo de exención de ISR e IVA.</t>
+        </is>
+      </c>
+      <c r="F34" s="35" t="inlineStr">
+        <is>
+          <t>Solicita tu resolución formal de exención de ISR, actualiza estatutos y junta directiva en el RTU y emite constancias de retención y exención.</t>
+        </is>
+      </c>
+      <c r="G34" s="36" t="inlineStr">
+        <is>
+          <t>Decreto 02-2003 (Ley de ONGs para el Desarrollo), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
+        </is>
+      </c>
+      <c r="H34" s="26" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="35" ht="42" customHeight="1">
-      <c r="A35" s="4" t="n">
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>Municipalidades</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>Autonomía Municipal y Régimen Exento</t>
         </is>
       </c>
-      <c r="E35" s="16" t="inlineStr">
-        <is>
-          <t>Las 340 municipalidades del país, mancomunidades y empresas municipales autónomas prestadoras de servicios públicos.</t>
-        </is>
-      </c>
-      <c r="F35" s="16" t="inlineStr">
-        <is>
-          <t>Inscripción de alcaldes y tesoreros en RTU, registro de flotillas vehiculares municipales exentas del ISCV y constancias de exención.</t>
-        </is>
-      </c>
-      <c r="G35" s="17" t="inlineStr">
+      <c r="E35" s="31" t="inlineStr">
+        <is>
+          <t>Las 340 corporaciones municipales autónomas de la República de Guatemala, mancomunidades y empresas municipales públicas prestadoras de servicios comunitarios.</t>
+        </is>
+      </c>
+      <c r="F35" s="32" t="inlineStr">
+        <is>
+          <t>Registra autoridades y tesoreros en el RTU, gestiona la exención del impuesto de circulación para flotillas municipales y tramita solvencias institucionales.</t>
+        </is>
+      </c>
+      <c r="G35" s="33" t="inlineStr">
         <is>
           <t>Constitución Política de la República (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
         </is>
       </c>
-      <c r="H35" s="7" t="n">
+      <c r="H35" s="22" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="36" ht="42" customHeight="1">
-      <c r="A36" s="8" t="n">
+    <row r="36" ht="50" customHeight="1">
+      <c r="A36" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="24" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="24" t="inlineStr">
         <is>
           <t>Entidades del Estado</t>
         </is>
       </c>
-      <c r="D36" s="10" t="inlineStr">
+      <c r="D36" s="25" t="inlineStr">
         <is>
           <t>Compras Públicas y Agentes de Retención</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
-        <is>
-          <t>Dependencias del Organismo Ejecutivo, Legislativo, Judicial, entidades autónomas y descentralizadas del sector público.</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="inlineStr">
-        <is>
-          <t>Registro de unidades ejecutoras en RTU, emisión de constancias de retención del IVA/ISR en compras del Estado y gestión vehicular oficial.</t>
-        </is>
-      </c>
-      <c r="G36" s="19" t="inlineStr">
-        <is>
-          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Decreto 10-2012 y Código Tributario.</t>
-        </is>
-      </c>
-      <c r="H36" s="11" t="n">
+      <c r="E36" s="34" t="inlineStr">
+        <is>
+          <t>Ministerios de Estado, secretarías, organismos de los poderes Ejecutivo, Legislativo y Judicial, y entidades públicas descentralizadas que operan como agentes de retención del IVA e ISR.</t>
+        </is>
+      </c>
+      <c r="F36" s="35" t="inlineStr">
+        <is>
+          <t>Habilita unidades ejecutoras en el RTU, emite constancias de retención en compras públicas y administra el parque vehicular oficial del Estado.</t>
+        </is>
+      </c>
+      <c r="G36" s="36" t="inlineStr">
+        <is>
+          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
+        </is>
+      </c>
+      <c r="H36" s="26" t="n">
         <v>26</v>
       </c>
     </row>
-    <row r="37" ht="42" customHeight="1">
-      <c r="A37" s="4" t="n">
+    <row r="37" ht="50" customHeight="1">
+      <c r="A37" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="20" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>Decreto</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D37" s="21" t="inlineStr">
         <is>
           <t>Exenciones y Fomento por Decreto Legislativo</t>
         </is>
       </c>
-      <c r="E37" s="16" t="inlineStr">
-        <is>
-          <t>Entidades o proyectos con beneficios fiscales otorgados por leyes ordinarias de fomento sectorial (turismo, energía renovable, reforestación).</t>
-        </is>
-      </c>
-      <c r="F37" s="16" t="inlineStr">
-        <is>
-          <t>Acreditación de resolución ministerial o dictamen de beneficio fiscal, exenciones específicas de aranceles y reporte periódico.</t>
-        </is>
-      </c>
-      <c r="G37" s="17" t="inlineStr">
-        <is>
-          <t>Decretos Legislativos específicos de fomento (Decreto 29-89, Decreto 65-89, Ley de Fomento a las Energías Renovables) y Código Tributario.</t>
-        </is>
-      </c>
-      <c r="H37" s="7" t="n">
+      <c r="E37" s="31" t="inlineStr">
+        <is>
+          <t>Personas o entidades beneficiarias de leyes de fomento económico y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso.</t>
+        </is>
+      </c>
+      <c r="F37" s="32" t="inlineStr">
+        <is>
+          <t>Acredita resoluciones ministeriales de calificación de fomento, gestiona exenciones arancelarias temporales y presenta reportes periódicos de cumplimiento.</t>
+        </is>
+      </c>
+      <c r="G37" s="33" t="inlineStr">
+        <is>
+          <t>Decretos específicos de fomento (Decreto 29-89 de Maquilas, Decreto 65-89 de Zonas Francas, Ley de Incentivos para Energías Renovables) y Código Tributario.</t>
+        </is>
+      </c>
+      <c r="H37" s="22" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(arquitectura): homologar Resumen Arquitectura en libro del Mapa con metodologia ATO e Interacciones completa
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -20,8 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="12">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,7 +47,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -56,7 +58,12 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E293B"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
@@ -79,22 +86,11 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <color rgb="00475569"/>
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -133,12 +129,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
@@ -156,13 +146,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FFFFFF"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -179,9 +183,38 @@
       </bottom>
     </border>
     <border>
-      <left style="thin">
+      <left/>
+      <right/>
+      <top style="medium">
         <color rgb="00FFFFFF"/>
-      </left>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color rgb="00FFFFFF"/>
       </right>
@@ -191,12 +224,13 @@
       <bottom style="medium">
         <color rgb="00FFFFFF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -220,74 +254,78 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -653,17 +691,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H29"/>
+  <dimension ref="B2:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -677,14 +715,14 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>RESUMEN EJECUTIVO DE ARQUITECTURA DE INFORMACIÓN — DEFINICIÓN DE SEGMENTOS, LEAD TEXT Y BASE JURÍDICA</t>
+          <t>ARQUITECTURA DE INFORMACIÓN DEL PORTAL WEB — DEFINICIÓN DE SEGMENTOS, LEAD TEXT, ATO Y BASE JURÍDICA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>TOTAL DEL PORTAL
+          <t>TOTAL CONTENIDOS
 739 Trámites</t>
         </is>
       </c>
@@ -700,13 +738,13 @@
 202 Trámites</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>PROFESIONALES
 45 Trámites</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>ENTES EXENTOS
 79 Trámites</t>
@@ -717,255 +755,528 @@
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>1. RESUMEN ESTRUCTURAL POR SEGMENTO (NIVEL 1) — DEFINICIONES INSTITUCIONALES</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  OPERADORES DE COMERCIO EXTERIOR  (202 Trámites — 27.3% del Portal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="44" customHeight="1">
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Qué es:</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
+          <t>1. SEGMENTOS PRINCIPALES DEL PORTAL (NIVEL 1) — DEFINICIONES INSTITUCIONALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Segmento (Nivel 1)</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Qué es: (Definición Operativa)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Lead text: (Texto Orientador de Interfaz)</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Base jurídica: (Fundamento Legal Oficial: CAUCA, RECAUCA, Leyes)</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Total Contenidos</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>% del Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1">
+      <c r="B11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Son todas las personas individuales o jurídicas que intervienen en el ingreso, permanencia, traslado y salida de mercancías del territorio aduanero nacional. Comprende tanto a los dueños de las mercancías (importadores y exportadores) como a los prestadores de servicios logísticos autorizados (auxiliares de la función pública, transportistas, depósitos) y empresas que operan bajo regímenes territoriales especiales.</t>
         </is>
       </c>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Lead text:</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Gestiona tus trámites aduaneros, consulta requisitos y haz seguimiento a tus operaciones según tu rol en la cadena logística.</t>
         </is>
       </c>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="n"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Base jurídica:</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>Código Tributario (Dto. 6-91), CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA (Resolución 224-2008 COMIECO).</t>
         </is>
       </c>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="12" t="n"/>
-      <c r="F14" s="12" t="n"/>
-      <c r="G14" s="12" t="n"/>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  CONTRIBUYENTES  (413 Trámites — 55.9% del Portal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Qué es:</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="G11" s="15" t="n">
+        <v>202</v>
+      </c>
+      <c r="H11" s="16">
+        <f>G11/$G$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="56" customHeight="1">
+      <c r="B12" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Contribuyentes</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>Son las personas individuales, jurídicas, patrimonios o entes afectos al cumplimiento de obligaciones tributarias internas en el territorio guatemalteco. Abarca a ciudadanos sin actividad económica activa, asalariados en relación de dependencia, pequeños contribuyentes, contribuyentes del régimen general del IVA e ISR, propietarios de vehículos y grandes/medianos contribuyentes especiales calificados.</t>
         </is>
       </c>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="12" t="n"/>
-      <c r="G17" s="12" t="n"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Lead text:</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>Cumple con tus obligaciones tributarias, emite tus facturas, actualiza tu RTU y gestiona tus trámites de vehículos e impuestos internos de forma ágil y 100% digital.</t>
         </is>
       </c>
-      <c r="D18" s="12" t="n"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Base jurídica:</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="F12" s="21" t="inlineStr">
         <is>
           <t>Constitución Política (Art. 135d), Código Tributario (Dto. 6-91), Ley del IVA (Dto. 27-92), Ley de Actualización Tributaria (Dto. 10-2012), Ley del ISCV (Dto. 70-94) y Ley de Simplificación Tributaria (Dto. 7-2019 / Dto. 31-2024).</t>
         </is>
       </c>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12" t="n"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PROFESIONALES  (45 Trámites — 6.1% del Portal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="44" customHeight="1">
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Qué es:</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="G12" s="22" t="n">
+        <v>413</v>
+      </c>
+      <c r="H12" s="23">
+        <f>G12/$G$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="56" customHeight="1">
+      <c r="B13" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Son las personas individuales colegiadas activas o técnicos acreditados ante la SAT que ejercen liberalmente su profesión o actúan como auxiliares técnicos en materia tributaria, mercantil y notarial. Comprende a abogados y notarios (traspasos vehiculares electrónicos y fe pública), peritos contadores, contadores públicos y auditores (CPA) y gestores tributarios acreditados.</t>
         </is>
       </c>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
-      <c r="F22" s="12" t="n"/>
-      <c r="G22" s="12" t="n"/>
-    </row>
-    <row r="23" ht="28" customHeight="1">
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Lead text:</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Accede a herramientas especializadas de fe pública, autorización de libros contables, presentación de dictámenes fiscales y gestión de trámites profesionales.</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="12" t="n"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>Base jurídica:</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Código de Notariado (Dto. 314), Ley de Colegiación Profesional Obligatoria (Dto. 72-2001), Decreto 2450 (Normas de la Profesión Contable), Ley de Timbres Fiscales (Dto. 37-92) y Código Tributario (Art. 57 "A" y 112).</t>
         </is>
       </c>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
-    </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ENTES EXENTOS  (79 Trámites — 10.7% del Portal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="44" customHeight="1">
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>Qué es:</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="G13" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="H13" s="16">
+        <f>G13/$G$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1">
+      <c r="B14" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>Son las personas jurídicas, entidades del sector público, organismos diplomáticos y organizaciones de la sociedad civil que, por mandato constitucional o ley específica ordinaria, gozan de exención total o parcial de tributos y aranceles en el territorio nacional. Incluye centros educativos, universidades, comunidades religiosas, ONGs, fundaciones sin fines de lucro, municipalidades y ministerios de Estado.</t>
         </is>
       </c>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="12" t="n"/>
-      <c r="F27" s="12" t="n"/>
-      <c r="G27" s="12" t="n"/>
-    </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Lead text:</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>Solicita y gestiona tus resoluciones de exención, emite constancias tributarias electrónicas y administra las obligaciones formales de tu entidad.</t>
         </is>
       </c>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12" t="n"/>
-    </row>
-    <row r="29" ht="32" customHeight="1">
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Base jurídica:</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>Constitución Política (Arts. 37, 73, 88 y 257), Ley de ONGs (Dto. 02-2003), Ley del IVA (Dto. 27-92, Art. 8), Ley de Actualización Tributaria (Dto. 10-2012, Art. 11), Código Municipal (Dto. 12-2002) y Ley Orgánica del Presupuesto (Dto. 101-97).</t>
         </is>
       </c>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
+      <c r="G14" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="H14" s="23">
+        <f>G14/$G$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="B15" s="24" t="inlineStr"/>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL PORTAL WEB SAT</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Universo total de fichas y servicios</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="inlineStr"/>
+      <c r="F15" s="24" t="inlineStr"/>
+      <c r="G15" s="27">
+        <f>SUM(G11:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="28">
+        <f>SUM(H11:H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>2. METODOLOGÍA CICLO DE VIDA ATO (AUSTRALIA) - SIN NÚMEROS VISIBLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>Etapa ATO</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>Descripción Funcional</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="n"/>
+      <c r="E18" s="30" t="n"/>
+      <c r="F18" s="31" t="n"/>
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t>Total Contenidos</t>
+        </is>
+      </c>
+      <c r="H18" s="29" t="inlineStr">
+        <is>
+          <t>% del Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Empezar y registrarse</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>Primer NIT, RTU Digital, padrones de importación/exportación y habilitación inicial</t>
+        </is>
+      </c>
+      <c r="D19" s="33" t="n"/>
+      <c r="E19" s="33" t="n"/>
+      <c r="F19" s="33" t="n"/>
+      <c r="G19" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="H19" s="16">
+        <f>G19/$G$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Operación y declaraciones</t>
+        </is>
+      </c>
+      <c r="C20" s="34" t="inlineStr">
+        <is>
+          <t>Facturación FEL, Declaraguate, DUCAs, retenciones, transferencias y pagos</t>
+        </is>
+      </c>
+      <c r="D20" s="35" t="n"/>
+      <c r="E20" s="35" t="n"/>
+      <c r="F20" s="35" t="n"/>
+      <c r="G20" s="22" t="n">
+        <v>260</v>
+      </c>
+      <c r="H20" s="23">
+        <f>G20/$G$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Consultas y herramientas</t>
+        </is>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>Verificadores en tiempo real, solvencia, selectivo aduanero, rampa y SAC</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="33" t="n"/>
+      <c r="G21" s="15" t="n">
+        <v>123</v>
+      </c>
+      <c r="H21" s="16">
+        <f>G21/$G$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Modificaciones y cierre</t>
+        </is>
+      </c>
+      <c r="C22" s="34" t="inlineStr">
+        <is>
+          <t>Actualización de RTU, traspaso vehicular, prórrogas, cese de actividades y subastas</t>
+        </is>
+      </c>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="35" t="n"/>
+      <c r="F22" s="35" t="n"/>
+      <c r="G22" s="22" t="n">
+        <v>123</v>
+      </c>
+      <c r="H22" s="23">
+        <f>G22/$G$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Normativa y asistencia</t>
+        </is>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Marco legal aduanero y tributario, devoluciones, criterios institucionales y cursos</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="15" t="n">
+        <v>137</v>
+      </c>
+      <c r="H23" s="16">
+        <f>G23/$G$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="B24" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL POR CICLO ATO</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>100% de contenidos clasificados según ciclo de vida del contribuyente</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="24" t="n"/>
+      <c r="G24" s="27">
+        <f>SUM(G19:G23)</f>
+        <v/>
+      </c>
+      <c r="H24" s="28">
+        <f>SUM(H19:H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>3. TIPOS DE INTERACCIÓN (CÓMO RESUELVE EL CIUDADANO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>Tipo de Interacción</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t>Modalidad Operativa</t>
+        </is>
+      </c>
+      <c r="D27" s="30" t="n"/>
+      <c r="E27" s="30" t="n"/>
+      <c r="F27" s="31" t="n"/>
+      <c r="G27" s="36" t="inlineStr">
+        <is>
+          <t>Total Contenidos</t>
+        </is>
+      </c>
+      <c r="H27" s="36" t="inlineStr">
+        <is>
+          <t>% del Portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Guía Informativa / Texto</t>
+        </is>
+      </c>
+      <c r="C28" s="34" t="inlineStr">
+        <is>
+          <t>Páginas explicativas, requisitos de trámites presenciales o mixtos</t>
+        </is>
+      </c>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
+      <c r="G28" s="22" t="n">
+        <v>462</v>
+      </c>
+      <c r="H28" s="23">
+        <f>G28/$G$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Trámite / Aplicativo en Línea</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="inlineStr">
+        <is>
+          <t>Servicios digitales transaccionales (Agencia Virtual, Declaraguate, TEV, FEL)</t>
+        </is>
+      </c>
+      <c r="D29" s="33" t="n"/>
+      <c r="E29" s="33" t="n"/>
+      <c r="F29" s="33" t="n"/>
+      <c r="G29" s="15" t="n">
+        <v>187</v>
+      </c>
+      <c r="H29" s="16">
+        <f>G29/$G$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>Consulta en Base de Datos</t>
+        </is>
+      </c>
+      <c r="C30" s="34" t="inlineStr">
+        <is>
+          <t>Herramientas de verificación sin autenticación previa (RTU público, solvencias)</t>
+        </is>
+      </c>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="35" t="n"/>
+      <c r="G30" s="22" t="n">
+        <v>83</v>
+      </c>
+      <c r="H30" s="23">
+        <f>G30/$G$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Descarga de Documento / Software</t>
+        </is>
+      </c>
+      <c r="C31" s="32" t="inlineStr">
+        <is>
+          <t>Descarga de formularios en PDF/Excel, software, manuales o legislación</t>
+        </is>
+      </c>
+      <c r="D31" s="33" t="n"/>
+      <c r="E31" s="33" t="n"/>
+      <c r="F31" s="33" t="n"/>
+      <c r="G31" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="H31" s="16">
+        <f>G31/$G$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="B32" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL INTERACCIONES</t>
+        </is>
+      </c>
+      <c r="C32" s="26" t="inlineStr">
+        <is>
+          <t>100% de contenidos catalogados según interacción digital</t>
+        </is>
+      </c>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="27">
+        <f>SUM(G28:G31)</f>
+        <v/>
+      </c>
+      <c r="H32" s="28">
+        <f>SUM(H28:H31)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="C24:G24"/>
+  <mergeCells count="20">
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="G6:H7"/>
     <mergeCell ref="B2:H3"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C18:F18"/>
     <mergeCell ref="B4:H4"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C24:F24"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="F6:G7"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="D6:E7"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="C21:F21"/>
     <mergeCell ref="C6:C7"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="F6:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1005,1084 +1316,1084 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Nivel 1: Segmento Oficial</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Nivel 2: Categoría / Área</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Nivel 3: Grupo / Actor Específico</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Nivel 4: Tema / Especialidad</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Trámites Contenidos</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Ruta de Navegación de Entrada (Miga de Pan)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="37" t="inlineStr">
         <is>
           <t>NIT sin Obligaciones</t>
         </is>
       </c>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="E7" s="33" t="inlineStr">
         <is>
           <t>Personas Individuales</t>
         </is>
       </c>
-      <c r="F7" s="21" t="inlineStr">
+      <c r="F7" s="33" t="inlineStr">
         <is>
           <t>RTU Digital y Solicitud de NIT</t>
         </is>
       </c>
-      <c r="G7" s="22" t="n">
+      <c r="G7" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="H7" s="33" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; NIT sin Obligaciones &gt; RTU Digital y Solicitud de NIT</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
+      <c r="D8" s="38" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="E8" s="25" t="inlineStr">
+      <c r="E8" s="35" t="inlineStr">
         <is>
           <t>Pequeño Contribuyente General</t>
         </is>
       </c>
-      <c r="F8" s="25" t="inlineStr">
+      <c r="F8" s="35" t="inlineStr">
         <is>
           <t>Régimen de 5% y Facturación FEL</t>
         </is>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="H8" s="25" t="inlineStr">
+      <c r="H8" s="35" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Régimen de 5% y Facturación FEL</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="19" t="n">
+      <c r="B9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D9" s="37" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="E9" s="33" t="inlineStr">
         <is>
           <t>Sector Primario y Agropecuario</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr">
+      <c r="F9" s="33" t="inlineStr">
         <is>
           <t>Regímenes Especiales Decreto 31-2024 / 7-2019</t>
         </is>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="G9" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="H9" s="33" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Regímenes Especiales Decreto 31-2024 / 7-2019</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
       </c>
-      <c r="E10" s="25" t="inlineStr">
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>Personas y Empresas en Régimen General</t>
         </is>
       </c>
-      <c r="F10" s="25" t="inlineStr">
+      <c r="F10" s="35" t="inlineStr">
         <is>
           <t>IVA General e Impuesto Sobre la Renta (ISR)</t>
         </is>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="25" t="inlineStr">
+      <c r="H10" s="35" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; IVA General e Impuesto Sobre la Renta (ISR)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D11" s="20" t="inlineStr">
+      <c r="D11" s="37" t="inlineStr">
         <is>
           <t>Asalariados</t>
         </is>
       </c>
-      <c r="E11" s="21" t="inlineStr">
+      <c r="E11" s="33" t="inlineStr">
         <is>
           <t>Trabajadores en Relación de Dependencia</t>
         </is>
       </c>
-      <c r="F11" s="21" t="inlineStr">
+      <c r="F11" s="33" t="inlineStr">
         <is>
           <t>Retenciones de ISR y Planilla del IVA</t>
         </is>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="G11" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="21" t="inlineStr">
+      <c r="H11" s="33" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Asalariados &gt; Retenciones de ISR y Planilla del IVA</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="D12" s="38" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
-      <c r="E12" s="25" t="inlineStr">
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>Propietarios y Compradores de Vehículos</t>
         </is>
       </c>
-      <c r="F12" s="25" t="inlineStr">
+      <c r="F12" s="35" t="inlineStr">
         <is>
           <t>Registro Fiscal de Vehículos (RFV)</t>
         </is>
       </c>
-      <c r="G12" s="26" t="n">
+      <c r="G12" s="22" t="n">
         <v>72</v>
       </c>
-      <c r="H12" s="25" t="inlineStr">
+      <c r="H12" s="35" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Vehículos &gt; Registro Fiscal de Vehículos (RFV)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="19" t="n">
+      <c r="B13" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes Especiales</t>
         </is>
       </c>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="E13" s="33" t="inlineStr">
         <is>
           <t>Grandes y Medianos Contribuyentes</t>
         </is>
       </c>
-      <c r="F13" s="21" t="inlineStr">
+      <c r="F13" s="33" t="inlineStr">
         <is>
           <t>Gerencias Especializadas de Fiscalización</t>
         </is>
       </c>
-      <c r="G13" s="22" t="n">
+      <c r="G13" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="H13" s="21" t="inlineStr">
+      <c r="H13" s="33" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyentes Especiales &gt; Gerencias Especializadas de Fiscalización</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D14" s="38" t="inlineStr">
         <is>
           <t>Facturación Electrónica</t>
         </is>
       </c>
-      <c r="E14" s="25" t="inlineStr">
+      <c r="E14" s="35" t="inlineStr">
         <is>
           <t>Emisores de DTE</t>
         </is>
       </c>
-      <c r="F14" s="25" t="inlineStr">
+      <c r="F14" s="35" t="inlineStr">
         <is>
           <t>Sistema FEL y Agencia Virtual</t>
         </is>
       </c>
-      <c r="G14" s="26" t="n">
+      <c r="G14" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H14" s="25" t="inlineStr">
+      <c r="H14" s="35" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Facturación Electrónica &gt; Sistema FEL y Agencia Virtual</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D15" s="20" t="inlineStr">
+      <c r="D15" s="37" t="inlineStr">
         <is>
           <t>Servicios al Contribuyente</t>
         </is>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E15" s="33" t="inlineStr">
         <is>
           <t>Ciudadanía y Usuarios de Agencia Virtual</t>
         </is>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="F15" s="33" t="inlineStr">
         <is>
           <t>Plataforma Digital, Citas y Solvencias</t>
         </is>
       </c>
-      <c r="G15" s="22" t="n">
+      <c r="G15" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="H15" s="21" t="inlineStr">
+      <c r="H15" s="33" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Servicios al Contribuyente &gt; Plataforma Digital, Citas y Solvencias</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C16" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D16" s="38" t="inlineStr">
         <is>
           <t>Importadores y Exportadores (Compartido)</t>
         </is>
       </c>
-      <c r="E16" s="25" t="inlineStr">
+      <c r="E16" s="35" t="inlineStr">
         <is>
           <t>Operadores Comerciales Generales</t>
         </is>
       </c>
-      <c r="F16" s="25" t="inlineStr">
+      <c r="F16" s="35" t="inlineStr">
         <is>
           <t>Gestiones Aduaneras Comunes y Arancel</t>
         </is>
       </c>
-      <c r="G16" s="26" t="n">
+      <c r="G16" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H16" s="25" t="inlineStr">
+      <c r="H16" s="35" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Importadores y Exportadores (Compartido) &gt; Gestiones Aduaneras Comunes y Arancel</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="19" t="n">
+      <c r="B17" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="37" t="inlineStr">
         <is>
           <t>Importadores</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="33" t="inlineStr">
         <is>
           <t>Importadores Registrados</t>
         </is>
       </c>
-      <c r="F17" s="21" t="inlineStr">
+      <c r="F17" s="33" t="inlineStr">
         <is>
           <t>Padrón de Importadores y DUCA-D</t>
         </is>
       </c>
-      <c r="G17" s="22" t="n">
+      <c r="G17" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="H17" s="21" t="inlineStr">
+      <c r="H17" s="33" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Importadores &gt; Padrón de Importadores y DUCA-D</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="C18" s="24" t="inlineStr">
+      <c r="C18" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D18" s="24" t="inlineStr">
+      <c r="D18" s="38" t="inlineStr">
         <is>
           <t>Exportadores</t>
         </is>
       </c>
-      <c r="E18" s="25" t="inlineStr">
+      <c r="E18" s="35" t="inlineStr">
         <is>
           <t>Exportadores Habituales y Ocasionales</t>
         </is>
       </c>
-      <c r="F18" s="25" t="inlineStr">
+      <c r="F18" s="35" t="inlineStr">
         <is>
           <t>Padrón de Exportadores y Devolución IVA</t>
         </is>
       </c>
-      <c r="G18" s="26" t="n">
+      <c r="G18" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="H18" s="25" t="inlineStr">
+      <c r="H18" s="35" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Exportadores &gt; Padrón de Exportadores y Devolución IVA</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="19" t="n">
+      <c r="B19" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="C19" s="20" t="inlineStr">
+      <c r="C19" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D19" s="37" t="inlineStr">
         <is>
           <t>Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E19" s="33" t="inlineStr">
         <is>
           <t>Operadores Certificados en Seguridad</t>
         </is>
       </c>
-      <c r="F19" s="21" t="inlineStr">
+      <c r="F19" s="33" t="inlineStr">
         <is>
           <t>Cadena Logística Segura y Carril Exprés</t>
         </is>
       </c>
-      <c r="G19" s="22" t="n">
+      <c r="G19" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="21" t="inlineStr">
+      <c r="H19" s="33" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Operador Económico Autorizado (OEA) &gt; Cadena Logística Segura y Carril Exprés</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="23" t="n">
+      <c r="B20" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="C20" s="24" t="inlineStr">
+      <c r="C20" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D20" s="24" t="inlineStr">
+      <c r="D20" s="38" t="inlineStr">
         <is>
           <t>Agentes Aduaneros</t>
         </is>
       </c>
-      <c r="E20" s="25" t="inlineStr">
+      <c r="E20" s="35" t="inlineStr">
         <is>
           <t>Auxiliares de la Función Pública Aduanera</t>
         </is>
       </c>
-      <c r="F20" s="25" t="inlineStr">
+      <c r="F20" s="35" t="inlineStr">
         <is>
           <t>Despacho Aduanero Oficial y Representación</t>
         </is>
       </c>
-      <c r="G20" s="26" t="n">
+      <c r="G20" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H20" s="25" t="inlineStr">
+      <c r="H20" s="35" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Agentes Aduaneros &gt; Despacho Aduanero Oficial y Representación</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="19" t="n">
+      <c r="B21" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C21" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D21" s="37" t="inlineStr">
         <is>
           <t>Apoderados Especiales Aduaneros</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E21" s="33" t="inlineStr">
         <is>
           <t>Representantes Legales Exclusivos</t>
         </is>
       </c>
-      <c r="F21" s="21" t="inlineStr">
+      <c r="F21" s="33" t="inlineStr">
         <is>
           <t>Despacho Aduanero por Cuenta Propia</t>
         </is>
       </c>
-      <c r="G21" s="22" t="n">
+      <c r="G21" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="H21" s="21" t="inlineStr">
+      <c r="H21" s="33" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Apoderados Especiales Aduaneros &gt; Despacho Aduanero por Cuenta Propia</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="23" t="n">
+      <c r="B22" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="C22" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D22" s="24" t="inlineStr">
+      <c r="D22" s="38" t="inlineStr">
         <is>
           <t>Empresas de Entrega Rápida o Courier</t>
         </is>
       </c>
-      <c r="E22" s="25" t="inlineStr">
+      <c r="E22" s="35" t="inlineStr">
         <is>
           <t>Mensajería y Envíos Expresos</t>
         </is>
       </c>
-      <c r="F22" s="25" t="inlineStr">
+      <c r="F22" s="35" t="inlineStr">
         <is>
           <t>Paquetería Internacional y Franquicias</t>
         </is>
       </c>
-      <c r="G22" s="26" t="n">
+      <c r="G22" s="22" t="n">
         <v>13</v>
       </c>
-      <c r="H22" s="25" t="inlineStr">
+      <c r="H22" s="35" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Empresas de Entrega Rápida o Courier &gt; Paquetería Internacional y Franquicias</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="19" t="n">
+      <c r="B23" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C23" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D23" s="37" t="inlineStr">
         <is>
           <t>Consolidadores y Desconsolidadores de Carga</t>
         </is>
       </c>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="E23" s="33" t="inlineStr">
         <is>
           <t>Operadores Logísticos y de Carga</t>
         </is>
       </c>
-      <c r="F23" s="21" t="inlineStr">
+      <c r="F23" s="33" t="inlineStr">
         <is>
           <t>Manifiestos CUSCAR y Guías Hijas</t>
         </is>
       </c>
-      <c r="G23" s="22" t="n">
+      <c r="G23" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="H23" s="21" t="inlineStr">
+      <c r="H23" s="33" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Consolidadores y Desconsolidadores de Carga &gt; Manifiestos CUSCAR y Guías Hijas</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="23" t="n">
+      <c r="B24" s="17" t="n">
         <v>18</v>
       </c>
-      <c r="C24" s="24" t="inlineStr">
+      <c r="C24" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D24" s="24" t="inlineStr">
+      <c r="D24" s="38" t="inlineStr">
         <is>
           <t>Transportistas Aduaneros</t>
         </is>
       </c>
-      <c r="E24" s="25" t="inlineStr">
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>Transporte Internacional Terrestre y Carga</t>
         </is>
       </c>
-      <c r="F24" s="25" t="inlineStr">
+      <c r="F24" s="35" t="inlineStr">
         <is>
           <t>Tránsito Aduanero Internacional y Marchamo</t>
         </is>
       </c>
-      <c r="G24" s="26" t="n">
+      <c r="G24" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H24" s="25" t="inlineStr">
+      <c r="H24" s="35" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Transportistas Aduaneros &gt; Tránsito Aduanero Internacional y Marchamo</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="B25" s="19" t="n">
+      <c r="B25" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="C25" s="20" t="inlineStr">
+      <c r="C25" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D25" s="20" t="inlineStr">
+      <c r="D25" s="37" t="inlineStr">
         <is>
           <t>Depósitos Aduaneros</t>
         </is>
       </c>
-      <c r="E25" s="21" t="inlineStr">
+      <c r="E25" s="33" t="inlineStr">
         <is>
           <t>Almacenes Fiscales, AGD y DAT</t>
         </is>
       </c>
-      <c r="F25" s="21" t="inlineStr">
+      <c r="F25" s="33" t="inlineStr">
         <is>
           <t>Custodia de Mercancías y Títulos de Crédito</t>
         </is>
       </c>
-      <c r="G25" s="22" t="n">
+      <c r="G25" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="H25" s="21" t="inlineStr">
+      <c r="H25" s="33" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; Depósitos Aduaneros &gt; Custodia de Mercancías y Títulos de Crédito</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="23" t="n">
+      <c r="B26" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="C26" s="24" t="inlineStr">
+      <c r="C26" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D26" s="24" t="inlineStr">
+      <c r="D26" s="38" t="inlineStr">
         <is>
           <t>ZDEEP - Entidades Administradoras</t>
         </is>
       </c>
-      <c r="E26" s="25" t="inlineStr">
+      <c r="E26" s="35" t="inlineStr">
         <is>
           <t>Polígonos ZDEEP</t>
         </is>
       </c>
-      <c r="F26" s="25" t="inlineStr">
+      <c r="F26" s="35" t="inlineStr">
         <is>
           <t>Administración de Zonas Especiales Públicas</t>
         </is>
       </c>
-      <c r="G26" s="26" t="n">
+      <c r="G26" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="H26" s="25" t="inlineStr">
+      <c r="H26" s="35" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; ZDEEP - Entidades Administradoras &gt; Administración de Zonas Especiales Públicas</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="19" t="n">
+      <c r="B27" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="C27" s="20" t="inlineStr">
+      <c r="C27" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D27" s="37" t="inlineStr">
         <is>
           <t>ZDEEP - Empresas Usuarias</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E27" s="33" t="inlineStr">
         <is>
           <t>Empresas Instaladas en ZDEEP</t>
         </is>
       </c>
-      <c r="F27" s="21" t="inlineStr">
+      <c r="F27" s="33" t="inlineStr">
         <is>
           <t>Transformación, Servicios y Exenciones</t>
         </is>
       </c>
-      <c r="G27" s="22" t="n">
+      <c r="G27" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="H27" s="21" t="inlineStr">
+      <c r="H27" s="33" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior &gt; ZDEEP - Empresas Usuarias &gt; Transformación, Servicios y Exenciones</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="23" t="n">
+      <c r="B28" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="C28" s="24" t="inlineStr">
+      <c r="C28" s="38" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D28" s="24" t="inlineStr">
+      <c r="D28" s="38" t="inlineStr">
         <is>
           <t>Abogados y Notarios</t>
         </is>
       </c>
-      <c r="E28" s="25" t="inlineStr">
+      <c r="E28" s="35" t="inlineStr">
         <is>
           <t>Notarios en Ejercicio</t>
         </is>
       </c>
-      <c r="F28" s="25" t="inlineStr">
+      <c r="F28" s="35" t="inlineStr">
         <is>
           <t>Papel Sellado de Protocolo y Avisos</t>
         </is>
       </c>
-      <c r="G28" s="26" t="n">
+      <c r="G28" s="22" t="n">
         <v>17</v>
       </c>
-      <c r="H28" s="25" t="inlineStr">
+      <c r="H28" s="35" t="inlineStr">
         <is>
           <t>Profesionales &gt; Abogados y Notarios &gt; Papel Sellado de Protocolo y Avisos</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="19" t="n">
+      <c r="B29" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="C29" s="20" t="inlineStr">
+      <c r="C29" s="37" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D29" s="20" t="inlineStr">
+      <c r="D29" s="37" t="inlineStr">
         <is>
           <t>Peritos Contadores</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E29" s="33" t="inlineStr">
         <is>
           <t>Contadores Registrados</t>
         </is>
       </c>
-      <c r="F29" s="21" t="inlineStr">
+      <c r="F29" s="33" t="inlineStr">
         <is>
           <t>Libros Contables y Declaraciones</t>
         </is>
       </c>
-      <c r="G29" s="22" t="n">
+      <c r="G29" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="H29" s="21" t="inlineStr">
+      <c r="H29" s="33" t="inlineStr">
         <is>
           <t>Profesionales &gt; Peritos Contadores &gt; Libros Contables y Declaraciones</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="23" t="n">
+      <c r="B30" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="C30" s="24" t="inlineStr">
+      <c r="C30" s="38" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D30" s="24" t="inlineStr">
+      <c r="D30" s="38" t="inlineStr">
         <is>
           <t>Auditores</t>
         </is>
       </c>
-      <c r="E30" s="25" t="inlineStr">
+      <c r="E30" s="35" t="inlineStr">
         <is>
           <t>Contadores Públicos y Auditores (CPA)</t>
         </is>
       </c>
-      <c r="F30" s="25" t="inlineStr">
+      <c r="F30" s="35" t="inlineStr">
         <is>
           <t>Dictámenes Tributarios y Devolución IVA</t>
         </is>
       </c>
-      <c r="G30" s="26" t="n">
+      <c r="G30" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="H30" s="25" t="inlineStr">
+      <c r="H30" s="35" t="inlineStr">
         <is>
           <t>Profesionales &gt; Auditores &gt; Dictámenes Tributarios y Devolución IVA</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="19" t="n">
+      <c r="B31" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C31" s="37" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="37" t="inlineStr">
         <is>
           <t>Gestores Tributarios</t>
         </is>
       </c>
-      <c r="E31" s="21" t="inlineStr">
+      <c r="E31" s="33" t="inlineStr">
         <is>
           <t>Gestores Acreditados SAT</t>
         </is>
       </c>
-      <c r="F31" s="21" t="inlineStr">
+      <c r="F31" s="33" t="inlineStr">
         <is>
           <t>Gafetes y Trámites Presenciales</t>
         </is>
       </c>
-      <c r="G31" s="22" t="n">
+      <c r="G31" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="H31" s="21" t="inlineStr">
+      <c r="H31" s="33" t="inlineStr">
         <is>
           <t>Profesionales &gt; Gestores Tributarios &gt; Gafetes y Trámites Presenciales</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="23" t="n">
+      <c r="B32" s="17" t="n">
         <v>26</v>
       </c>
-      <c r="C32" s="24" t="inlineStr">
+      <c r="C32" s="38" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D32" s="24" t="inlineStr">
+      <c r="D32" s="38" t="inlineStr">
         <is>
           <t>Servicios Profesionales</t>
         </is>
       </c>
-      <c r="E32" s="25" t="inlineStr">
+      <c r="E32" s="35" t="inlineStr">
         <is>
           <t>Profesionales Liberales Independientes</t>
         </is>
       </c>
-      <c r="F32" s="25" t="inlineStr">
+      <c r="F32" s="35" t="inlineStr">
         <is>
           <t>Facturación por Honorarios y Retenciones</t>
         </is>
       </c>
-      <c r="G32" s="26" t="n">
+      <c r="G32" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="H32" s="25" t="inlineStr">
+      <c r="H32" s="35" t="inlineStr">
         <is>
           <t>Profesionales &gt; Servicios Profesionales &gt; Facturación por Honorarios y Retenciones</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="19" t="n">
+      <c r="B33" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C33" s="37" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D33" s="20" t="inlineStr">
+      <c r="D33" s="37" t="inlineStr">
         <is>
           <t>Constitucionales</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
+      <c r="E33" s="33" t="inlineStr">
         <is>
           <t>Universidades, Colegios e Iglesias</t>
         </is>
       </c>
-      <c r="F33" s="21" t="inlineStr">
+      <c r="F33" s="33" t="inlineStr">
         <is>
           <t>Exenciones Tributarias de Rango Constitucional</t>
         </is>
       </c>
-      <c r="G33" s="22" t="n">
+      <c r="G33" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="H33" s="21" t="inlineStr">
+      <c r="H33" s="33" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Constitucionales &gt; Exenciones Tributarias de Rango Constitucional</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="23" t="n">
+      <c r="B34" s="17" t="n">
         <v>28</v>
       </c>
-      <c r="C34" s="24" t="inlineStr">
+      <c r="C34" s="38" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D34" s="24" t="inlineStr">
+      <c r="D34" s="38" t="inlineStr">
         <is>
           <t>No Lucrativos</t>
         </is>
       </c>
-      <c r="E34" s="25" t="inlineStr">
+      <c r="E34" s="35" t="inlineStr">
         <is>
           <t>ONGs, Fundaciones y Cooperativas</t>
         </is>
       </c>
-      <c r="F34" s="25" t="inlineStr">
+      <c r="F34" s="35" t="inlineStr">
         <is>
           <t>Reconocimiento de Exención de ISR e IVA</t>
         </is>
       </c>
-      <c r="G34" s="26" t="n">
+      <c r="G34" s="22" t="n">
         <v>14</v>
       </c>
-      <c r="H34" s="25" t="inlineStr">
+      <c r="H34" s="35" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; No Lucrativos &gt; Reconocimiento de Exención de ISR e IVA</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="19" t="n">
+      <c r="B35" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C35" s="37" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D35" s="37" t="inlineStr">
         <is>
           <t>Municipalidades</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E35" s="33" t="inlineStr">
         <is>
           <t>Gobiernos Locales y Empresas Municipales</t>
         </is>
       </c>
-      <c r="F35" s="21" t="inlineStr">
+      <c r="F35" s="33" t="inlineStr">
         <is>
           <t>Autonomía Municipal y Régimen Exento</t>
         </is>
       </c>
-      <c r="G35" s="22" t="n">
+      <c r="G35" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="H35" s="21" t="inlineStr">
+      <c r="H35" s="33" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Municipalidades &gt; Autonomía Municipal y Régimen Exento</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="23" t="n">
+      <c r="B36" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="C36" s="24" t="inlineStr">
+      <c r="C36" s="38" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D36" s="24" t="inlineStr">
+      <c r="D36" s="38" t="inlineStr">
         <is>
           <t>Entidades del Estado</t>
         </is>
       </c>
-      <c r="E36" s="25" t="inlineStr">
+      <c r="E36" s="35" t="inlineStr">
         <is>
           <t>Ministerios, Secretarías y Organismos del Estado</t>
         </is>
       </c>
-      <c r="F36" s="25" t="inlineStr">
+      <c r="F36" s="35" t="inlineStr">
         <is>
           <t>Compras Públicas y Agentes de Retención</t>
         </is>
       </c>
-      <c r="G36" s="26" t="n">
+      <c r="G36" s="22" t="n">
         <v>26</v>
       </c>
-      <c r="H36" s="25" t="inlineStr">
+      <c r="H36" s="35" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Entidades del Estado &gt; Compras Públicas y Agentes de Retención</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="19" t="n">
+      <c r="B37" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="C37" s="20" t="inlineStr">
+      <c r="C37" s="37" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D37" s="20" t="inlineStr">
+      <c r="D37" s="37" t="inlineStr">
         <is>
           <t>Decreto</t>
         </is>
       </c>
-      <c r="E37" s="21" t="inlineStr">
+      <c r="E37" s="33" t="inlineStr">
         <is>
           <t>Entidades con Incentivos Especiales</t>
         </is>
       </c>
-      <c r="F37" s="21" t="inlineStr">
+      <c r="F37" s="33" t="inlineStr">
         <is>
           <t>Exenciones y Fomento por Decreto Legislativo</t>
         </is>
       </c>
-      <c r="G37" s="22" t="n">
+      <c r="G37" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="H37" s="21" t="inlineStr">
+      <c r="H37" s="33" t="inlineStr">
         <is>
           <t>Entes Exentos &gt; Decreto &gt; Exenciones y Fomento por Decreto Legislativo</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="27" t="inlineStr"/>
-      <c r="C38" s="28" t="inlineStr">
+      <c r="B38" s="24" t="inlineStr"/>
+      <c r="C38" s="25" t="inlineStr">
         <is>
           <t>TOTAL DEL PORTAL</t>
         </is>
       </c>
-      <c r="D38" s="29" t="inlineStr">
+      <c r="D38" s="26" t="inlineStr">
         <is>
           <t>4 Segmentos y 31 Categorías Principales</t>
         </is>
       </c>
-      <c r="E38" s="27" t="inlineStr"/>
-      <c r="F38" s="27" t="inlineStr"/>
-      <c r="G38" s="30">
+      <c r="E38" s="24" t="inlineStr"/>
+      <c r="F38" s="24" t="inlineStr"/>
+      <c r="G38" s="27">
         <f>SUM(G7:G37)</f>
         <v/>
       </c>
-      <c r="H38" s="28" t="inlineStr">
+      <c r="H38" s="25" t="inlineStr">
         <is>
           <t>739 Trámites Oficiales Integrados</t>
         </is>
@@ -2132,1222 +2443,1222 @@
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Segmento (Nivel 1)</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Categoría / Rol (Nivel 2/3)</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Tema / Especialidad (Nivel 4)</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Qué es: (Definición Operativa de la Figura)</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Lead text: (Texto Orientador de Interfaz)</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Base jurídica: (Fundamento Legal Oficial: CAUCA, RECAUCA, Leyes)</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Trámites</t>
         </is>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>NIT sin Obligaciones</t>
         </is>
       </c>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="D7" s="33" t="inlineStr">
         <is>
           <t>RTU Digital y Solicitud de NIT</t>
         </is>
       </c>
-      <c r="E7" s="31" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Categoría destinada a personas individuales (estudiantes, personas en relación de dependencia sin renta afecta o ciudadanos en el extranjero) que requieren un Número de Identificación Tributaria únicamente para actos civiles, contractuales, bancarios o de registro público, sin realizar actividades mercantiles ni prestación de servicios técnicos afectos.</t>
         </is>
       </c>
-      <c r="F7" s="32" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Inscribe tu primer NIT en línea, actualiza tus datos de residencia y obtén tu constancia de solvencia fiscal sin necesidad de acudir a una agencia.</t>
         </is>
       </c>
-      <c r="G7" s="33" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>Código Tributario (Decreto 6-91, Arts. 112 y 120), Ley de Actualización Tributaria (Decreto 10-2012) y Acuerdo de Directorio SAT 08-2020.</t>
         </is>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="15" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="8" ht="50" customHeight="1">
-      <c r="A8" s="23" t="n">
+      <c r="A8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B8" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="38" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="35" t="inlineStr">
         <is>
           <t>Régimen de 5% y Facturación FEL</t>
         </is>
       </c>
-      <c r="E8" s="34" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>Régimen simplificado para personas individuales o jurídicas cuyas ventas de bienes o prestación de servicios no superan el monto de Q150,000 en el año calendario, tributando bajo una tarifa definitiva del 5% sobre ingresos brutos mensuales sin derecho a crédito fiscal.</t>
         </is>
       </c>
-      <c r="F8" s="35" t="inlineStr">
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>Emite tus facturas electrónicas FEL de pequeño contribuyente, declara mensualmente el 5% en Declaraguate y mantén tus libros al día.</t>
         </is>
       </c>
-      <c r="G8" s="36" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Ley del IVA (Decreto 27-92, Arts. 45 al 50) y Ley de Simplificación Tributaria (Decreto 7-2019, Régimen Electrónico de Pequeño Contribuyente).</t>
         </is>
       </c>
-      <c r="H8" s="26" t="n">
+      <c r="H8" s="22" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="9" ht="50" customHeight="1">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="37" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="33" t="inlineStr">
         <is>
           <t>Regímenes Especiales Decreto 31-2024 / 7-2019</t>
         </is>
       </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Regímenes tributarios especiales creados para productores, ganaderos y comercializadores del sector agropecuario, artesanal y primario que comercializan productos no transformados.</t>
         </is>
       </c>
-      <c r="F9" s="32" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Inscríbete en el régimen especial agropecuario, liquida tu Impuesto a la Confianza Tributaria y emite comprobantes oficiales simplificados.</t>
         </is>
       </c>
-      <c r="G9" s="33" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Ley de Simplificación Tributaria (Decreto 7-2019) y Ley para la Integración del Sector Productivo Primario y Agropecuario (Decreto 31-2024).</t>
         </is>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="15" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="10" ht="50" customHeight="1">
-      <c r="A10" s="23" t="n">
+      <c r="A10" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
       </c>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="D10" s="35" t="inlineStr">
         <is>
           <t>IVA General e Impuesto Sobre la Renta (ISR)</t>
         </is>
       </c>
-      <c r="E10" s="34" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>Régimen aplicable a personas individuales y sociedades mercantiles con ingresos superiores a Q150,000 o afiliados voluntariamente al Régimen General del IVA (12%) y regímenes del ISR (Opcional Simplificado 5%/7% o Sobre Utilidades de Actividades Lucrativas 25%).</t>
         </is>
       </c>
-      <c r="F10" s="35" t="inlineStr">
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>Declara y paga tu IVA mensual, liquida tus pagos trimestrales o retenciones de ISR, gestiona tu crédito fiscal y factura mediante FEL.</t>
         </is>
       </c>
-      <c r="G10" s="36" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Ley del IVA (Decreto 27-92), Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del Impuesto de Solidaridad (Decreto 73-2008).</t>
         </is>
       </c>
-      <c r="H10" s="26" t="n">
+      <c r="H10" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="50" customHeight="1">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="37" t="inlineStr">
         <is>
           <t>Asalariados</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="33" t="inlineStr">
         <is>
           <t>Retenciones de ISR y Planilla del IVA</t>
         </is>
       </c>
-      <c r="E11" s="31" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Régimen tributario de rentas del trabajo en relación de dependencia aplicable a trabajadores contratados por patronos públicos o privados que perciben ingresos salariales sujetos a retención del ISR.</t>
         </is>
       </c>
-      <c r="F11" s="32" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Consulta tus retenciones de ISR practicadas por tu patrono, ingresa tu planilla del IVA con facturas FEL y solicita devolución de retenciones en exceso.</t>
         </is>
       </c>
-      <c r="G11" s="33" t="inlineStr">
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>Ley de Actualización Tributaria (Decreto 10-2012, Arts. 68 al 82 - Rentas del Trabajo en Relación de Dependencia).</t>
         </is>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="H11" s="15" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="12" ht="50" customHeight="1">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
-      <c r="D12" s="25" t="inlineStr">
+      <c r="D12" s="35" t="inlineStr">
         <is>
           <t>Registro Fiscal de Vehículos (RFV)</t>
         </is>
       </c>
-      <c r="E12" s="34" t="inlineStr">
+      <c r="E12" s="19" t="inlineStr">
         <is>
           <t>Registro Fiscal de Vehículos (RFV) que administra el parque vehicular nacional, altas, bajas, modificaciones y el impuesto anual de circulación para propietarios y compradores de automotores terrestres, marítimos y aéreos.</t>
         </is>
       </c>
-      <c r="F12" s="35" t="inlineStr">
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>Paga tu calcomanía anual de circulación (ISCV), tramita primeras placas, realiza traspasos vehiculares y repón distintivos extraviados.</t>
         </is>
       </c>
-      <c r="G12" s="36" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Ley del Impuesto sobre Circulación de Vehículos Terrestres, Marítimos y Aéreos (Decreto 70-94) y Código Tributario (Decreto 6-91).</t>
         </is>
       </c>
-      <c r="H12" s="26" t="n">
+      <c r="H12" s="22" t="n">
         <v>72</v>
       </c>
     </row>
     <row r="13" ht="50" customHeight="1">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes Especiales</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="D13" s="33" t="inlineStr">
         <is>
           <t>Gerencias Especializadas de Fiscalización</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Segmento de control fiscal diferenciado conformado por grandes y medianos contribuyentes calificados por resolución de la SAT en función de su representatividad en la recaudación, facturación y relevancia sectorial.</t>
         </is>
       </c>
-      <c r="F13" s="32" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Gestiona tus obligaciones en agencias especializadas, presenta estados financieros auditados y cumple con estudios de precios de transferencia.</t>
         </is>
       </c>
-      <c r="G13" s="33" t="inlineStr">
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3) y Resoluciones de Directorio de Calificación de Contribuyentes Especiales.</t>
         </is>
       </c>
-      <c r="H13" s="22" t="n">
+      <c r="H13" s="15" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="14" ht="50" customHeight="1">
-      <c r="A14" s="23" t="n">
+      <c r="A14" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr">
         <is>
           <t>Facturación Electrónica</t>
         </is>
       </c>
-      <c r="D14" s="25" t="inlineStr">
+      <c r="D14" s="35" t="inlineStr">
         <is>
           <t>Sistema FEL y Agencia Virtual</t>
         </is>
       </c>
-      <c r="E14" s="34" t="inlineStr">
+      <c r="E14" s="19" t="inlineStr">
         <is>
           <t>Régimen obligatorio de emisión, transmisión y certificación de Documentos Tributarios Electrónicos (DTE) a través del sistema FEL y certificadores autorizados para todos los contribuyentes afiliados al régimen tributario nacional.</t>
         </is>
       </c>
-      <c r="F14" s="35" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>Habilítate como emisor de factura electrónica FEL, emite facturas gratuitas desde la Agencia Virtual y administra tus documentos emitidos y recibidos.</t>
         </is>
       </c>
-      <c r="G14" s="36" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Ley del IVA (Decreto 27-92, Arts. 29 y 29 "A") y Acuerdo de Directorio SAT 13-2018 (Régimen FEL).</t>
         </is>
       </c>
-      <c r="H14" s="26" t="n">
+      <c r="H14" s="22" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="15" ht="50" customHeight="1">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
+      <c r="C15" s="37" t="inlineStr">
         <is>
           <t>Servicios al Contribuyente</t>
         </is>
       </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="D15" s="33" t="inlineStr">
         <is>
           <t>Plataforma Digital, Citas y Solvencias</t>
         </is>
       </c>
-      <c r="E15" s="31" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Plataforma de servicios transversales de atención ciudadana, autenticación digital, expedición de solvencias fiscales, agendamiento de citas presenciales y consultas públicas en bases de datos de la SAT.</t>
         </is>
       </c>
-      <c r="F15" s="32" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Crea o desbloquea tu Agencia Virtual, genera tu solvencia fiscal con código QR, agenda citas presenciales y consulta el estado de tus gestiones.</t>
         </is>
       </c>
-      <c r="G15" s="33" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>Código Tributario (Decreto 6-91, Art. 57 "A" y Art. 120) y Acuerdos de Directorio de Servicios Electrónicos.</t>
         </is>
       </c>
-      <c r="H15" s="22" t="n">
+      <c r="H15" s="15" t="n">
         <v>67</v>
       </c>
     </row>
     <row r="16" ht="50" customHeight="1">
-      <c r="A16" s="23" t="n">
+      <c r="A16" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C16" s="38" t="inlineStr">
         <is>
           <t>Importadores y Exportadores (Compartido)</t>
         </is>
       </c>
-      <c r="D16" s="25" t="inlineStr">
+      <c r="D16" s="35" t="inlineStr">
         <is>
           <t>Gestiones Aduaneras Comunes y Arancel</t>
         </is>
       </c>
-      <c r="E16" s="34" t="inlineStr">
+      <c r="E16" s="19" t="inlineStr">
         <is>
           <t>Operadores comerciales que realizan indistintamente gestiones transversales de entrada y salida de mercancías, consultas arancelarias y pagos tributarios aduaneros en las aduanas de la República.</t>
         </is>
       </c>
-      <c r="F16" s="35" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>Consulta el Arancel Integrado Centroamericano (SAC), realiza pagos por BancaSAT y tramita solvencias aduaneras unificadas.</t>
         </is>
       </c>
-      <c r="G16" s="36" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Convenio sobre el Régimen Arancelario y Aduanero Centroamericano, CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA IV (Resolución 224-2008 COMIECO).</t>
         </is>
       </c>
-      <c r="H16" s="26" t="n">
+      <c r="H16" s="22" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="17" ht="50" customHeight="1">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="37" t="inlineStr">
         <is>
           <t>Importadores</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="33" t="inlineStr">
         <is>
           <t>Padrón de Importadores y DUCA-D</t>
         </is>
       </c>
-      <c r="E17" s="31" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Personas individuales o jurídicas autorizadas en el padrón aduanero de la SAT para introducir legalmente mercancías extranjeras al territorio aduanero nacional para su consumo, uso o transformación.</t>
         </is>
       </c>
-      <c r="F17" s="32" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Inscríbete en el padrón de importadores, liquida tus declaraciones aduaneras DUCA-D, consulta aranceles y rescata mercancías en aduana.</t>
         </is>
       </c>
-      <c r="G17" s="33" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Acuerdo Relativo a la Aplicación del Artículo VII del GATT (Valoración OMC).</t>
         </is>
       </c>
-      <c r="H17" s="22" t="n">
+      <c r="H17" s="15" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="18" ht="50" customHeight="1">
-      <c r="A18" s="23" t="n">
+      <c r="A18" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="24" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C18" s="24" t="inlineStr">
+      <c r="C18" s="38" t="inlineStr">
         <is>
           <t>Exportadores</t>
         </is>
       </c>
-      <c r="D18" s="25" t="inlineStr">
+      <c r="D18" s="35" t="inlineStr">
         <is>
           <t>Padrón de Exportadores y Devolución IVA</t>
         </is>
       </c>
-      <c r="E18" s="34" t="inlineStr">
+      <c r="E18" s="19" t="inlineStr">
         <is>
           <t>Personas individuales o jurídicas inscritas en el Registro de Exportadores de la SAT que despachan mercancías de origen nacional o nacionalizadas hacia mercados del exterior.</t>
         </is>
       </c>
-      <c r="F18" s="35" t="inlineStr">
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>Registra tus exportaciones con código VUPE, emite facturas con régimen especial y gestiona la devolución de crédito fiscal del IVA.</t>
         </is>
       </c>
-      <c r="G18" s="36" t="inlineStr">
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Ley de Fomento y Maquila (Decreto 29-89) y CAUCA/RECAUCA IV.</t>
         </is>
       </c>
-      <c r="H18" s="26" t="n">
+      <c r="H18" s="22" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="19" ht="50" customHeight="1">
-      <c r="A19" s="19" t="n">
+      <c r="A19" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C19" s="20" t="inlineStr">
+      <c r="C19" s="37" t="inlineStr">
         <is>
           <t>Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="33" t="inlineStr">
         <is>
           <t>Cadena Logística Segura y Carril Exprés</t>
         </is>
       </c>
-      <c r="E19" s="31" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Operadores de la cadena logística internacional certificados por la Intendencia de Aduanas por mantener rigurosos estándares de seguridad y confiabilidad en sus operaciones transfronterizas.</t>
         </is>
       </c>
-      <c r="F19" s="32" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>Accede a carriles exprés preferenciales, prioridad en contingencias y despacho ágil con selectivo rojo reducido.</t>
         </is>
       </c>
-      <c r="G19" s="33" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio de la SAT sobre el Programa OEA-Guatemala.</t>
         </is>
       </c>
-      <c r="H19" s="22" t="n">
+      <c r="H19" s="15" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="20" ht="50" customHeight="1">
-      <c r="A20" s="23" t="n">
+      <c r="A20" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C20" s="24" t="inlineStr">
+      <c r="C20" s="38" t="inlineStr">
         <is>
           <t>Agentes Aduaneros</t>
         </is>
       </c>
-      <c r="D20" s="25" t="inlineStr">
+      <c r="D20" s="35" t="inlineStr">
         <is>
           <t>Despacho Aduanero Oficial y Representación</t>
         </is>
       </c>
-      <c r="E20" s="34" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>Profesionales auxiliares de la función pública aduanera autorizados para actuar por cuenta de terceros en los trámites y operaciones de desaduanamiento ante la SAT.</t>
         </is>
       </c>
-      <c r="F20" s="35" t="inlineStr">
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>Gestiona tu carné y habilitación oficial, presenta pólizas de seguro de caución y transmite declaraciones con firma electrónica.</t>
         </is>
       </c>
-      <c r="G20" s="36" t="inlineStr">
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>CAUCA IV (Arts. 22 al 28), RECAUCA IV (Arts. 74 al 85) y Ley Nacional de Aduanas.</t>
         </is>
       </c>
-      <c r="H20" s="26" t="n">
+      <c r="H20" s="22" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="21" ht="50" customHeight="1">
-      <c r="A21" s="19" t="n">
+      <c r="A21" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="20" t="inlineStr">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C21" s="20" t="inlineStr">
+      <c r="C21" s="37" t="inlineStr">
         <is>
           <t>Apoderados Especiales Aduaneros</t>
         </is>
       </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="D21" s="33" t="inlineStr">
         <is>
           <t>Despacho Aduanero por Cuenta Propia</t>
         </is>
       </c>
-      <c r="E21" s="31" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Personas individuales mandatarias designadas exclusivamente por una persona jurídica para representarla formalmente en sus despachos aduaneros propios.</t>
         </is>
       </c>
-      <c r="F21" s="32" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>Registra tu mandato legal, actualiza tu carné de apoderado y tramita declaraciones DUCA corporativas.</t>
         </is>
       </c>
-      <c r="G21" s="33" t="inlineStr">
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>CAUCA IV (Art. 21), RECAUCA IV (Arts. 86 al 90) y Código de Notariado.</t>
         </is>
       </c>
-      <c r="H21" s="22" t="n">
+      <c r="H21" s="15" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="22" ht="50" customHeight="1">
-      <c r="A22" s="23" t="n">
+      <c r="A22" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C22" s="24" t="inlineStr">
+      <c r="C22" s="38" t="inlineStr">
         <is>
           <t>Empresas de Entrega Rápida o Courier</t>
         </is>
       </c>
-      <c r="D22" s="25" t="inlineStr">
+      <c r="D22" s="35" t="inlineStr">
         <is>
           <t>Paquetería Internacional y Franquicias</t>
         </is>
       </c>
-      <c r="E22" s="34" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>Empresas de mensajería y paquetería urgente autorizadas para transportar y desaduanar envíos postales exprés y encomiendas internacionales no comerciales.</t>
         </is>
       </c>
-      <c r="F22" s="35" t="inlineStr">
+      <c r="F22" s="20" t="inlineStr">
         <is>
           <t>Transmite manifiestos courier, aplica franquicias simplificadas y habilita recintos desconsolidadores de paquetería.</t>
         </is>
       </c>
-      <c r="G22" s="36" t="inlineStr">
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>CAUCA IV y RECAUCA IV (Arts. 574 al 596 - Régimen de Envíos de Entrega Rápida o Courier).</t>
         </is>
       </c>
-      <c r="H22" s="26" t="n">
+      <c r="H22" s="22" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="23" ht="50" customHeight="1">
-      <c r="A23" s="19" t="n">
+      <c r="A23" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C23" s="20" t="inlineStr">
+      <c r="C23" s="37" t="inlineStr">
         <is>
           <t>Consolidadores y Desconsolidadores de Carga</t>
         </is>
       </c>
-      <c r="D23" s="21" t="inlineStr">
+      <c r="D23" s="33" t="inlineStr">
         <is>
           <t>Manifiestos CUSCAR y Guías Hijas</t>
         </is>
       </c>
-      <c r="E23" s="31" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Operadores logísticos autorizados para agrupar o separar mercancías pertenecientes a distintos consignatarios bajo un solo documento matriz de transporte.</t>
         </is>
       </c>
-      <c r="F23" s="32" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Transmite manifiestos CUSCAR, emite guías hijas y reporta inconsistencias o averías de carga ante la aduana.</t>
         </is>
       </c>
-      <c r="G23" s="33" t="inlineStr">
+      <c r="G23" s="14" t="inlineStr">
         <is>
           <t>CAUCA IV y RECAUCA IV (Arts. 102 al 109 - Auxiliares Consolidador y Desconsolidador de Carga).</t>
         </is>
       </c>
-      <c r="H23" s="22" t="n">
+      <c r="H23" s="15" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="24" ht="50" customHeight="1">
-      <c r="A24" s="23" t="n">
+      <c r="A24" s="17" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C24" s="24" t="inlineStr">
+      <c r="C24" s="38" t="inlineStr">
         <is>
           <t>Transportistas Aduaneros</t>
         </is>
       </c>
-      <c r="D24" s="25" t="inlineStr">
+      <c r="D24" s="35" t="inlineStr">
         <is>
           <t>Tránsito Aduanero Internacional y Marchamo</t>
         </is>
       </c>
-      <c r="E24" s="34" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>Empresas y conductores autorizados para realizar el traslado de mercancías bajo control aduanero dentro del territorio nacional o en tránsito internacional centroamericano.</t>
         </is>
       </c>
-      <c r="F24" s="35" t="inlineStr">
+      <c r="F24" s="20" t="inlineStr">
         <is>
           <t>Registra medios de transporte, activa marchamos electrónicos RFID y transmite declaraciones de tránsito DUCA-T.</t>
         </is>
       </c>
-      <c r="G24" s="36" t="inlineStr">
+      <c r="G24" s="21" t="inlineStr">
         <is>
           <t>CAUCA IV (Arts. 18 al 20), RECAUCA IV (Tránsito Aduanero Internacional Terrestre) y Reglamentos de Transporte Centroamericano.</t>
         </is>
       </c>
-      <c r="H24" s="26" t="n">
+      <c r="H24" s="22" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="25" ht="50" customHeight="1">
-      <c r="A25" s="19" t="n">
+      <c r="A25" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="B25" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C25" s="20" t="inlineStr">
+      <c r="C25" s="37" t="inlineStr">
         <is>
           <t>Depósitos Aduaneros</t>
         </is>
       </c>
-      <c r="D25" s="21" t="inlineStr">
+      <c r="D25" s="33" t="inlineStr">
         <is>
           <t>Custodia de Mercancías y Títulos de Crédito</t>
         </is>
       </c>
-      <c r="E25" s="31" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Recintos públicos o privados (Almacenes Fiscales, Almacenes Generales de Depósito y Depósitos Aduaneros Temporales DAT) autorizados para custodiar mercancías con suspensión de tributos aduaneros.</t>
         </is>
       </c>
-      <c r="F25" s="32" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>Controla inventarios de custodia, gestiona actas de recepción, emite certificados de depósito (AGD) y tramita prórrogas de permanencia.</t>
         </is>
       </c>
-      <c r="G25" s="33" t="inlineStr">
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>Decreto 1236 (Ley de Almacenes Generales de Depósito), CAUCA IV y RECAUCA IV (Arts. 119 al 129 - Régimen de Depósito Aduanero).</t>
         </is>
       </c>
-      <c r="H25" s="22" t="n">
+      <c r="H25" s="15" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="26" ht="50" customHeight="1">
-      <c r="A26" s="23" t="n">
+      <c r="A26" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C26" s="24" t="inlineStr">
+      <c r="C26" s="38" t="inlineStr">
         <is>
           <t>ZDEEP - Entidades Administradoras</t>
         </is>
       </c>
-      <c r="D26" s="25" t="inlineStr">
+      <c r="D26" s="35" t="inlineStr">
         <is>
           <t>Administración de Zonas Especiales Públicas</t>
         </is>
       </c>
-      <c r="E26" s="34" t="inlineStr">
+      <c r="E26" s="19" t="inlineStr">
         <is>
           <t>Personas jurídicas públicas o privadas autorizadas por ZOLIC y SAT para desarrollar, operar y vigilar la infraestructura de polígonos industriales y logísticos ZDEEP.</t>
         </is>
       </c>
-      <c r="F26" s="35" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>Delimita polígonos aduaneros, administra garitas de control y supervisa el perímetro de seguridad de la zona especial.</t>
         </is>
       </c>
-      <c r="G26" s="36" t="inlineStr">
+      <c r="G26" s="21" t="inlineStr">
         <is>
           <t>Decreto 22-73 (Ley Orgánica de ZOLIC reformada), CAUCA IV, RECAUCA IV y Resoluciones Conjuntas SAT-ZOLIC.</t>
         </is>
       </c>
-      <c r="H26" s="26" t="n">
+      <c r="H26" s="22" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="27" ht="50" customHeight="1">
-      <c r="A27" s="19" t="n">
+      <c r="A27" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B27" s="20" t="inlineStr">
+      <c r="B27" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C27" s="20" t="inlineStr">
+      <c r="C27" s="37" t="inlineStr">
         <is>
           <t>ZDEEP - Empresas Usuarias</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D27" s="33" t="inlineStr">
         <is>
           <t>Transformación, Servicios y Exenciones</t>
         </is>
       </c>
-      <c r="E27" s="31" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Empresas industriales, comerciales o de servicios instaladas y operando dentro de los recintos calificados como ZDEEP para producir o transformar con beneficios fiscales.</t>
         </is>
       </c>
-      <c r="F27" s="32" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Ingresa materias primas con suspensión de DAI e IVA, realiza descargos de producción y goza de exenciones tributarias.</t>
         </is>
       </c>
-      <c r="G27" s="33" t="inlineStr">
+      <c r="G27" s="14" t="inlineStr">
         <is>
           <t>Decreto 22-73 (Régimen Fiscal ZDEEP), Ley de Actualización Tributaria (Decreto 10-2012) y CAUCA/RECAUCA IV.</t>
         </is>
       </c>
-      <c r="H27" s="22" t="n">
+      <c r="H27" s="15" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="28" ht="50" customHeight="1">
-      <c r="A28" s="23" t="n">
+      <c r="A28" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C28" s="24" t="inlineStr">
+      <c r="C28" s="38" t="inlineStr">
         <is>
           <t>Abogados y Notarios</t>
         </is>
       </c>
-      <c r="D28" s="25" t="inlineStr">
+      <c r="D28" s="35" t="inlineStr">
         <is>
           <t>Papel Sellado de Protocolo y Avisos</t>
         </is>
       </c>
-      <c r="E28" s="34" t="inlineStr">
+      <c r="E28" s="19" t="inlineStr">
         <is>
           <t>Profesionales del derecho colegiados activos autorizados para ejercer la fe pública notarial, redactar instrumentos públicos y autorizar traspasos electrónicos de vehículos ante la SAT.</t>
         </is>
       </c>
-      <c r="F28" s="35" t="inlineStr">
+      <c r="F28" s="20" t="inlineStr">
         <is>
           <t>Compra papel sellado especial para protocolos, adquiere timbres fiscales, realiza traspasos vehiculares electrónicos (TEV) y presenta avisos notariales.</t>
         </is>
       </c>
-      <c r="G28" s="36" t="inlineStr">
+      <c r="G28" s="21" t="inlineStr">
         <is>
           <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales y de Papel Sellado Especial para Protocolos (Decreto 37-92) y Código Tributario.</t>
         </is>
       </c>
-      <c r="H28" s="26" t="n">
+      <c r="H28" s="22" t="n">
         <v>17</v>
       </c>
     </row>
     <row r="29" ht="50" customHeight="1">
-      <c r="A29" s="19" t="n">
+      <c r="A29" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B29" s="37" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C29" s="20" t="inlineStr">
+      <c r="C29" s="37" t="inlineStr">
         <is>
           <t>Peritos Contadores</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="33" t="inlineStr">
         <is>
           <t>Libros Contables y Declaraciones</t>
         </is>
       </c>
-      <c r="E29" s="31" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Técnicos y profesionales contables inscritos y autorizados ante la SAT para llevar y firmar registros contables de contribuyentes, certificar estados financieros y realizar gestiones tributarias.</t>
         </is>
       </c>
-      <c r="F29" s="32" t="inlineStr">
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Inscríbete y actualiza tus datos en el Registro de Contadores, autoriza libros contables computarizados y asocia contribuyentes a tu perfil.</t>
         </is>
       </c>
-      <c r="G29" s="33" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Decreto 2450 (Normas que Regulan el Ejercicio de la Profesión de Contador), Código de Comercio (Decreto 2-70) y Código Tributario (Arts. 112 y 120).</t>
         </is>
       </c>
-      <c r="H29" s="22" t="n">
+      <c r="H29" s="15" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="30" ht="50" customHeight="1">
-      <c r="A30" s="23" t="n">
+      <c r="A30" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="38" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C30" s="24" t="inlineStr">
+      <c r="C30" s="38" t="inlineStr">
         <is>
           <t>Auditores</t>
         </is>
       </c>
-      <c r="D30" s="25" t="inlineStr">
+      <c r="D30" s="35" t="inlineStr">
         <is>
           <t>Dictámenes Tributarios y Devolución IVA</t>
         </is>
       </c>
-      <c r="E30" s="34" t="inlineStr">
+      <c r="E30" s="19" t="inlineStr">
         <is>
           <t>Contadores Públicos y Auditores (CPA) colegiados activos y firmas de auditoría facultados para emitir dictámenes sobre estados financieros, devolución de crédito fiscal e informes de precios de transferencia.</t>
         </is>
       </c>
-      <c r="F30" s="35" t="inlineStr">
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>Emite dictámenes de crédito fiscal para exportadores, dictámenes de estados financieros para licitaciones y presenta informes tributarios requeridos por SAT.</t>
         </is>
       </c>
-      <c r="G30" s="36" t="inlineStr">
+      <c r="G30" s="21" t="inlineStr">
         <is>
           <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001), Ley del IVA (Decreto 27-92, Art. 23 bis) y Ley de Actualización Tributaria (Decreto 10-2012).</t>
         </is>
       </c>
-      <c r="H30" s="26" t="n">
+      <c r="H30" s="22" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="31" ht="50" customHeight="1">
-      <c r="A31" s="19" t="n">
+      <c r="A31" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="37" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C31" s="37" t="inlineStr">
         <is>
           <t>Gestores Tributarios</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="D31" s="33" t="inlineStr">
         <is>
           <t>Gafetes y Trámites Presenciales</t>
         </is>
       </c>
-      <c r="E31" s="31" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Personas individuales autorizadas y acreditadas formalmente ante la SAT para representar a terceros en la tramitación presencial de gestiones administrativas tributarias y aduaneras.</t>
         </is>
       </c>
-      <c r="F31" s="32" t="inlineStr">
+      <c r="F31" s="13" t="inlineStr">
         <is>
           <t>Tramita y renueva tu carné oficial de gestor tributario, registra tus datos biométricos y gestiona expedientes autorizados en agencias tributarias.</t>
         </is>
       </c>
-      <c r="G31" s="33" t="inlineStr">
+      <c r="G31" s="14" t="inlineStr">
         <is>
           <t>Acuerdos de Directorio de la SAT sobre Regulación y Acreditación de Gestores Tributarios y Código Tributario.</t>
         </is>
       </c>
-      <c r="H31" s="22" t="n">
+      <c r="H31" s="15" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="32" ht="50" customHeight="1">
-      <c r="A32" s="23" t="n">
+      <c r="A32" s="17" t="n">
         <v>26</v>
       </c>
-      <c r="B32" s="24" t="inlineStr">
+      <c r="B32" s="38" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C32" s="24" t="inlineStr">
+      <c r="C32" s="38" t="inlineStr">
         <is>
           <t>Servicios Profesionales</t>
         </is>
       </c>
-      <c r="D32" s="25" t="inlineStr">
+      <c r="D32" s="35" t="inlineStr">
         <is>
           <t>Facturación por Honorarios y Retenciones</t>
         </is>
       </c>
-      <c r="E32" s="34" t="inlineStr">
+      <c r="E32" s="19" t="inlineStr">
         <is>
           <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de consultoría por honorarios profesionales.</t>
         </is>
       </c>
-      <c r="F32" s="35" t="inlineStr">
+      <c r="F32" s="20" t="inlineStr">
         <is>
           <t>Emite facturas electrónicas FEL por honorarios, liquida retenciones de ISR, actualiza tu colegiado activo y consulta tu solvencia fiscal.</t>
         </is>
       </c>
-      <c r="G32" s="36" t="inlineStr">
+      <c r="G32" s="21" t="inlineStr">
         <is>
           <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del IVA (Decreto 27-92).</t>
         </is>
       </c>
-      <c r="H32" s="26" t="n">
+      <c r="H32" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="33" ht="50" customHeight="1">
-      <c r="A33" s="19" t="n">
+      <c r="A33" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="B33" s="20" t="inlineStr">
+      <c r="B33" s="37" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C33" s="37" t="inlineStr">
         <is>
           <t>Constitucionales</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D33" s="33" t="inlineStr">
         <is>
           <t>Exenciones Tributarias de Rango Constitucional</t>
         </is>
       </c>
-      <c r="E33" s="31" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Instituciones educativas, universidades, comunidades religiosas, misiones diplomáticas y cuerpos consulares que gozan de exención de impuestos por mandato directo de la Carta Magna.</t>
         </is>
       </c>
-      <c r="F33" s="32" t="inlineStr">
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>Inscribe tu personería jurídica exenta en el RTU, emite constancias electrónicas de exención de IVA y timbres, y acredita representación legal.</t>
         </is>
       </c>
-      <c r="G33" s="33" t="inlineStr">
+      <c r="G33" s="14" t="inlineStr">
         <is>
           <t>Constitución Política de la República de Guatemala (Arts. 37, 73, 88), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
         </is>
       </c>
-      <c r="H33" s="22" t="n">
+      <c r="H33" s="15" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="34" ht="50" customHeight="1">
-      <c r="A34" s="23" t="n">
+      <c r="A34" s="17" t="n">
         <v>28</v>
       </c>
-      <c r="B34" s="24" t="inlineStr">
+      <c r="B34" s="38" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C34" s="24" t="inlineStr">
+      <c r="C34" s="38" t="inlineStr">
         <is>
           <t>No Lucrativos</t>
         </is>
       </c>
-      <c r="D34" s="25" t="inlineStr">
+      <c r="D34" s="35" t="inlineStr">
         <is>
           <t>Reconocimiento de Exención de ISR e IVA</t>
         </is>
       </c>
-      <c r="E34" s="34" t="inlineStr">
+      <c r="E34" s="19" t="inlineStr">
         <is>
           <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas, asociaciones civiles sin fines de lucro y cooperativas que solicitan reconocimiento administrativo de exención de ISR e IVA.</t>
         </is>
       </c>
-      <c r="F34" s="35" t="inlineStr">
+      <c r="F34" s="20" t="inlineStr">
         <is>
           <t>Solicita tu resolución formal de exención de ISR, actualiza estatutos y junta directiva en el RTU y emite constancias de retención y exención.</t>
         </is>
       </c>
-      <c r="G34" s="36" t="inlineStr">
+      <c r="G34" s="21" t="inlineStr">
         <is>
           <t>Decreto 02-2003 (Ley de ONGs para el Desarrollo), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
         </is>
       </c>
-      <c r="H34" s="26" t="n">
+      <c r="H34" s="22" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="35" ht="50" customHeight="1">
-      <c r="A35" s="19" t="n">
+      <c r="A35" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="B35" s="37" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C35" s="37" t="inlineStr">
         <is>
           <t>Municipalidades</t>
         </is>
       </c>
-      <c r="D35" s="21" t="inlineStr">
+      <c r="D35" s="33" t="inlineStr">
         <is>
           <t>Autonomía Municipal y Régimen Exento</t>
         </is>
       </c>
-      <c r="E35" s="31" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Las 340 corporaciones municipales autónomas de la República de Guatemala, mancomunidades y empresas municipales públicas prestadoras de servicios comunitarios.</t>
         </is>
       </c>
-      <c r="F35" s="32" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>Registra autoridades y tesoreros en el RTU, gestiona la exención del impuesto de circulación para flotillas municipales y tramita solvencias institucionales.</t>
         </is>
       </c>
-      <c r="G35" s="33" t="inlineStr">
+      <c r="G35" s="14" t="inlineStr">
         <is>
           <t>Constitución Política de la República (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
         </is>
       </c>
-      <c r="H35" s="22" t="n">
+      <c r="H35" s="15" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="36" ht="50" customHeight="1">
-      <c r="A36" s="23" t="n">
+      <c r="A36" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="B36" s="24" t="inlineStr">
+      <c r="B36" s="38" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C36" s="24" t="inlineStr">
+      <c r="C36" s="38" t="inlineStr">
         <is>
           <t>Entidades del Estado</t>
         </is>
       </c>
-      <c r="D36" s="25" t="inlineStr">
+      <c r="D36" s="35" t="inlineStr">
         <is>
           <t>Compras Públicas y Agentes de Retención</t>
         </is>
       </c>
-      <c r="E36" s="34" t="inlineStr">
+      <c r="E36" s="19" t="inlineStr">
         <is>
           <t>Ministerios de Estado, secretarías, organismos de los poderes Ejecutivo, Legislativo y Judicial, y entidades públicas descentralizadas que operan como agentes de retención del IVA e ISR.</t>
         </is>
       </c>
-      <c r="F36" s="35" t="inlineStr">
+      <c r="F36" s="20" t="inlineStr">
         <is>
           <t>Habilita unidades ejecutoras en el RTU, emite constancias de retención en compras públicas y administra el parque vehicular oficial del Estado.</t>
         </is>
       </c>
-      <c r="G36" s="36" t="inlineStr">
+      <c r="G36" s="21" t="inlineStr">
         <is>
           <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
         </is>
       </c>
-      <c r="H36" s="26" t="n">
+      <c r="H36" s="22" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="37" ht="50" customHeight="1">
-      <c r="A37" s="19" t="n">
+      <c r="A37" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="B37" s="37" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C37" s="20" t="inlineStr">
+      <c r="C37" s="37" t="inlineStr">
         <is>
           <t>Decreto</t>
         </is>
       </c>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="D37" s="33" t="inlineStr">
         <is>
           <t>Exenciones y Fomento por Decreto Legislativo</t>
         </is>
       </c>
-      <c r="E37" s="31" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Personas o entidades beneficiarias de leyes de fomento económico y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso.</t>
         </is>
       </c>
-      <c r="F37" s="32" t="inlineStr">
+      <c r="F37" s="13" t="inlineStr">
         <is>
           <t>Acredita resoluciones ministeriales de calificación de fomento, gestiona exenciones arancelarias temporales y presenta reportes periódicos de cumplimiento.</t>
         </is>
       </c>
-      <c r="G37" s="33" t="inlineStr">
+      <c r="G37" s="14" t="inlineStr">
         <is>
           <t>Decretos específicos de fomento (Decreto 29-89 de Maquilas, Decreto 65-89 de Zonas Francas, Ley de Incentivos para Energías Renovables) y Código Tributario.</t>
         </is>
       </c>
-      <c r="H37" s="22" t="n">
+      <c r="H37" s="15" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(arquitectura): reconstruir hoja Mapa de Navegacion con 33 categorias canonicas, subtotales por segmento y 100% cobertura (739 tramites)
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas por Rol y Categoría" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fichas por Rol y Categoría'!$A$6:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fichas por Rol y Categoría'!$A$6:$H$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,8 +89,14 @@
       <color rgb="00475569"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -145,8 +151,14 @@
         <bgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -226,11 +238,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0064748B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -325,7 +351,36 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1288,16 +1343,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H38"/>
+  <dimension ref="B2:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1311,7 +1368,7 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>MAPA ESTRUCTURAL DE NAVEGACIÓN DEL PORTAL WEB (ARQUITECTURA DE INFORMACIÓN CENTRADA EN EL CIUDADANO)</t>
+          <t>MAPA ESTRUCTURAL DE NAVEGACIÓN DEL PORTAL WEB — TAXONOMÍA CANÓNICA (N1 A N3) Y CONTEO OFICIAL DE COBERTURA</t>
         </is>
       </c>
     </row>
@@ -1328,31 +1385,41 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Nivel 2: Categoría / Área</t>
+          <t>Nivel 2: Régimen / Área</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Nivel 3: Grupo / Actor Específico</t>
+          <t>Nivel 3: Categoría / Actor</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Nivel 4: Tema / Especialidad</t>
+          <t>Alcance y Especialidad de Navegación</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Trámites Contenidos</t>
+          <t>Trámites</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Ruta de Navegación de Entrada (Miga de Pan)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
+          <t>% Segmento</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>% Portal</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Ruta Canónica de Navegación (Miga de Pan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
       <c r="B7" s="10" t="n">
         <v>1</v>
       </c>
@@ -1368,57 +1435,73 @@
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>Personas Individuales</t>
-        </is>
-      </c>
-      <c r="F7" s="33" t="inlineStr">
-        <is>
-          <t>RTU Digital y Solicitud de NIT</t>
+          <t>NIT sin Obligaciones</t>
+        </is>
+      </c>
+      <c r="F7" s="38" t="inlineStr">
+        <is>
+          <t>Inscripción de primer NIT, actualización de datos de residencia y solvencia fiscal para personas sin actividad mercantil.</t>
         </is>
       </c>
       <c r="G7" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="H7" s="33" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; NIT sin Obligaciones &gt; RTU Digital y Solicitud de NIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
+      <c r="H7" s="39">
+        <f>G7/$G$18</f>
+        <v/>
+      </c>
+      <c r="I7" s="39">
+        <f>G7/$G$44</f>
+        <v/>
+      </c>
+      <c r="J7" s="38" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; NIT sin Obligaciones &gt; NIT sin Obligaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
       <c r="B8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="38" t="inlineStr">
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D8" s="38" t="inlineStr">
+      <c r="D8" s="40" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
       <c r="E8" s="35" t="inlineStr">
         <is>
-          <t>Pequeño Contribuyente General</t>
-        </is>
-      </c>
-      <c r="F8" s="35" t="inlineStr">
-        <is>
-          <t>Régimen de 5% y Facturación FEL</t>
+          <t>Pequeños Contribuyentes</t>
+        </is>
+      </c>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>Régimen del 5% definitivo, facturación FEL, régimen electrónico y regímenes especiales del sector primario y agropecuario.</t>
         </is>
       </c>
       <c r="G8" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="H8" s="35" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Régimen de 5% y Facturación FEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
+      <c r="H8" s="42">
+        <f>G8/$G$18</f>
+        <v/>
+      </c>
+      <c r="I8" s="42">
+        <f>G8/$G$44</f>
+        <v/>
+      </c>
+      <c r="J8" s="41" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Pequeños Contribuyentes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
       <c r="B9" s="10" t="n">
         <v>3</v>
       </c>
@@ -1429,62 +1512,78 @@
       </c>
       <c r="D9" s="37" t="inlineStr">
         <is>
-          <t>Pequeños Contribuyentes</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="E9" s="33" t="inlineStr">
         <is>
-          <t>Sector Primario y Agropecuario</t>
-        </is>
-      </c>
-      <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>Regímenes Especiales Decreto 31-2024 / 7-2019</t>
+          <t>Declaraciones y Pagos</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
+          <t>Declaración y pago de IVA General, pagos trimestrales o mensuales de ISR, liquidación de ISO y formularios electrónicos.</t>
         </is>
       </c>
       <c r="G9" s="15" t="n">
-        <v>22</v>
-      </c>
-      <c r="H9" s="33" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Regímenes Especiales Decreto 31-2024 / 7-2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
+        <v>87</v>
+      </c>
+      <c r="H9" s="39">
+        <f>G9/$G$18</f>
+        <v/>
+      </c>
+      <c r="I9" s="39">
+        <f>G9/$G$44</f>
+        <v/>
+      </c>
+      <c r="J9" s="38" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; Declaraciones y Pagos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
       <c r="B10" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="38" t="inlineStr">
+      <c r="C10" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D10" s="38" t="inlineStr">
+      <c r="D10" s="40" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
       </c>
       <c r="E10" s="35" t="inlineStr">
         <is>
-          <t>Personas y Empresas en Régimen General</t>
-        </is>
-      </c>
-      <c r="F10" s="35" t="inlineStr">
-        <is>
-          <t>IVA General e Impuesto Sobre la Renta (ISR)</t>
+          <t>RTU Digital y Agencia Virtual</t>
+        </is>
+      </c>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>Inscripción y actualización periódica en el RTU, modificación de domicilios, altas de establecimientos y gestión de usuarios.</t>
         </is>
       </c>
       <c r="G10" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="35" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Contribuyente General &gt; IVA General e Impuesto Sobre la Renta (ISR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
+        <v>78</v>
+      </c>
+      <c r="H10" s="42">
+        <f>G10/$G$18</f>
+        <v/>
+      </c>
+      <c r="I10" s="42">
+        <f>G10/$G$44</f>
+        <v/>
+      </c>
+      <c r="J10" s="41" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; RTU Digital y Agencia Virtual</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
       <c r="B11" s="10" t="n">
         <v>5</v>
       </c>
@@ -1495,62 +1594,78 @@
       </c>
       <c r="D11" s="37" t="inlineStr">
         <is>
-          <t>Asalariados</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="E11" s="33" t="inlineStr">
         <is>
-          <t>Trabajadores en Relación de Dependencia</t>
-        </is>
-      </c>
-      <c r="F11" s="33" t="inlineStr">
-        <is>
-          <t>Retenciones de ISR y Planilla del IVA</t>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>Registro Fiscal de Vehículos (RFV), calcomanía anual ISCV, primeras placas, traspasos y reposición de distintivos.</t>
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="H11" s="33" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Asalariados &gt; Retenciones de ISR y Planilla del IVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
+        <v>72</v>
+      </c>
+      <c r="H11" s="39">
+        <f>G11/$G$18</f>
+        <v/>
+      </c>
+      <c r="I11" s="39">
+        <f>G11/$G$44</f>
+        <v/>
+      </c>
+      <c r="J11" s="38" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; Vehículos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
       <c r="B12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="C12" s="38" t="inlineStr">
+      <c r="C12" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D12" s="38" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="D12" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="E12" s="35" t="inlineStr">
         <is>
-          <t>Propietarios y Compradores de Vehículos</t>
-        </is>
-      </c>
-      <c r="F12" s="35" t="inlineStr">
-        <is>
-          <t>Registro Fiscal de Vehículos (RFV)</t>
+          <t>Servicios al Contribuyente</t>
+        </is>
+      </c>
+      <c r="F12" s="41" t="inlineStr">
+        <is>
+          <t>Agendamiento de citas presenciales, solvencia fiscal con código QR, consultas públicas y asistencia tributaria.</t>
         </is>
       </c>
       <c r="G12" s="22" t="n">
-        <v>72</v>
-      </c>
-      <c r="H12" s="35" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Vehículos &gt; Registro Fiscal de Vehículos (RFV)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
+        <v>67</v>
+      </c>
+      <c r="H12" s="42">
+        <f>G12/$G$18</f>
+        <v/>
+      </c>
+      <c r="I12" s="42">
+        <f>G12/$G$44</f>
+        <v/>
+      </c>
+      <c r="J12" s="41" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; Servicios al Contribuyente</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
       <c r="B13" s="10" t="n">
         <v>7</v>
       </c>
@@ -1561,62 +1676,78 @@
       </c>
       <c r="D13" s="37" t="inlineStr">
         <is>
-          <t>Contribuyentes Especiales</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="E13" s="33" t="inlineStr">
         <is>
-          <t>Grandes y Medianos Contribuyentes</t>
-        </is>
-      </c>
-      <c r="F13" s="33" t="inlineStr">
-        <is>
-          <t>Gerencias Especializadas de Fiscalización</t>
+          <t>Empresas y Sociedades</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>Inscripción y cese de sociedades mercantiles, habilitación de sucursales, nombramiento de representantes legales y personerías.</t>
         </is>
       </c>
       <c r="G13" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="H13" s="33" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Contribuyentes Especiales &gt; Gerencias Especializadas de Fiscalización</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
+        <v>32</v>
+      </c>
+      <c r="H13" s="39">
+        <f>G13/$G$18</f>
+        <v/>
+      </c>
+      <c r="I13" s="39">
+        <f>G13/$G$44</f>
+        <v/>
+      </c>
+      <c r="J13" s="38" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; Empresas y Sociedades</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
       <c r="B14" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="C14" s="38" t="inlineStr">
+      <c r="C14" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D14" s="38" t="inlineStr">
+      <c r="D14" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyente General</t>
+        </is>
+      </c>
+      <c r="E14" s="35" t="inlineStr">
         <is>
           <t>Facturación Electrónica</t>
         </is>
       </c>
-      <c r="E14" s="35" t="inlineStr">
-        <is>
-          <t>Emisores de DTE</t>
-        </is>
-      </c>
-      <c r="F14" s="35" t="inlineStr">
-        <is>
-          <t>Sistema FEL y Agencia Virtual</t>
+      <c r="F14" s="41" t="inlineStr">
+        <is>
+          <t>Habilitación como emisor FEL, emisión de facturas y notas de crédito en Agencia Virtual, y anulación de DTE.</t>
         </is>
       </c>
       <c r="G14" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H14" s="35" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Facturación Electrónica &gt; Sistema FEL y Agencia Virtual</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
+      <c r="H14" s="42">
+        <f>G14/$G$18</f>
+        <v/>
+      </c>
+      <c r="I14" s="42">
+        <f>G14/$G$44</f>
+        <v/>
+      </c>
+      <c r="J14" s="41" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; Facturación Electrónica</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
       <c r="B15" s="10" t="n">
         <v>9</v>
       </c>
@@ -1627,782 +1758,1194 @@
       </c>
       <c r="D15" s="37" t="inlineStr">
         <is>
-          <t>Servicios al Contribuyente</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr">
         <is>
-          <t>Ciudadanía y Usuarios de Agencia Virtual</t>
-        </is>
-      </c>
-      <c r="F15" s="33" t="inlineStr">
-        <is>
-          <t>Plataforma Digital, Citas y Solvencias</t>
+          <t>Solvencia y Convenios</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>Suscripción de convenios de pago en cuotas, facilidades crediticias y regularización de omisos y saldos pendientes.</t>
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>67</v>
-      </c>
-      <c r="H15" s="33" t="inlineStr">
-        <is>
-          <t>Contribuyentes &gt; Servicios al Contribuyente &gt; Plataforma Digital, Citas y Solvencias</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
+        <v>7</v>
+      </c>
+      <c r="H15" s="39">
+        <f>G15/$G$18</f>
+        <v/>
+      </c>
+      <c r="I15" s="39">
+        <f>G15/$G$44</f>
+        <v/>
+      </c>
+      <c r="J15" s="38" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; Solvencia y Convenios</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
       <c r="B16" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D16" s="38" t="inlineStr">
-        <is>
-          <t>Importadores y Exportadores (Compartido)</t>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyentes</t>
+        </is>
+      </c>
+      <c r="D16" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="E16" s="35" t="inlineStr">
         <is>
-          <t>Operadores Comerciales Generales</t>
-        </is>
-      </c>
-      <c r="F16" s="35" t="inlineStr">
-        <is>
-          <t>Gestiones Aduaneras Comunes y Arancel</t>
+          <t>Asalariados</t>
+        </is>
+      </c>
+      <c r="F16" s="41" t="inlineStr">
+        <is>
+          <t>Rentas del trabajo en relación de dependencia, planilla electrónica del IVA y devolución de retenciones de ISR.</t>
         </is>
       </c>
       <c r="G16" s="22" t="n">
-        <v>16</v>
-      </c>
-      <c r="H16" s="35" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Importadores y Exportadores (Compartido) &gt; Gestiones Aduaneras Comunes y Arancel</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="H16" s="42">
+        <f>G16/$G$18</f>
+        <v/>
+      </c>
+      <c r="I16" s="42">
+        <f>G16/$G$44</f>
+        <v/>
+      </c>
+      <c r="J16" s="41" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyente General &gt; Asalariados</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
       <c r="B17" s="10" t="n">
         <v>11</v>
       </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
-          <t>Operadores de Comercio Exterior</t>
+          <t>Contribuyentes</t>
         </is>
       </c>
       <c r="D17" s="37" t="inlineStr">
         <is>
-          <t>Importadores</t>
+          <t>Contribuyentes Especiales</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
         <is>
-          <t>Importadores Registrados</t>
-        </is>
-      </c>
-      <c r="F17" s="33" t="inlineStr">
-        <is>
-          <t>Padrón de Importadores y DUCA-D</t>
+          <t>Contribuyentes Especiales</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr">
+        <is>
+          <t>Atención en gerencias diferenciadas, presentación de estados financieros auditados y precios de transferencia.</t>
         </is>
       </c>
       <c r="G17" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="H17" s="33" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Importadores &gt; Padrón de Importadores y DUCA-D</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="17" t="n">
+      <c r="H17" s="39">
+        <f>G17/$G$18</f>
+        <v/>
+      </c>
+      <c r="I17" s="39">
+        <f>G17/$G$44</f>
+        <v/>
+      </c>
+      <c r="J17" s="38" t="inlineStr">
+        <is>
+          <t>Contribuyentes &gt; Contribuyentes Especiales &gt; Contribuyentes Especiales</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="B18" s="43" t="inlineStr"/>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>SUBTOTAL CONTRIBUYENTES</t>
+        </is>
+      </c>
+      <c r="D18" s="45" t="inlineStr">
+        <is>
+          <t>11 Categorías / Actores</t>
+        </is>
+      </c>
+      <c r="E18" s="43" t="inlineStr"/>
+      <c r="F18" s="43" t="inlineStr"/>
+      <c r="G18" s="46">
+        <f>SUM(G7:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="46" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I18" s="47">
+        <f>G18/$G$44</f>
+        <v/>
+      </c>
+      <c r="J18" s="45" t="inlineStr">
+        <is>
+          <t>Cobertura completa de Contribuyentes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="B19" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="C18" s="38" t="inlineStr">
+      <c r="C19" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D18" s="38" t="inlineStr">
+      <c r="D19" s="37" t="inlineStr">
+        <is>
+          <t>1. Importadores y Exportadores</t>
+        </is>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>Importadores y Exportadores (Compartido)</t>
+        </is>
+      </c>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
+          <t>Arancel Integrado Centroamericano (SAC), pagos aduaneros por BancaSAT, DUCAs comunes y solvencia aduanera.</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H19" s="39">
+        <f>G19/$G$31</f>
+        <v/>
+      </c>
+      <c r="I19" s="39">
+        <f>G19/$G$44</f>
+        <v/>
+      </c>
+      <c r="J19" s="38" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Importadores y Exportadores (Compartido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="B20" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D20" s="40" t="inlineStr">
+        <is>
+          <t>1. Importadores y Exportadores</t>
+        </is>
+      </c>
+      <c r="E20" s="35" t="inlineStr">
+        <is>
+          <t>Importadores</t>
+        </is>
+      </c>
+      <c r="F20" s="41" t="inlineStr">
+        <is>
+          <t>Inscripción en padrón de importadores, liquidación de DUCA-D, valoración aduanera y rescate de mercancías.</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" s="42">
+        <f>G20/$G$31</f>
+        <v/>
+      </c>
+      <c r="I20" s="42">
+        <f>G20/$G$44</f>
+        <v/>
+      </c>
+      <c r="J20" s="41" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Importadores</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="B21" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C21" s="37" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D21" s="37" t="inlineStr">
+        <is>
+          <t>1. Importadores y Exportadores</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
         <is>
           <t>Exportadores</t>
         </is>
       </c>
-      <c r="E18" s="35" t="inlineStr">
-        <is>
-          <t>Exportadores Habituales y Ocasionales</t>
-        </is>
-      </c>
-      <c r="F18" s="35" t="inlineStr">
-        <is>
-          <t>Padrón de Exportadores y Devolución IVA</t>
-        </is>
-      </c>
-      <c r="G18" s="22" t="n">
+      <c r="F21" s="38" t="inlineStr">
+        <is>
+          <t>Registro de exportadores VUPE, autorización de embarques y devolución de crédito fiscal del IVA para exportadores.</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="H18" s="35" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Exportadores &gt; Padrón de Exportadores y Devolución IVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="10" t="n">
-        <v>13</v>
-      </c>
-      <c r="C19" s="37" t="inlineStr">
+      <c r="H21" s="39">
+        <f>G21/$G$31</f>
+        <v/>
+      </c>
+      <c r="I21" s="39">
+        <f>G21/$G$44</f>
+        <v/>
+      </c>
+      <c r="J21" s="38" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Exportadores</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="B22" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="C22" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D19" s="37" t="inlineStr">
+      <c r="D22" s="40" t="inlineStr">
+        <is>
+          <t>1. Importadores y Exportadores</t>
+        </is>
+      </c>
+      <c r="E22" s="35" t="inlineStr">
         <is>
           <t>Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
-      <c r="E19" s="33" t="inlineStr">
-        <is>
-          <t>Operadores Certificados en Seguridad</t>
-        </is>
-      </c>
-      <c r="F19" s="33" t="inlineStr">
-        <is>
-          <t>Cadena Logística Segura y Carril Exprés</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="n">
+      <c r="F22" s="41" t="inlineStr">
+        <is>
+          <t>Certificación en seguridad de la cadena de suministro, carril exprés aduanero y reducción de selectivo rojo.</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="33" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Operador Económico Autorizado (OEA) &gt; Cadena Logística Segura y Carril Exprés</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="17" t="n">
-        <v>14</v>
-      </c>
-      <c r="C20" s="38" t="inlineStr">
+      <c r="H22" s="42">
+        <f>G22/$G$31</f>
+        <v/>
+      </c>
+      <c r="I22" s="42">
+        <f>G22/$G$44</f>
+        <v/>
+      </c>
+      <c r="J22" s="41" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Operador Económico Autorizado (OEA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="B23" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C23" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D20" s="38" t="inlineStr">
+      <c r="D23" s="37" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="E23" s="33" t="inlineStr">
+        <is>
+          <t>Depósitos Aduaneros</t>
+        </is>
+      </c>
+      <c r="F23" s="38" t="inlineStr">
+        <is>
+          <t>Almacenes Fiscales, Almacenes Generales de Depósito (AGD) y Depósitos Aduaneros Temporales (DAT).</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="H23" s="39">
+        <f>G23/$G$31</f>
+        <v/>
+      </c>
+      <c r="I23" s="39">
+        <f>G23/$G$44</f>
+        <v/>
+      </c>
+      <c r="J23" s="38" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Depósitos Aduaneros</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="B24" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D24" s="40" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>Agentes Aduaneros</t>
         </is>
       </c>
-      <c r="E20" s="35" t="inlineStr">
-        <is>
-          <t>Auxiliares de la Función Pública Aduanera</t>
-        </is>
-      </c>
-      <c r="F20" s="35" t="inlineStr">
-        <is>
-          <t>Despacho Aduanero Oficial y Representación</t>
-        </is>
-      </c>
-      <c r="G20" s="22" t="n">
-        <v>16</v>
-      </c>
-      <c r="H20" s="35" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Agentes Aduaneros &gt; Despacho Aduanero Oficial y Representación</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="C21" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D21" s="37" t="inlineStr">
-        <is>
-          <t>Apoderados Especiales Aduaneros</t>
-        </is>
-      </c>
-      <c r="E21" s="33" t="inlineStr">
-        <is>
-          <t>Representantes Legales Exclusivos</t>
-        </is>
-      </c>
-      <c r="F21" s="33" t="inlineStr">
-        <is>
-          <t>Despacho Aduanero por Cuenta Propia</t>
-        </is>
-      </c>
-      <c r="G21" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="H21" s="33" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Apoderados Especiales Aduaneros &gt; Despacho Aduanero por Cuenta Propia</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="17" t="n">
-        <v>16</v>
-      </c>
-      <c r="C22" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D22" s="38" t="inlineStr">
-        <is>
-          <t>Empresas de Entrega Rápida o Courier</t>
-        </is>
-      </c>
-      <c r="E22" s="35" t="inlineStr">
-        <is>
-          <t>Mensajería y Envíos Expresos</t>
-        </is>
-      </c>
-      <c r="F22" s="35" t="inlineStr">
-        <is>
-          <t>Paquetería Internacional y Franquicias</t>
-        </is>
-      </c>
-      <c r="G22" s="22" t="n">
-        <v>13</v>
-      </c>
-      <c r="H22" s="35" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Empresas de Entrega Rápida o Courier &gt; Paquetería Internacional y Franquicias</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="C23" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D23" s="37" t="inlineStr">
-        <is>
-          <t>Consolidadores y Desconsolidadores de Carga</t>
-        </is>
-      </c>
-      <c r="E23" s="33" t="inlineStr">
-        <is>
-          <t>Operadores Logísticos y de Carga</t>
-        </is>
-      </c>
-      <c r="F23" s="33" t="inlineStr">
-        <is>
-          <t>Manifiestos CUSCAR y Guías Hijas</t>
-        </is>
-      </c>
-      <c r="G23" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="H23" s="33" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Consolidadores y Desconsolidadores de Carga &gt; Manifiestos CUSCAR y Guías Hijas</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="C24" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D24" s="38" t="inlineStr">
-        <is>
-          <t>Transportistas Aduaneros</t>
-        </is>
-      </c>
-      <c r="E24" s="35" t="inlineStr">
-        <is>
-          <t>Transporte Internacional Terrestre y Carga</t>
-        </is>
-      </c>
-      <c r="F24" s="35" t="inlineStr">
-        <is>
-          <t>Tránsito Aduanero Internacional y Marchamo</t>
+      <c r="F24" s="41" t="inlineStr">
+        <is>
+          <t>Habilitación de carné oficial, constitución de pólizas de caución y transmisión de DUCAs con firma electrónica.</t>
         </is>
       </c>
       <c r="G24" s="22" t="n">
         <v>16</v>
       </c>
-      <c r="H24" s="35" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Transportistas Aduaneros &gt; Tránsito Aduanero Internacional y Marchamo</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
+      <c r="H24" s="42">
+        <f>G24/$G$31</f>
+        <v/>
+      </c>
+      <c r="I24" s="42">
+        <f>G24/$G$44</f>
+        <v/>
+      </c>
+      <c r="J24" s="41" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Agentes Aduaneros</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
       <c r="B25" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="C25" s="37" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D25" s="37" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>Apoderados Especiales Aduaneros</t>
+        </is>
+      </c>
+      <c r="F25" s="38" t="inlineStr">
+        <is>
+          <t>Representación exclusiva de personas jurídicas en despachos aduaneros propios, carné y renovación de fianza.</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H25" s="39">
+        <f>G25/$G$31</f>
+        <v/>
+      </c>
+      <c r="I25" s="39">
+        <f>G25/$G$44</f>
+        <v/>
+      </c>
+      <c r="J25" s="38" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Apoderados Especiales Aduaneros</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="B26" s="17" t="n">
         <v>19</v>
       </c>
-      <c r="C25" s="37" t="inlineStr">
+      <c r="C26" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D25" s="37" t="inlineStr">
-        <is>
-          <t>Depósitos Aduaneros</t>
-        </is>
-      </c>
-      <c r="E25" s="33" t="inlineStr">
-        <is>
-          <t>Almacenes Fiscales, AGD y DAT</t>
-        </is>
-      </c>
-      <c r="F25" s="33" t="inlineStr">
-        <is>
-          <t>Custodia de Mercancías y Títulos de Crédito</t>
-        </is>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>50</v>
-      </c>
-      <c r="H25" s="33" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; Depósitos Aduaneros &gt; Custodia de Mercancías y Títulos de Crédito</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="17" t="n">
+      <c r="D26" s="40" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="E26" s="35" t="inlineStr">
+        <is>
+          <t>Transportistas Aduaneros</t>
+        </is>
+      </c>
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>Registro de unidades y conductores, transmisión de DUCA-T y colocación de marchamo electrónico RFID.</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="n">
+        <v>16</v>
+      </c>
+      <c r="H26" s="42">
+        <f>G26/$G$31</f>
+        <v/>
+      </c>
+      <c r="I26" s="42">
+        <f>G26/$G$44</f>
+        <v/>
+      </c>
+      <c r="J26" s="41" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Transportistas Aduaneros</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="B27" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="C26" s="38" t="inlineStr">
+      <c r="C27" s="37" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D26" s="38" t="inlineStr">
+      <c r="D27" s="37" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="E27" s="33" t="inlineStr">
+        <is>
+          <t>Empresas de Entrega Rápida o Courier</t>
+        </is>
+      </c>
+      <c r="F27" s="38" t="inlineStr">
+        <is>
+          <t>Despacho simplificado de paquetería urgente, manifiestos courier y recintos desconsolidadores de encomiendas.</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="H27" s="39">
+        <f>G27/$G$31</f>
+        <v/>
+      </c>
+      <c r="I27" s="39">
+        <f>G27/$G$44</f>
+        <v/>
+      </c>
+      <c r="J27" s="38" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Empresas de Entrega Rápida o Courier</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="B28" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D28" s="40" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="E28" s="35" t="inlineStr">
+        <is>
+          <t>Consolidadores y Desconsolidadores de Carga</t>
+        </is>
+      </c>
+      <c r="F28" s="41" t="inlineStr">
+        <is>
+          <t>Transmisión de manifiesto electrónico CUSCAR, desconsolidación de conocimientos de embarque y guías hijas.</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="H28" s="42">
+        <f>G28/$G$31</f>
+        <v/>
+      </c>
+      <c r="I28" s="42">
+        <f>G28/$G$44</f>
+        <v/>
+      </c>
+      <c r="J28" s="41" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Consolidadores y Desconsolidadores de Carga</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="B29" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="C29" s="37" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="D29" s="37" t="inlineStr">
+        <is>
+          <t>3. Regímenes Territoriales y Zonas Especiales</t>
+        </is>
+      </c>
+      <c r="E29" s="33" t="inlineStr">
         <is>
           <t>ZDEEP - Entidades Administradoras</t>
         </is>
       </c>
-      <c r="E26" s="35" t="inlineStr">
-        <is>
-          <t>Polígonos ZDEEP</t>
-        </is>
-      </c>
-      <c r="F26" s="35" t="inlineStr">
-        <is>
-          <t>Administración de Zonas Especiales Públicas</t>
-        </is>
-      </c>
-      <c r="G26" s="22" t="n">
+      <c r="F29" s="38" t="inlineStr">
+        <is>
+          <t>Habilitación de polígonos industriales ZDEEP, supervisión perimetral, garitas de control y recintos aduaneros.</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="H26" s="35" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; ZDEEP - Entidades Administradoras &gt; Administración de Zonas Especiales Públicas</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="C27" s="37" t="inlineStr">
+      <c r="H29" s="39">
+        <f>G29/$G$31</f>
+        <v/>
+      </c>
+      <c r="I29" s="39">
+        <f>G29/$G$44</f>
+        <v/>
+      </c>
+      <c r="J29" s="38" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 3. Regímenes Territoriales y Zonas Especiales &gt; ZDEEP - Entidades Administradoras</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="B30" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="C30" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D27" s="37" t="inlineStr">
+      <c r="D30" s="40" t="inlineStr">
+        <is>
+          <t>3. Regímenes Territoriales y Zonas Especiales</t>
+        </is>
+      </c>
+      <c r="E30" s="35" t="inlineStr">
         <is>
           <t>ZDEEP - Empresas Usuarias</t>
         </is>
       </c>
-      <c r="E27" s="33" t="inlineStr">
-        <is>
-          <t>Empresas Instaladas en ZDEEP</t>
-        </is>
-      </c>
-      <c r="F27" s="33" t="inlineStr">
-        <is>
-          <t>Transformación, Servicios y Exenciones</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="n">
+      <c r="F30" s="41" t="inlineStr">
+        <is>
+          <t>Ingreso de insumos con suspensión arancelaria, descargos de transformación y exenciones tributarias de fomento.</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="H27" s="33" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; ZDEEP - Empresas Usuarias &gt; Transformación, Servicios y Exenciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="C28" s="38" t="inlineStr">
+      <c r="H30" s="42">
+        <f>G30/$G$31</f>
+        <v/>
+      </c>
+      <c r="I30" s="42">
+        <f>G30/$G$44</f>
+        <v/>
+      </c>
+      <c r="J30" s="41" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; 3. Regímenes Territoriales y Zonas Especiales &gt; ZDEEP - Empresas Usuarias</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="B31" s="43" t="inlineStr"/>
+      <c r="C31" s="44" t="inlineStr">
+        <is>
+          <t>SUBTOTAL OPERADORES DE COMERCIO EXTERIOR</t>
+        </is>
+      </c>
+      <c r="D31" s="45" t="inlineStr">
+        <is>
+          <t>12 Categorías / Actores</t>
+        </is>
+      </c>
+      <c r="E31" s="43" t="inlineStr"/>
+      <c r="F31" s="43" t="inlineStr"/>
+      <c r="G31" s="46">
+        <f>SUM(G19:G30)</f>
+        <v/>
+      </c>
+      <c r="H31" s="46" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I31" s="47">
+        <f>G31/$G$44</f>
+        <v/>
+      </c>
+      <c r="J31" s="45" t="inlineStr">
+        <is>
+          <t>Cobertura completa de Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="B32" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="C32" s="40" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D28" s="38" t="inlineStr">
+      <c r="D32" s="40" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
+        </is>
+      </c>
+      <c r="E32" s="35" t="inlineStr">
         <is>
           <t>Abogados y Notarios</t>
         </is>
       </c>
-      <c r="E28" s="35" t="inlineStr">
-        <is>
-          <t>Notarios en Ejercicio</t>
-        </is>
-      </c>
-      <c r="F28" s="35" t="inlineStr">
-        <is>
-          <t>Papel Sellado de Protocolo y Avisos</t>
-        </is>
-      </c>
-      <c r="G28" s="22" t="n">
+      <c r="F32" s="41" t="inlineStr">
+        <is>
+          <t>Compra de papel sellado de protocolo (SAT-7130), timbres fiscales y traspasos electrónicos vehiculares (TEV).</t>
+        </is>
+      </c>
+      <c r="G32" s="22" t="n">
         <v>17</v>
       </c>
-      <c r="H28" s="35" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Abogados y Notarios &gt; Papel Sellado de Protocolo y Avisos</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="10" t="n">
-        <v>23</v>
-      </c>
-      <c r="C29" s="37" t="inlineStr">
+      <c r="H32" s="42">
+        <f>G32/$G$37</f>
+        <v/>
+      </c>
+      <c r="I32" s="42">
+        <f>G32/$G$44</f>
+        <v/>
+      </c>
+      <c r="J32" s="41" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Abogados y Notarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="B33" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C33" s="37" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D29" s="37" t="inlineStr">
+      <c r="D33" s="37" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
+        </is>
+      </c>
+      <c r="E33" s="33" t="inlineStr">
         <is>
           <t>Peritos Contadores</t>
         </is>
       </c>
-      <c r="E29" s="33" t="inlineStr">
-        <is>
-          <t>Contadores Registrados</t>
-        </is>
-      </c>
-      <c r="F29" s="33" t="inlineStr">
-        <is>
-          <t>Libros Contables y Declaraciones</t>
-        </is>
-      </c>
-      <c r="G29" s="15" t="n">
+      <c r="F33" s="38" t="inlineStr">
+        <is>
+          <t>Inscripción en el Registro de Contadores, autorización de libros contables digitales y firma de balances.</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="H29" s="33" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Peritos Contadores &gt; Libros Contables y Declaraciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="C30" s="38" t="inlineStr">
+      <c r="H33" s="39">
+        <f>G33/$G$37</f>
+        <v/>
+      </c>
+      <c r="I33" s="39">
+        <f>G33/$G$44</f>
+        <v/>
+      </c>
+      <c r="J33" s="38" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Peritos Contadores</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="B34" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D30" s="38" t="inlineStr">
-        <is>
-          <t>Auditores</t>
-        </is>
-      </c>
-      <c r="E30" s="35" t="inlineStr">
-        <is>
-          <t>Contadores Públicos y Auditores (CPA)</t>
-        </is>
-      </c>
-      <c r="F30" s="35" t="inlineStr">
-        <is>
-          <t>Dictámenes Tributarios y Devolución IVA</t>
-        </is>
-      </c>
-      <c r="G30" s="22" t="n">
-        <v>4</v>
-      </c>
-      <c r="H30" s="35" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Auditores &gt; Dictámenes Tributarios y Devolución IVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="C31" s="37" t="inlineStr">
+      <c r="D34" s="40" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
+        </is>
+      </c>
+      <c r="E34" s="35" t="inlineStr">
+        <is>
+          <t>Gestores Tributarios</t>
+        </is>
+      </c>
+      <c r="F34" s="41" t="inlineStr">
+        <is>
+          <t>Acreditación oficial ante SAT, renovación de gafetes, registro biométrico y representación presencial autorizada.</t>
+        </is>
+      </c>
+      <c r="G34" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="H34" s="42">
+        <f>G34/$G$37</f>
+        <v/>
+      </c>
+      <c r="I34" s="42">
+        <f>G34/$G$44</f>
+        <v/>
+      </c>
+      <c r="J34" s="41" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Gestores Tributarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1">
+      <c r="B35" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="C35" s="37" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="D31" s="37" t="inlineStr">
-        <is>
-          <t>Gestores Tributarios</t>
-        </is>
-      </c>
-      <c r="E31" s="33" t="inlineStr">
-        <is>
-          <t>Gestores Acreditados SAT</t>
-        </is>
-      </c>
-      <c r="F31" s="33" t="inlineStr">
-        <is>
-          <t>Gafetes y Trámites Presenciales</t>
-        </is>
-      </c>
-      <c r="G31" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="H31" s="33" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Gestores Tributarios &gt; Gafetes y Trámites Presenciales</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="17" t="n">
-        <v>26</v>
-      </c>
-      <c r="C32" s="38" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="D32" s="38" t="inlineStr">
+      <c r="D35" s="37" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
+        </is>
+      </c>
+      <c r="E35" s="33" t="inlineStr">
         <is>
           <t>Servicios Profesionales</t>
         </is>
       </c>
-      <c r="E32" s="35" t="inlineStr">
-        <is>
-          <t>Profesionales Liberales Independientes</t>
-        </is>
-      </c>
-      <c r="F32" s="35" t="inlineStr">
-        <is>
-          <t>Facturación por Honorarios y Retenciones</t>
-        </is>
-      </c>
-      <c r="G32" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="H32" s="35" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Servicios Profesionales &gt; Facturación por Honorarios y Retenciones</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="B33" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D33" s="37" t="inlineStr">
-        <is>
-          <t>Constitucionales</t>
-        </is>
-      </c>
-      <c r="E33" s="33" t="inlineStr">
-        <is>
-          <t>Universidades, Colegios e Iglesias</t>
-        </is>
-      </c>
-      <c r="F33" s="33" t="inlineStr">
-        <is>
-          <t>Exenciones Tributarias de Rango Constitucional</t>
-        </is>
-      </c>
-      <c r="G33" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="H33" s="33" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Constitucionales &gt; Exenciones Tributarias de Rango Constitucional</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="17" t="n">
-        <v>28</v>
-      </c>
-      <c r="C34" s="38" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D34" s="38" t="inlineStr">
-        <is>
-          <t>No Lucrativos</t>
-        </is>
-      </c>
-      <c r="E34" s="35" t="inlineStr">
-        <is>
-          <t>ONGs, Fundaciones y Cooperativas</t>
-        </is>
-      </c>
-      <c r="F34" s="35" t="inlineStr">
-        <is>
-          <t>Reconocimiento de Exención de ISR e IVA</t>
-        </is>
-      </c>
-      <c r="G34" s="22" t="n">
-        <v>14</v>
-      </c>
-      <c r="H34" s="35" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; No Lucrativos &gt; Reconocimiento de Exención de ISR e IVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="10" t="n">
-        <v>29</v>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D35" s="37" t="inlineStr">
-        <is>
-          <t>Municipalidades</t>
-        </is>
-      </c>
-      <c r="E35" s="33" t="inlineStr">
-        <is>
-          <t>Gobiernos Locales y Empresas Municipales</t>
-        </is>
-      </c>
-      <c r="F35" s="33" t="inlineStr">
-        <is>
-          <t>Autonomía Municipal y Régimen Exento</t>
+      <c r="F35" s="38" t="inlineStr">
+        <is>
+          <t>Facturación FEL por honorarios profesionales, retenciones de ISR y actualización de constancia de colegiado activo.</t>
         </is>
       </c>
       <c r="G35" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="H35" s="33" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Municipalidades &gt; Autonomía Municipal y Régimen Exento</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
+      <c r="H35" s="39">
+        <f>G35/$G$37</f>
+        <v/>
+      </c>
+      <c r="I35" s="39">
+        <f>G35/$G$44</f>
+        <v/>
+      </c>
+      <c r="J35" s="38" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Servicios Profesionales</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
       <c r="B36" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D36" s="40" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
+        </is>
+      </c>
+      <c r="E36" s="35" t="inlineStr">
+        <is>
+          <t>Auditores</t>
+        </is>
+      </c>
+      <c r="F36" s="41" t="inlineStr">
+        <is>
+          <t>Dictámenes de crédito fiscal para exportadores, dictámenes de estados financieros e informes tributarios.</t>
+        </is>
+      </c>
+      <c r="G36" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="H36" s="42">
+        <f>G36/$G$37</f>
+        <v/>
+      </c>
+      <c r="I36" s="42">
+        <f>G36/$G$44</f>
+        <v/>
+      </c>
+      <c r="J36" s="41" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Auditores</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1">
+      <c r="B37" s="43" t="inlineStr"/>
+      <c r="C37" s="44" t="inlineStr">
+        <is>
+          <t>SUBTOTAL PROFESIONALES</t>
+        </is>
+      </c>
+      <c r="D37" s="45" t="inlineStr">
+        <is>
+          <t>5 Categorías / Actores</t>
+        </is>
+      </c>
+      <c r="E37" s="43" t="inlineStr"/>
+      <c r="F37" s="43" t="inlineStr"/>
+      <c r="G37" s="46">
+        <f>SUM(G32:G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="46" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I37" s="47">
+        <f>G37/$G$44</f>
+        <v/>
+      </c>
+      <c r="J37" s="45" t="inlineStr">
+        <is>
+          <t>Cobertura completa de Profesionales</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="B38" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D38" s="40" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
+        </is>
+      </c>
+      <c r="E38" s="35" t="inlineStr">
+        <is>
+          <t>Constitucionales</t>
+        </is>
+      </c>
+      <c r="F38" s="41" t="inlineStr">
+        <is>
+          <t>Exención constitucional de impuestos para universidades, colegios, iglesias y misiones diplomáticas.</t>
+        </is>
+      </c>
+      <c r="G38" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="H38" s="42">
+        <f>G38/$G$43</f>
+        <v/>
+      </c>
+      <c r="I38" s="42">
+        <f>G38/$G$44</f>
+        <v/>
+      </c>
+      <c r="J38" s="41" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; Constitucionales</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="B39" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="C36" s="38" t="inlineStr">
+      <c r="C39" s="37" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D36" s="38" t="inlineStr">
+      <c r="D39" s="37" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
+        </is>
+      </c>
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>Decreto</t>
+        </is>
+      </c>
+      <c r="F39" s="38" t="inlineStr">
+        <is>
+          <t>Entidades con incentivos y exenciones especiales otorgadas por leyes ordinarias de fomento sectorial.</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H39" s="39">
+        <f>G39/$G$43</f>
+        <v/>
+      </c>
+      <c r="I39" s="39">
+        <f>G39/$G$44</f>
+        <v/>
+      </c>
+      <c r="J39" s="38" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; Decreto</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="B40" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D40" s="40" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
+        </is>
+      </c>
+      <c r="E40" s="35" t="inlineStr">
+        <is>
+          <t>No Lucrativos</t>
+        </is>
+      </c>
+      <c r="F40" s="41" t="inlineStr">
+        <is>
+          <t>Resoluciones de exención de ISR e IVA para ONGs, fundaciones benéficas, asociaciones y cooperativas.</t>
+        </is>
+      </c>
+      <c r="G40" s="22" t="n">
+        <v>14</v>
+      </c>
+      <c r="H40" s="42">
+        <f>G40/$G$43</f>
+        <v/>
+      </c>
+      <c r="I40" s="42">
+        <f>G40/$G$44</f>
+        <v/>
+      </c>
+      <c r="J40" s="41" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; No Lucrativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1">
+      <c r="B41" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="C41" s="37" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D41" s="37" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
+        </is>
+      </c>
+      <c r="E41" s="33" t="inlineStr">
         <is>
           <t>Entidades del Estado</t>
         </is>
       </c>
-      <c r="E36" s="35" t="inlineStr">
-        <is>
-          <t>Ministerios, Secretarías y Organismos del Estado</t>
-        </is>
-      </c>
-      <c r="F36" s="35" t="inlineStr">
-        <is>
-          <t>Compras Públicas y Agentes de Retención</t>
-        </is>
-      </c>
-      <c r="G36" s="22" t="n">
+      <c r="F41" s="38" t="inlineStr">
+        <is>
+          <t>Ministerios, secretarías, organismos del Estado, compras públicas y emisión de constancias de retención.</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="n">
         <v>26</v>
       </c>
-      <c r="H36" s="35" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Entidades del Estado &gt; Compras Públicas y Agentes de Retención</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="B37" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="C37" s="37" t="inlineStr">
+      <c r="H41" s="39">
+        <f>G41/$G$43</f>
+        <v/>
+      </c>
+      <c r="I41" s="39">
+        <f>G41/$G$44</f>
+        <v/>
+      </c>
+      <c r="J41" s="38" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Sector Público y Entidades del Estado &gt; Entidades del Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="24" customHeight="1">
+      <c r="B42" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="C42" s="40" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="D37" s="37" t="inlineStr">
-        <is>
-          <t>Decreto</t>
-        </is>
-      </c>
-      <c r="E37" s="33" t="inlineStr">
-        <is>
-          <t>Entidades con Incentivos Especiales</t>
-        </is>
-      </c>
-      <c r="F37" s="33" t="inlineStr">
-        <is>
-          <t>Exenciones y Fomento por Decreto Legislativo</t>
-        </is>
-      </c>
-      <c r="G37" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="H37" s="33" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Decreto &gt; Exenciones y Fomento por Decreto Legislativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="24" t="inlineStr"/>
-      <c r="C38" s="25" t="inlineStr">
-        <is>
-          <t>TOTAL DEL PORTAL</t>
-        </is>
-      </c>
-      <c r="D38" s="26" t="inlineStr">
-        <is>
-          <t>4 Segmentos y 31 Categorías Principales</t>
-        </is>
-      </c>
-      <c r="E38" s="24" t="inlineStr"/>
-      <c r="F38" s="24" t="inlineStr"/>
-      <c r="G38" s="27">
-        <f>SUM(G7:G37)</f>
-        <v/>
-      </c>
-      <c r="H38" s="25" t="inlineStr">
-        <is>
-          <t>739 Trámites Oficiales Integrados</t>
+      <c r="D42" s="40" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
+        </is>
+      </c>
+      <c r="E42" s="35" t="inlineStr">
+        <is>
+          <t>Municipalidades</t>
+        </is>
+      </c>
+      <c r="F42" s="41" t="inlineStr">
+        <is>
+          <t>Autonomía municipal, inscripción de corporaciones y flotillas vehiculares municipales exentas del ISCV.</t>
+        </is>
+      </c>
+      <c r="G42" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="H42" s="42">
+        <f>G42/$G$43</f>
+        <v/>
+      </c>
+      <c r="I42" s="42">
+        <f>G42/$G$44</f>
+        <v/>
+      </c>
+      <c r="J42" s="41" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Sector Público y Entidades del Estado &gt; Municipalidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="24" customHeight="1">
+      <c r="B43" s="43" t="inlineStr"/>
+      <c r="C43" s="44" t="inlineStr">
+        <is>
+          <t>SUBTOTAL ENTES EXENTOS</t>
+        </is>
+      </c>
+      <c r="D43" s="45" t="inlineStr">
+        <is>
+          <t>5 Categorías / Actores</t>
+        </is>
+      </c>
+      <c r="E43" s="43" t="inlineStr"/>
+      <c r="F43" s="43" t="inlineStr"/>
+      <c r="G43" s="46">
+        <f>SUM(G38:G42)</f>
+        <v/>
+      </c>
+      <c r="H43" s="46" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I43" s="47">
+        <f>G43/$G$44</f>
+        <v/>
+      </c>
+      <c r="J43" s="45" t="inlineStr">
+        <is>
+          <t>Cobertura completa de Entes Exentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
+      <c r="B44" s="48" t="inlineStr"/>
+      <c r="C44" s="49" t="inlineStr">
+        <is>
+          <t>TOTAL PORTAL WEB SAT</t>
+        </is>
+      </c>
+      <c r="D44" s="50" t="inlineStr">
+        <is>
+          <t>4 Segmentos y 33 Categorías</t>
+        </is>
+      </c>
+      <c r="E44" s="48" t="inlineStr"/>
+      <c r="F44" s="49" t="inlineStr">
+        <is>
+          <t>Universo Total de Fichas Oficiales</t>
+        </is>
+      </c>
+      <c r="G44" s="51">
+        <f>G18+G31+G37+G43</f>
+        <v/>
+      </c>
+      <c r="H44" s="52" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="53" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="J44" s="49" t="inlineStr">
+        <is>
+          <t>739 Trámites 100% Mapeados</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B2:H3"/>
+    <mergeCell ref="B2:J3"/>
+    <mergeCell ref="B4:J4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2414,17 +2957,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H37"/>
+  <dimension ref="A2:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2438,7 +2981,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MATRIZ COMPLETA DE LAS 31 CATEGORÍAS DEL PORTAL CON SUS TEXTOS ORIENTADORES Y MARCO NORMATIVO OFICIAL</t>
+          <t>MATRIZ COMPLETA DE LAS 33 CATEGORÍAS DEL PORTAL CON SUS TEXTOS ORIENTADORES Y MARCO NORMATIVO OFICIAL</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2998,12 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Categoría / Rol (Nivel 2/3)</t>
+          <t>Régimen / Área (Nivel 2)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Tema / Especialidad (Nivel 4)</t>
+          <t>Categoría / Actor (Nivel 3)</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2484,7 +3027,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1">
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="10" t="n">
         <v>1</v>
       </c>
@@ -2500,17 +3043,17 @@
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>RTU Digital y Solicitud de NIT</t>
+          <t>NIT sin Obligaciones</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Categoría destinada a personas individuales (estudiantes, personas en relación de dependencia sin renta afecta o ciudadanos en el extranjero) que requieren un Número de Identificación Tributaria únicamente para actos civiles, contractuales, bancarios o de registro público, sin realizar actividades mercantiles ni prestación de servicios técnicos afectos.</t>
+          <t>Categoría destinada a personas individuales (estudiantes, asalariados no afectos, personas que compran bienes o abren cuentas bancarias) que requieren un Número de Identificación Tributaria únicamente para actos civiles, contractuales o notariales sin realizar actividades mercantiles ni prestación de servicios técnicos afectos.</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Inscribe tu primer NIT en línea, actualiza tus datos de residencia y obtén tu constancia de solvencia fiscal sin necesidad de acudir a una agencia.</t>
+          <t>Inscribe tu primer NIT en línea, actualiza tus datos de residencia y obtén tu solvencia fiscal sin acudir a una agencia.</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
@@ -2522,45 +3065,45 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" ht="50" customHeight="1">
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="38" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C8" s="38" t="inlineStr">
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
       <c r="D8" s="35" t="inlineStr">
         <is>
-          <t>Régimen de 5% y Facturación FEL</t>
+          <t>Pequeños Contribuyentes</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Régimen simplificado para personas individuales o jurídicas cuyas ventas de bienes o prestación de servicios no superan el monto de Q150,000 en el año calendario, tributando bajo una tarifa definitiva del 5% sobre ingresos brutos mensuales sin derecho a crédito fiscal.</t>
+          <t>Régimen simplificado para personas individuales o jurídicas cuyas ventas de bienes o prestación de servicios no superan el monto de Q150,000 en el año calendario, tributando bajo una tarifa definitiva del 5% sobre ingresos brutos mensuales sin derecho a crédito fiscal, incluyendo productores agropecuarios (ICT).</t>
         </is>
       </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
-          <t>Emite tus facturas electrónicas FEL de pequeño contribuyente, declara mensualmente el 5% en Declaraguate y mantén tus libros al día.</t>
+          <t>Emite tus facturas FEL de pequeño contribuyente, declara el 5% mensual en Declaraguate y consulta tus libros digitales.</t>
         </is>
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>Ley del IVA (Decreto 27-92, Arts. 45 al 50) y Ley de Simplificación Tributaria (Decreto 7-2019, Régimen Electrónico de Pequeño Contribuyente).</t>
+          <t>Ley del IVA (Decreto 27-92, Arts. 45 al 50), Decreto 7-2019 (Régimen Electrónico) y Decreto 31-2024 (Sector Primario y Agropecuario).</t>
         </is>
       </c>
       <c r="H8" s="22" t="n">
         <v>22</v>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="10" t="n">
         <v>3</v>
       </c>
@@ -2571,72 +3114,72 @@
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
-          <t>Pequeños Contribuyentes</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="D9" s="33" t="inlineStr">
         <is>
-          <t>Regímenes Especiales Decreto 31-2024 / 7-2019</t>
+          <t>Declaraciones y Pagos</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Regímenes tributarios especiales creados para productores, ganaderos y comercializadores del sector agropecuario, artesanal y primario que comercializan productos no transformados.</t>
+          <t>Gestión y liquidación periódica de impuestos internos directos e indirectos (IVA General 12%, ISR Actividades Lucrativas, ISO, Timbres Fiscales, IETAP) mediante formularios oficiales en Declaraguate y boletas de pago SAT-2000.</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Inscríbete en el régimen especial agropecuario, liquida tu Impuesto a la Confianza Tributaria y emite comprobantes oficiales simplificados.</t>
+          <t>Llena tus formularios oficiales en Declaraguate, genera tu boleta SAT-2000 y paga electrónicamente desde BancaSAT.</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>Ley de Simplificación Tributaria (Decreto 7-2019) y Ley para la Integración del Sector Productivo Primario y Agropecuario (Decreto 31-2024).</t>
+          <t>Código Tributario (Decreto 6-91), Ley del IVA (Decreto 27-92) y Ley de Actualización Tributaria (Decreto 10-2012, Libros I y II).</t>
         </is>
       </c>
       <c r="H9" s="15" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" ht="50" customHeight="1">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
       <c r="A10" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="38" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C10" s="38" t="inlineStr">
+      <c r="C10" s="40" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
       </c>
       <c r="D10" s="35" t="inlineStr">
         <is>
-          <t>IVA General e Impuesto Sobre la Renta (ISR)</t>
+          <t>RTU Digital y Agencia Virtual</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Régimen aplicable a personas individuales y sociedades mercantiles con ingresos superiores a Q150,000 o afiliados voluntariamente al Régimen General del IVA (12%) y regímenes del ISR (Opcional Simplificado 5%/7% o Sobre Utilidades de Actividades Lucrativas 25%).</t>
+          <t>Plataforma digital de identidad tributaria y expediente electrónico del contribuyente para actualización obligatoria de datos de residencia, actividades económicas, establecimientos mercantiles, contadores, representantes legales y afiliaciones fiscales.</t>
         </is>
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>Declara y paga tu IVA mensual, liquida tus pagos trimestrales o retenciones de ISR, gestiona tu crédito fiscal y factura mediante FEL.</t>
+          <t>Actualiza tus datos en el RTU Digital, modifica tus actividades económicas y administra tus accesos en la Agencia Virtual.</t>
         </is>
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>Ley del IVA (Decreto 27-92), Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del Impuesto de Solidaridad (Decreto 73-2008).</t>
+          <t>Código Tributario (Decreto 6-91, Art. 120) y Acuerdo de Directorio SAT 08-2020 (RTU Digital obligatorio).</t>
         </is>
       </c>
       <c r="H10" s="22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" ht="50" customHeight="1">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" s="10" t="n">
         <v>5</v>
       </c>
@@ -2647,72 +3190,72 @@
       </c>
       <c r="C11" s="37" t="inlineStr">
         <is>
-          <t>Asalariados</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="D11" s="33" t="inlineStr">
         <is>
-          <t>Retenciones de ISR y Planilla del IVA</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Régimen tributario de rentas del trabajo en relación de dependencia aplicable a trabajadores contratados por patronos públicos o privados que perciben ingresos salariales sujetos a retención del ISR.</t>
+          <t>Registro Fiscal de Vehículos (RFV) que administra la propiedad, tenencia, modificaciones de características y el pago anual del Impuesto sobre Circulación de Vehículos (ISCV) para automotores terrestres, marítimos y aéreos.</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Consulta tus retenciones de ISR practicadas por tu patrono, ingresa tu planilla del IVA con facturas FEL y solicita devolución de retenciones en exceso.</t>
+          <t>Paga tu calcomanía ISCV, tramita primeras placas, realiza traspasos con notario y repón distintivos extraviados.</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>Ley de Actualización Tributaria (Decreto 10-2012, Arts. 68 al 82 - Rentas del Trabajo en Relación de Dependencia).</t>
+          <t>Ley del Impuesto sobre Circulación de Vehículos Terrestres, Marítimos y Aéreos (Decreto 70-94) y Código Tributario.</t>
         </is>
       </c>
       <c r="H11" s="15" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" ht="50" customHeight="1">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="D12" s="35" t="inlineStr">
         <is>
-          <t>Registro Fiscal de Vehículos (RFV)</t>
+          <t>Servicios al Contribuyente</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>Registro Fiscal de Vehículos (RFV) que administra el parque vehicular nacional, altas, bajas, modificaciones y el impuesto anual de circulación para propietarios y compradores de automotores terrestres, marítimos y aéreos.</t>
+          <t>Canales de atención presencial y remota, agendamiento de citas en oficinas tributarias del país, expedición de solvencias fiscales inmediatas y herramientas de consulta pública en registros de la SAT.</t>
         </is>
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
-          <t>Paga tu calcomanía anual de circulación (ISCV), tramita primeras placas, realiza traspasos vehiculares y repón distintivos extraviados.</t>
+          <t>Agenda tu cita en agencias tributarias, solicita tu solvencia fiscal con código QR y consulta el estado de tus gestiones.</t>
         </is>
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Ley del Impuesto sobre Circulación de Vehículos Terrestres, Marítimos y Aéreos (Decreto 70-94) y Código Tributario (Decreto 6-91).</t>
+          <t>Código Tributario (Decreto 6-91, Art. 57 "A") y Ley Orgánica de la SAT (Decreto 1-98).</t>
         </is>
       </c>
       <c r="H12" s="22" t="n">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" ht="50" customHeight="1">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="10" t="n">
         <v>7</v>
       </c>
@@ -2723,60 +3266,60 @@
       </c>
       <c r="C13" s="37" t="inlineStr">
         <is>
-          <t>Contribuyentes Especiales</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="D13" s="33" t="inlineStr">
         <is>
-          <t>Gerencias Especializadas de Fiscalización</t>
+          <t>Empresas y Sociedades</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Segmento de control fiscal diferenciado conformado por grandes y medianos contribuyentes calificados por resolución de la SAT en función de su representatividad en la recaudación, facturación y relevancia sectorial.</t>
+          <t>Personas jurídicas, sociedades anónimas, empresas mercantiles, sucursales extranjeras y contratos asociativos sujetos al cumplimiento de obligaciones societarias y mercantiles ante la administración tributaria.</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>Gestiona tus obligaciones en agencias especializadas, presenta estados financieros auditados y cumple con estudios de precios de transferencia.</t>
+          <t>Inscribe y actualiza representantes legales, habilita sucursales mercantiles y gestiona modificaciones societarias en el RTU.</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3) y Resoluciones de Directorio de Calificación de Contribuyentes Especiales.</t>
+          <t>Código de Comercio (Decreto 2-70), Código Tributario (Decreto 6-91) y Ley de Actualización Tributaria.</t>
         </is>
       </c>
       <c r="H13" s="15" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" ht="50" customHeight="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
       <c r="A14" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="38" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr">
+      <c r="C14" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyente General</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
         <is>
           <t>Facturación Electrónica</t>
         </is>
       </c>
-      <c r="D14" s="35" t="inlineStr">
-        <is>
-          <t>Sistema FEL y Agencia Virtual</t>
-        </is>
-      </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>Régimen obligatorio de emisión, transmisión y certificación de Documentos Tributarios Electrónicos (DTE) a través del sistema FEL y certificadores autorizados para todos los contribuyentes afiliados al régimen tributario nacional.</t>
+          <t>Régimen obligatorio de Factura Electrónica en Línea (FEL) para la emisión, anulación, transmisión y consulta de Documentos Tributarios Electrónicos (DTE) a través de Agencia Virtual o certificadores autorizados.</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>Habilítate como emisor de factura electrónica FEL, emite facturas gratuitas desde la Agencia Virtual y administra tus documentos emitidos y recibidos.</t>
+          <t>Habilítate como emisor FEL gratuito, autoriza tus formatos de documentos y administra tus comprobantes fiscales digitales.</t>
         </is>
       </c>
       <c r="G14" s="21" t="inlineStr">
@@ -2788,7 +3331,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" ht="50" customHeight="1">
+    <row r="15" ht="54" customHeight="1">
       <c r="A15" s="10" t="n">
         <v>9</v>
       </c>
@@ -2799,148 +3342,148 @@
       </c>
       <c r="C15" s="37" t="inlineStr">
         <is>
-          <t>Servicios al Contribuyente</t>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>Plataforma Digital, Citas y Solvencias</t>
+          <t>Solvencia y Convenios</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Plataforma de servicios transversales de atención ciudadana, autenticación digital, expedición de solvencias fiscales, agendamiento de citas presenciales y consultas públicas en bases de datos de la SAT.</t>
+          <t>Instrumentos de regularización fiscal, suscripción de convenios de pago por mora o determinación de oficio, facilidades crediticias y constancias de no adeudo tributario.</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>Crea o desbloquea tu Agencia Virtual, genera tu solvencia fiscal con código QR, agenda citas presenciales y consulta el estado de tus gestiones.</t>
+          <t>Solicita facilidades de pago en cuotas, suscribe convenios tributarios y obtén tu solvencia fiscal al regularizar tus saldos.</t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>Código Tributario (Decreto 6-91, Art. 57 "A" y Art. 120) y Acuerdos de Directorio de Servicios Electrónicos.</t>
+          <t>Código Tributario (Decreto 6-91, Arts. 40 y 57 "A") y Acuerdos de Directorio de Facilidades de Pago.</t>
         </is>
       </c>
       <c r="H15" s="15" t="n">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" ht="50" customHeight="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
       <c r="A16" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="C16" s="38" t="inlineStr">
-        <is>
-          <t>Importadores y Exportadores (Compartido)</t>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyentes</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>Contribuyente General</t>
         </is>
       </c>
       <c r="D16" s="35" t="inlineStr">
         <is>
-          <t>Gestiones Aduaneras Comunes y Arancel</t>
+          <t>Asalariados</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
         <is>
-          <t>Operadores comerciales que realizan indistintamente gestiones transversales de entrada y salida de mercancías, consultas arancelarias y pagos tributarios aduaneros en las aduanas de la República.</t>
+          <t>Trabajadores contratados por patronos públicos o privados afectos a retenciones mensuales de ISR, proyección anual de retención y presentación de la planilla del IVA por compras personales.</t>
         </is>
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Consulta el Arancel Integrado Centroamericano (SAC), realiza pagos por BancaSAT y tramita solvencias aduaneras unificadas.</t>
+          <t>Presenta tu planilla electrónica del IVA con comprobantes FEL y solicita devolución de retenciones de ISR en exceso.</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>Convenio sobre el Régimen Arancelario y Aduanero Centroamericano, CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA IV (Resolución 224-2008 COMIECO).</t>
+          <t>Ley de Actualización Tributaria (Decreto 10-2012, Arts. 68 al 82 - Rentas del Trabajo).</t>
         </is>
       </c>
       <c r="H16" s="22" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" ht="50" customHeight="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
       <c r="A17" s="10" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="37" t="inlineStr">
         <is>
-          <t>Operadores de Comercio Exterior</t>
+          <t>Contribuyentes</t>
         </is>
       </c>
       <c r="C17" s="37" t="inlineStr">
         <is>
-          <t>Importadores</t>
+          <t>Contribuyentes Especiales</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>Padrón de Importadores y DUCA-D</t>
+          <t>Contribuyentes Especiales</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Personas individuales o jurídicas autorizadas en el padrón aduanero de la SAT para introducir legalmente mercancías extranjeras al territorio aduanero nacional para su consumo, uso o transformación.</t>
+          <t>Empresas calificadas por resolución de la SAT como grandes o medianos contribuyentes especiales sujetas a esquemas intensivos de fiscalización, atención diferenciada y cumplimiento de precios de transferencia.</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Inscríbete en el padrón de importadores, liquida tus declaraciones aduaneras DUCA-D, consulta aranceles y rescata mercancías en aduana.</t>
+          <t>Gestiona tus obligaciones en gerencias especializadas, presenta estados financieros auditados y reporta precios de transferencia.</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Acuerdo Relativo a la Aplicación del Artículo VII del GATT (Valoración OMC).</t>
+          <t>Ley Orgánica de la SAT (Decreto 1-98, Art. 3) y Resoluciones de Directorio de Calificación de Contribuyentes Especiales.</t>
         </is>
       </c>
       <c r="H17" s="15" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="18" ht="50" customHeight="1">
+    <row r="18" ht="54" customHeight="1">
       <c r="A18" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="38" t="inlineStr">
+      <c r="B18" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C18" s="38" t="inlineStr">
-        <is>
-          <t>Exportadores</t>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>1. Importadores y Exportadores</t>
         </is>
       </c>
       <c r="D18" s="35" t="inlineStr">
         <is>
-          <t>Padrón de Exportadores y Devolución IVA</t>
+          <t>Importadores y Exportadores (Compartido)</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>Personas individuales o jurídicas inscritas en el Registro de Exportadores de la SAT que despachan mercancías de origen nacional o nacionalizadas hacia mercados del exterior.</t>
+          <t>Operadores comerciales que realizan indistintamente gestiones transversales de entrada y salida de mercancías, consultas arancelarias y pagos tributarios aduaneros en las aduanas de la República.</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>Registra tus exportaciones con código VUPE, emite facturas con régimen especial y gestiona la devolución de crédito fiscal del IVA.</t>
+          <t>Consulta el Arancel Integrado Centroamericano (SAC), realiza pagos por BancaSAT y tramita solvencias aduaneras unificadas.</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Ley de Fomento y Maquila (Decreto 29-89) y CAUCA/RECAUCA IV.</t>
+          <t>Convenio sobre el Régimen Arancelario y Aduanero Centroamericano, CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA IV (Resolución 224-2008 COMIECO).</t>
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" ht="50" customHeight="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="10" t="n">
         <v>13</v>
       </c>
@@ -2951,72 +3494,72 @@
       </c>
       <c r="C19" s="37" t="inlineStr">
         <is>
-          <t>Operador Económico Autorizado (OEA)</t>
+          <t>1. Importadores y Exportadores</t>
         </is>
       </c>
       <c r="D19" s="33" t="inlineStr">
         <is>
-          <t>Cadena Logística Segura y Carril Exprés</t>
+          <t>Importadores</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Operadores de la cadena logística internacional certificados por la Intendencia de Aduanas por mantener rigurosos estándares de seguridad y confiabilidad en sus operaciones transfronterizas.</t>
+          <t>Personas individuales o jurídicas autorizadas en el padrón aduanero de la SAT para introducir legalmente mercancías extranjeras al territorio aduanero nacional para su consumo, uso o transformación.</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Accede a carriles exprés preferenciales, prioridad en contingencias y despacho ágil con selectivo rojo reducido.</t>
+          <t>Inscríbete en el padrón de importadores, liquida tus declaraciones aduaneras DUCA-D, consulta aranceles y rescata mercancías en aduana.</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio de la SAT sobre el Programa OEA-Guatemala.</t>
+          <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Acuerdo Relativo a la Aplicación del Artículo VII del GATT (Valoración OMC).</t>
         </is>
       </c>
       <c r="H19" s="15" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" ht="50" customHeight="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="38" t="inlineStr">
+      <c r="B20" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C20" s="38" t="inlineStr">
-        <is>
-          <t>Agentes Aduaneros</t>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>1. Importadores y Exportadores</t>
         </is>
       </c>
       <c r="D20" s="35" t="inlineStr">
         <is>
-          <t>Despacho Aduanero Oficial y Representación</t>
+          <t>Exportadores</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
         <is>
-          <t>Profesionales auxiliares de la función pública aduanera autorizados para actuar por cuenta de terceros en los trámites y operaciones de desaduanamiento ante la SAT.</t>
+          <t>Personas individuales o jurídicas inscritas en el Registro de Exportadores de la SAT que despachan mercancías de origen nacional o nacionalizadas hacia mercados del exterior.</t>
         </is>
       </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
-          <t>Gestiona tu carné y habilitación oficial, presenta pólizas de seguro de caución y transmite declaraciones con firma electrónica.</t>
+          <t>Registra tus exportaciones con código VUPE, emite facturas con régimen especial y gestiona la devolución de crédito fiscal del IVA.</t>
         </is>
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>CAUCA IV (Arts. 22 al 28), RECAUCA IV (Arts. 74 al 85) y Ley Nacional de Aduanas.</t>
+          <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Ley de Fomento y Maquila (Decreto 29-89) y CAUCA/RECAUCA IV.</t>
         </is>
       </c>
       <c r="H20" s="22" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" ht="50" customHeight="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1">
       <c r="A21" s="10" t="n">
         <v>15</v>
       </c>
@@ -3027,72 +3570,72 @@
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
-          <t>Apoderados Especiales Aduaneros</t>
+          <t>1. Importadores y Exportadores</t>
         </is>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>Despacho Aduanero por Cuenta Propia</t>
+          <t>Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Personas individuales mandatarias designadas exclusivamente por una persona jurídica para representarla formalmente en sus despachos aduaneros propios.</t>
+          <t>Operadores de la cadena logística internacional certificados por la Intendencia de Aduanas por mantener rigurosos estándares de seguridad y confiabilidad en sus operaciones transfronterizas.</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Registra tu mandato legal, actualiza tu carné de apoderado y tramita declaraciones DUCA corporativas.</t>
+          <t>Accede a carriles exprés preferenciales, prioridad en contingencias y despacho ágil con selectivo rojo reducido.</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>CAUCA IV (Art. 21), RECAUCA IV (Arts. 86 al 90) y Código de Notariado.</t>
+          <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio de la SAT sobre el Programa OEA-Guatemala.</t>
         </is>
       </c>
       <c r="H21" s="15" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" ht="50" customHeight="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1">
       <c r="A22" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="38" t="inlineStr">
+      <c r="B22" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C22" s="38" t="inlineStr">
-        <is>
-          <t>Empresas de Entrega Rápida o Courier</t>
+      <c r="C22" s="40" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
       <c r="D22" s="35" t="inlineStr">
         <is>
-          <t>Paquetería Internacional y Franquicias</t>
+          <t>Depósitos Aduaneros</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>Empresas de mensajería y paquetería urgente autorizadas para transportar y desaduanar envíos postales exprés y encomiendas internacionales no comerciales.</t>
+          <t>Recintos públicos o privados autorizados para custodiar mercancías con suspensión de tributos aduaneros, emisión de certificados de depósito y bonos de prenda (AGD) y actas de recepción DAT.</t>
         </is>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
-          <t>Transmite manifiestos courier, aplica franquicias simplificadas y habilita recintos desconsolidadores de paquetería.</t>
+          <t>Controla inventarios de custodia, gestiona actas de recepción, emite certificados de depósito (AGD) y tramita prórrogas de permanencia.</t>
         </is>
       </c>
       <c r="G22" s="21" t="inlineStr">
         <is>
-          <t>CAUCA IV y RECAUCA IV (Arts. 574 al 596 - Régimen de Envíos de Entrega Rápida o Courier).</t>
+          <t>Decreto 1236 (Ley de Almacenes Generales de Depósito), CAUCA IV y RECAUCA IV (Arts. 119 al 129 - Régimen de Depósito Aduanero).</t>
         </is>
       </c>
       <c r="H22" s="22" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" ht="50" customHeight="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
       <c r="A23" s="10" t="n">
         <v>17</v>
       </c>
@@ -3103,72 +3646,72 @@
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
-          <t>Consolidadores y Desconsolidadores de Carga</t>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
-          <t>Manifiestos CUSCAR y Guías Hijas</t>
+          <t>Agentes Aduaneros</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Operadores logísticos autorizados para agrupar o separar mercancías pertenecientes a distintos consignatarios bajo un solo documento matriz de transporte.</t>
+          <t>Profesionales auxiliares de la función pública aduanera autorizados para actuar por cuenta de terceros en los trámites y operaciones de desaduanamiento ante la SAT.</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Transmite manifiestos CUSCAR, emite guías hijas y reporta inconsistencias o averías de carga ante la aduana.</t>
+          <t>Gestiona tu carné y habilitación oficial, presenta pólizas de seguro de caución y transmite declaraciones con firma electrónica.</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>CAUCA IV y RECAUCA IV (Arts. 102 al 109 - Auxiliares Consolidador y Desconsolidador de Carga).</t>
+          <t>CAUCA IV (Arts. 22 al 28), RECAUCA IV (Arts. 74 al 85) y Ley Nacional de Aduanas.</t>
         </is>
       </c>
       <c r="H23" s="15" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" ht="50" customHeight="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" ht="54" customHeight="1">
       <c r="A24" s="17" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="38" t="inlineStr">
+      <c r="B24" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C24" s="38" t="inlineStr">
-        <is>
-          <t>Transportistas Aduaneros</t>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
       <c r="D24" s="35" t="inlineStr">
         <is>
-          <t>Tránsito Aduanero Internacional y Marchamo</t>
+          <t>Apoderados Especiales Aduaneros</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>Empresas y conductores autorizados para realizar el traslado de mercancías bajo control aduanero dentro del territorio nacional o en tránsito internacional centroamericano.</t>
+          <t>Personas individuales mandatarias designadas exclusivamente por una persona jurídica para representarla formalmente en sus despachos aduaneros propios.</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
-          <t>Registra medios de transporte, activa marchamos electrónicos RFID y transmite declaraciones de tránsito DUCA-T.</t>
+          <t>Registra tu mandato legal, actualiza tu carné de apoderado y tramita declaraciones DUCA corporativas.</t>
         </is>
       </c>
       <c r="G24" s="21" t="inlineStr">
         <is>
-          <t>CAUCA IV (Arts. 18 al 20), RECAUCA IV (Tránsito Aduanero Internacional Terrestre) y Reglamentos de Transporte Centroamericano.</t>
+          <t>CAUCA IV (Art. 21), RECAUCA IV (Arts. 86 al 90) y Código de Notariado.</t>
         </is>
       </c>
       <c r="H24" s="22" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="25" ht="50" customHeight="1">
+    <row r="25" ht="54" customHeight="1">
       <c r="A25" s="10" t="n">
         <v>19</v>
       </c>
@@ -3179,72 +3722,72 @@
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
-          <t>Depósitos Aduaneros</t>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
-          <t>Custodia de Mercancías y Títulos de Crédito</t>
+          <t>Transportistas Aduaneros</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Recintos públicos o privados (Almacenes Fiscales, Almacenes Generales de Depósito y Depósitos Aduaneros Temporales DAT) autorizados para custodiar mercancías con suspensión de tributos aduaneros.</t>
+          <t>Empresas y conductores autorizados para realizar el traslado de mercancías bajo control aduanero dentro del territorio nacional o en tránsito internacional centroamericano.</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Controla inventarios de custodia, gestiona actas de recepción, emite certificados de depósito (AGD) y tramita prórrogas de permanencia.</t>
+          <t>Registra medios de transporte, activa marchamos electrónicos RFID y transmite declaraciones de tránsito DUCA-T.</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>Decreto 1236 (Ley de Almacenes Generales de Depósito), CAUCA IV y RECAUCA IV (Arts. 119 al 129 - Régimen de Depósito Aduanero).</t>
+          <t>CAUCA IV (Arts. 18 al 20), RECAUCA IV (Tránsito Aduanero Internacional Terrestre) y Reglamentos de Transporte Centroamericano.</t>
         </is>
       </c>
       <c r="H25" s="15" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" ht="50" customHeight="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
       <c r="A26" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="38" t="inlineStr">
+      <c r="B26" s="40" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C26" s="38" t="inlineStr">
-        <is>
-          <t>ZDEEP - Entidades Administradoras</t>
+      <c r="C26" s="40" t="inlineStr">
+        <is>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
       <c r="D26" s="35" t="inlineStr">
         <is>
-          <t>Administración de Zonas Especiales Públicas</t>
+          <t>Empresas de Entrega Rápida o Courier</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>Personas jurídicas públicas o privadas autorizadas por ZOLIC y SAT para desarrollar, operar y vigilar la infraestructura de polígonos industriales y logísticos ZDEEP.</t>
+          <t>Empresas de mensajería y paquetería urgente autorizadas para transportar y desaduanar envíos postales exprés y encomiendas internacionales no comerciales.</t>
         </is>
       </c>
       <c r="F26" s="20" t="inlineStr">
         <is>
-          <t>Delimita polígonos aduaneros, administra garitas de control y supervisa el perímetro de seguridad de la zona especial.</t>
+          <t>Transmite manifiestos courier, aplica franquicias simplificadas y habilita recintos desconsolidadores de paquetería.</t>
         </is>
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>Decreto 22-73 (Ley Orgánica de ZOLIC reformada), CAUCA IV, RECAUCA IV y Resoluciones Conjuntas SAT-ZOLIC.</t>
+          <t>CAUCA IV y RECAUCA IV (Arts. 574 al 596 - Régimen de Envíos de Entrega Rápida o Courier).</t>
         </is>
       </c>
       <c r="H26" s="22" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" ht="50" customHeight="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1">
       <c r="A27" s="10" t="n">
         <v>21</v>
       </c>
@@ -3255,148 +3798,148 @@
       </c>
       <c r="C27" s="37" t="inlineStr">
         <is>
-          <t>ZDEEP - Empresas Usuarias</t>
+          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>Transformación, Servicios y Exenciones</t>
+          <t>Consolidadores y Desconsolidadores de Carga</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Empresas industriales, comerciales o de servicios instaladas y operando dentro de los recintos calificados como ZDEEP para producir o transformar con beneficios fiscales.</t>
+          <t>Operadores logísticos autorizados para agrupar o separar mercancías pertenecientes a distintos consignatarios bajo un solo documento matriz de transporte.</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
-          <t>Ingresa materias primas con suspensión de DAI e IVA, realiza descargos de producción y goza de exenciones tributarias.</t>
+          <t>Transmite manifiestos CUSCAR, emite guías hijas y reporta inconsistencias o averías de carga ante la aduana.</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>Decreto 22-73 (Régimen Fiscal ZDEEP), Ley de Actualización Tributaria (Decreto 10-2012) y CAUCA/RECAUCA IV.</t>
+          <t>CAUCA IV y RECAUCA IV (Arts. 102 al 109 - Auxiliares Consolidador y Desconsolidador de Carga).</t>
         </is>
       </c>
       <c r="H27" s="15" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="28" ht="50" customHeight="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" ht="54" customHeight="1">
       <c r="A28" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="B28" s="38" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="C28" s="38" t="inlineStr">
-        <is>
-          <t>Abogados y Notarios</t>
+      <c r="B28" s="40" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior</t>
+        </is>
+      </c>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>3. Regímenes Territoriales y Zonas Especiales</t>
         </is>
       </c>
       <c r="D28" s="35" t="inlineStr">
         <is>
-          <t>Papel Sellado de Protocolo y Avisos</t>
+          <t>ZDEEP - Entidades Administradoras</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>Profesionales del derecho colegiados activos autorizados para ejercer la fe pública notarial, redactar instrumentos públicos y autorizar traspasos electrónicos de vehículos ante la SAT.</t>
+          <t>Personas jurídicas públicas o privadas autorizadas por ZOLIC y SAT para desarrollar, operar y vigilar la infraestructura de polígonos industriales y logísticos ZDEEP.</t>
         </is>
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Compra papel sellado especial para protocolos, adquiere timbres fiscales, realiza traspasos vehiculares electrónicos (TEV) y presenta avisos notariales.</t>
+          <t>Delimita polígonos aduaneros, administra garitas de control y supervisa el perímetro de seguridad de la zona especial.</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
         <is>
-          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales y de Papel Sellado Especial para Protocolos (Decreto 37-92) y Código Tributario.</t>
+          <t>Decreto 22-73 (Ley Orgánica de ZOLIC reformada), CAUCA IV, RECAUCA IV y Resoluciones Conjuntas SAT-ZOLIC.</t>
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" ht="50" customHeight="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" ht="54" customHeight="1">
       <c r="A29" s="10" t="n">
         <v>23</v>
       </c>
       <c r="B29" s="37" t="inlineStr">
         <is>
-          <t>Profesionales</t>
+          <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
       <c r="C29" s="37" t="inlineStr">
         <is>
-          <t>Peritos Contadores</t>
+          <t>3. Regímenes Territoriales y Zonas Especiales</t>
         </is>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
-          <t>Libros Contables y Declaraciones</t>
+          <t>ZDEEP - Empresas Usuarias</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Técnicos y profesionales contables inscritos y autorizados ante la SAT para llevar y firmar registros contables de contribuyentes, certificar estados financieros y realizar gestiones tributarias.</t>
+          <t>Empresas industriales, comerciales o de servicios instaladas y operando dentro de los recintos calificados como ZDEEP para producir o transformar con beneficios fiscales.</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Inscríbete y actualiza tus datos en el Registro de Contadores, autoriza libros contables computarizados y asocia contribuyentes a tu perfil.</t>
+          <t>Ingresa materias primas con suspensión de DAI e IVA, realiza descargos de producción y goza de exenciones tributarias.</t>
         </is>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>Decreto 2450 (Normas que Regulan el Ejercicio de la Profesión de Contador), Código de Comercio (Decreto 2-70) y Código Tributario (Arts. 112 y 120).</t>
+          <t>Decreto 22-73 (Régimen Fiscal ZDEEP), Ley de Actualización Tributaria (Decreto 10-2012) y CAUCA/RECAUCA IV.</t>
         </is>
       </c>
       <c r="H29" s="15" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" ht="50" customHeight="1">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" ht="54" customHeight="1">
       <c r="A30" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="B30" s="38" t="inlineStr">
+      <c r="B30" s="40" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C30" s="38" t="inlineStr">
-        <is>
-          <t>Auditores</t>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
         </is>
       </c>
       <c r="D30" s="35" t="inlineStr">
         <is>
-          <t>Dictámenes Tributarios y Devolución IVA</t>
+          <t>Abogados y Notarios</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>Contadores Públicos y Auditores (CPA) colegiados activos y firmas de auditoría facultados para emitir dictámenes sobre estados financieros, devolución de crédito fiscal e informes de precios de transferencia.</t>
+          <t>Profesionales del derecho colegiados activos autorizados para ejercer la fe pública notarial, redactar instrumentos públicos y autorizar traspasos electrónicos de vehículos ante la SAT.</t>
         </is>
       </c>
       <c r="F30" s="20" t="inlineStr">
         <is>
-          <t>Emite dictámenes de crédito fiscal para exportadores, dictámenes de estados financieros para licitaciones y presenta informes tributarios requeridos por SAT.</t>
+          <t>Compra papel sellado especial para protocolos, adquiere timbres fiscales, realiza traspasos vehiculares electrónicos (TEV) y presenta avisos notariales.</t>
         </is>
       </c>
       <c r="G30" s="21" t="inlineStr">
         <is>
-          <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001), Ley del IVA (Decreto 27-92, Art. 23 bis) y Ley de Actualización Tributaria (Decreto 10-2012).</t>
+          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales y de Papel Sellado Especial para Protocolos (Decreto 37-92) y Código Tributario.</t>
         </is>
       </c>
       <c r="H30" s="22" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" ht="50" customHeight="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" ht="54" customHeight="1">
       <c r="A31" s="10" t="n">
         <v>25</v>
       </c>
@@ -3407,148 +3950,148 @@
       </c>
       <c r="C31" s="37" t="inlineStr">
         <is>
-          <t>Gestores Tributarios</t>
+          <t>Servicios Profesionales y Terceras Personas</t>
         </is>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
-          <t>Gafetes y Trámites Presenciales</t>
+          <t>Peritos Contadores</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Personas individuales autorizadas y acreditadas formalmente ante la SAT para representar a terceros en la tramitación presencial de gestiones administrativas tributarias y aduaneras.</t>
+          <t>Técnicos y profesionales contables inscritos y autorizados ante la SAT para llevar y firmar registros contables de contribuyentes, certificar estados financieros y realizar gestiones tributarias.</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>Tramita y renueva tu carné oficial de gestor tributario, registra tus datos biométricos y gestiona expedientes autorizados en agencias tributarias.</t>
+          <t>Inscríbete y actualiza tus datos en el Registro de Contadores, autoriza libros contables computarizados y asocia contribuyentes a tu perfil.</t>
         </is>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>Acuerdos de Directorio de la SAT sobre Regulación y Acreditación de Gestores Tributarios y Código Tributario.</t>
+          <t>Decreto 2450 (Normas que Regulan el Ejercicio de la Profesión de Contador), Código de Comercio (Decreto 2-70) y Código Tributario (Arts. 112 y 120).</t>
         </is>
       </c>
       <c r="H31" s="15" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" ht="50" customHeight="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
       <c r="A32" s="17" t="n">
         <v>26</v>
       </c>
-      <c r="B32" s="38" t="inlineStr">
+      <c r="B32" s="40" t="inlineStr">
         <is>
           <t>Profesionales</t>
         </is>
       </c>
-      <c r="C32" s="38" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales</t>
+      <c r="C32" s="40" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
         </is>
       </c>
       <c r="D32" s="35" t="inlineStr">
         <is>
-          <t>Facturación por Honorarios y Retenciones</t>
+          <t>Gestores Tributarios</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de consultoría por honorarios profesionales.</t>
+          <t>Personas individuales autorizadas y acreditadas formalmente ante la SAT para representar a terceros en la tramitación presencial de gestiones administrativas tributarias y aduaneras.</t>
         </is>
       </c>
       <c r="F32" s="20" t="inlineStr">
         <is>
-          <t>Emite facturas electrónicas FEL por honorarios, liquida retenciones de ISR, actualiza tu colegiado activo y consulta tu solvencia fiscal.</t>
+          <t>Tramita y renueva tu carné oficial de gestor tributario, registra tus datos biométricos y gestiona expedientes autorizados en agencias tributarias.</t>
         </is>
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
-          <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del IVA (Decreto 27-92).</t>
+          <t>Acuerdos de Directorio de la SAT sobre Regulación y Acreditación de Gestores Tributarios y Código Tributario.</t>
         </is>
       </c>
       <c r="H32" s="22" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" ht="50" customHeight="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" ht="54" customHeight="1">
       <c r="A33" s="10" t="n">
         <v>27</v>
       </c>
       <c r="B33" s="37" t="inlineStr">
         <is>
-          <t>Entes Exentos</t>
+          <t>Profesionales</t>
         </is>
       </c>
       <c r="C33" s="37" t="inlineStr">
         <is>
-          <t>Constitucionales</t>
+          <t>Servicios Profesionales y Terceras Personas</t>
         </is>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
-          <t>Exenciones Tributarias de Rango Constitucional</t>
+          <t>Servicios Profesionales</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Instituciones educativas, universidades, comunidades religiosas, misiones diplomáticas y cuerpos consulares que gozan de exención de impuestos por mandato directo de la Carta Magna.</t>
+          <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de consultoría por honorarios profesionales.</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr">
         <is>
-          <t>Inscribe tu personería jurídica exenta en el RTU, emite constancias electrónicas de exención de IVA y timbres, y acredita representación legal.</t>
+          <t>Emite facturas electrónicas FEL por honorarios, liquida retenciones de ISR, actualiza tu colegiado activo y consulta tu solvencia fiscal.</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>Constitución Política de la República de Guatemala (Arts. 37, 73, 88), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
+          <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del IVA (Decreto 27-92).</t>
         </is>
       </c>
       <c r="H33" s="15" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="34" ht="50" customHeight="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" ht="54" customHeight="1">
       <c r="A34" s="17" t="n">
         <v>28</v>
       </c>
-      <c r="B34" s="38" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="C34" s="38" t="inlineStr">
-        <is>
-          <t>No Lucrativos</t>
+      <c r="B34" s="40" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Terceras Personas</t>
         </is>
       </c>
       <c r="D34" s="35" t="inlineStr">
         <is>
-          <t>Reconocimiento de Exención de ISR e IVA</t>
+          <t>Auditores</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas, asociaciones civiles sin fines de lucro y cooperativas que solicitan reconocimiento administrativo de exención de ISR e IVA.</t>
+          <t>Contadores Públicos y Auditores (CPA) colegiados activos y firmas de auditoría facultados para emitir dictámenes sobre estados financieros, devolución de crédito fiscal e informes de precios de transferencia.</t>
         </is>
       </c>
       <c r="F34" s="20" t="inlineStr">
         <is>
-          <t>Solicita tu resolución formal de exención de ISR, actualiza estatutos y junta directiva en el RTU y emite constancias de retención y exención.</t>
+          <t>Emite dictámenes de crédito fiscal para exportadores, dictámenes de estados financieros para licitaciones y presenta informes tributarios requeridos por SAT.</t>
         </is>
       </c>
       <c r="G34" s="21" t="inlineStr">
         <is>
-          <t>Decreto 02-2003 (Ley de ONGs para el Desarrollo), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
+          <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001), Ley del IVA (Decreto 27-92, Art. 23 bis) y Ley de Actualización Tributaria (Decreto 10-2012).</t>
         </is>
       </c>
       <c r="H34" s="22" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" ht="50" customHeight="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" ht="54" customHeight="1">
       <c r="A35" s="10" t="n">
         <v>29</v>
       </c>
@@ -3559,72 +4102,72 @@
       </c>
       <c r="C35" s="37" t="inlineStr">
         <is>
-          <t>Municipalidades</t>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
-          <t>Autonomía Municipal y Régimen Exento</t>
+          <t>Constitucionales</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>Las 340 corporaciones municipales autónomas de la República de Guatemala, mancomunidades y empresas municipales públicas prestadoras de servicios comunitarios.</t>
+          <t>Instituciones educativas, universidades, comunidades religiosas, misiones diplomáticas y cuerpos consulares que gozan de exención de impuestos por mandato directo de la Carta Magna.</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Registra autoridades y tesoreros en el RTU, gestiona la exención del impuesto de circulación para flotillas municipales y tramita solvencias institucionales.</t>
+          <t>Inscribe tu personería jurídica exenta en el RTU, emite constancias electrónicas de exención de IVA y timbres, y acredita representación legal.</t>
         </is>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>Constitución Política de la República (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
+          <t>Constitución Política de la República de Guatemala (Arts. 37, 73, 88), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
         </is>
       </c>
       <c r="H35" s="15" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" ht="50" customHeight="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" ht="54" customHeight="1">
       <c r="A36" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="B36" s="38" t="inlineStr">
+      <c r="B36" s="40" t="inlineStr">
         <is>
           <t>Entes Exentos</t>
         </is>
       </c>
-      <c r="C36" s="38" t="inlineStr">
-        <is>
-          <t>Entidades del Estado</t>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="D36" s="35" t="inlineStr">
         <is>
-          <t>Compras Públicas y Agentes de Retención</t>
+          <t>Decreto</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>Ministerios de Estado, secretarías, organismos de los poderes Ejecutivo, Legislativo y Judicial, y entidades públicas descentralizadas que operan como agentes de retención del IVA e ISR.</t>
+          <t>Personas o entidades beneficiarias de leyes de fomento económico y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso.</t>
         </is>
       </c>
       <c r="F36" s="20" t="inlineStr">
         <is>
-          <t>Habilita unidades ejecutoras en el RTU, emite constancias de retención en compras públicas y administra el parque vehicular oficial del Estado.</t>
+          <t>Acredita resoluciones ministeriales de calificación de fomento, gestiona exenciones arancelarias temporales y presenta reportes periódicos de cumplimiento.</t>
         </is>
       </c>
       <c r="G36" s="21" t="inlineStr">
         <is>
-          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
+          <t>Decretos específicos de fomento (Decreto 29-89 de Maquilas, Decreto 65-89 de Zonas Francas, Ley de Incentivos para Energías Renovables) y Código Tributario.</t>
         </is>
       </c>
       <c r="H36" s="22" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="37" ht="50" customHeight="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" ht="54" customHeight="1">
       <c r="A37" s="10" t="n">
         <v>31</v>
       </c>
@@ -3635,35 +4178,140 @@
       </c>
       <c r="C37" s="37" t="inlineStr">
         <is>
-          <t>Decreto</t>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="D37" s="33" t="inlineStr">
         <is>
-          <t>Exenciones y Fomento por Decreto Legislativo</t>
+          <t>No Lucrativos</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Personas o entidades beneficiarias de leyes de fomento económico y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso.</t>
+          <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas, asociaciones civiles sin fines de lucro y cooperativas que solicitan reconocimiento administrativo de exención de ISR e IVA.</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>Acredita resoluciones ministeriales de calificación de fomento, gestiona exenciones arancelarias temporales y presenta reportes periódicos de cumplimiento.</t>
+          <t>Solicita tu resolución formal de exención de ISR, actualiza estatutos y junta directiva en el RTU y emite constancias de retención y exención.</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>Decretos específicos de fomento (Decreto 29-89 de Maquilas, Decreto 65-89 de Zonas Francas, Ley de Incentivos para Energías Renovables) y Código Tributario.</t>
+          <t>Decreto 02-2003 (Ley de ONGs para el Desarrollo), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
         </is>
       </c>
       <c r="H37" s="15" t="n">
-        <v>16</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" ht="54" customHeight="1">
+      <c r="A38" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="B38" s="40" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="inlineStr">
+        <is>
+          <t>Entidades del Estado</t>
+        </is>
+      </c>
+      <c r="E38" s="19" t="inlineStr">
+        <is>
+          <t>Ministerios de Estado, secretarías, organismos de los poderes Ejecutivo, Legislativo y Judicial, y entidades públicas descentralizadas que operan como agentes de retención del IVA e ISR.</t>
+        </is>
+      </c>
+      <c r="F38" s="20" t="inlineStr">
+        <is>
+          <t>Habilita unidades ejecutoras en el RTU, emite constancias de retención en compras públicas y administra el parque vehicular oficial del Estado.</t>
+        </is>
+      </c>
+      <c r="G38" s="21" t="inlineStr">
+        <is>
+          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
+        </is>
+      </c>
+      <c r="H38" s="22" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" ht="54" customHeight="1">
+      <c r="A39" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B39" s="37" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="C39" s="37" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
+        </is>
+      </c>
+      <c r="D39" s="33" t="inlineStr">
+        <is>
+          <t>Municipalidades</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>Las 340 corporaciones municipales autónomas de la República de Guatemala, mancomunidades y empresas municipales públicas prestadoras de servicios comunitarios.</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Registra autoridades y tesoreros en el RTU, gestiona la exención del impuesto de circulación para flotillas municipales y tramita solvencias institucionales.</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>Constitución Política de la República (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="48" t="inlineStr"/>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>TOTAL PORTAL WEB SAT</t>
+        </is>
+      </c>
+      <c r="C40" s="50" t="inlineStr">
+        <is>
+          <t>4 Segmentos Oficiales</t>
+        </is>
+      </c>
+      <c r="D40" s="50" t="inlineStr">
+        <is>
+          <t>33 Categorías</t>
+        </is>
+      </c>
+      <c r="E40" s="50" t="inlineStr">
+        <is>
+          <t>100% de la arquitectura de información clasificada</t>
+        </is>
+      </c>
+      <c r="F40" s="48" t="inlineStr"/>
+      <c r="G40" s="48" t="inlineStr"/>
+      <c r="H40" s="53">
+        <f>SUM(H7:H39)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:H37"/>
+  <autoFilter ref="A6:H39"/>
   <mergeCells count="2">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A2:H3"/>

</xml_diff>

<commit_message>
fix(taxonomy): estandarizar textos de macrogrupos a estandar ATO de 1 sola linea en excel y frontend
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -867,7 +867,7 @@
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Gestiona tus trámites aduaneros, consulta requisitos y haz seguimiento a tus operaciones según tu rol en la cadena logística.</t>
+          <t>Servicios e información aduanera para la importación, exportación y logística.</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Cumple con tus obligaciones tributarias, emite tus facturas, actualiza tu RTU y gestiona tus trámites de vehículos e impuestos internos de forma ágil y 100% digital.</t>
+          <t>Información y servicios tributarios para personas y empresas.</t>
         </is>
       </c>
       <c r="F12" s="21" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Accede a herramientas especializadas de fe pública, autorización de libros contables, presentación de dictámenes fiscales y gestión de trámites profesionales.</t>
+          <t>Herramientas y servicios especializados para profesionales tributarios y auxiliares.</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Solicita y gestiona tus resoluciones de exención, emite constancias tributarias electrónicas y administra las obligaciones formales de tu entidad.</t>
+          <t>Información y gestiones tributarias para entidades públicas y organizaciones no lucrativas.</t>
         </is>
       </c>
       <c r="F14" s="21" t="inlineStr">

</xml_diff>

<commit_message>
fix(etl): depurar universo de contribuyentes de 413 a 344 tramites canonicos y reubicar contenidos cruzados
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -778,25 +778,25 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>TOTAL CONTENIDOS
-739 Trámites</t>
+676 Trámites</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>CONTRIBUYENTES
-413 Trámites</t>
+344 Trámites</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>COMERCIO EXTERIOR
-202 Trámites</t>
+204 Trámites</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
           <t>PROFESIONALES
-45 Trámites</t>
+49 Trámites</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H11" s="16">
         <f>G11/$G$15</f>
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="G12" s="22" t="n">
-        <v>413</v>
+        <v>344</v>
       </c>
       <c r="H12" s="23">
         <f>G12/$G$15</f>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="G13" s="15" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="H13" s="16">
         <f>G13/$G$15</f>
@@ -1049,7 +1049,7 @@
       <c r="E19" s="33" t="n"/>
       <c r="F19" s="33" t="n"/>
       <c r="G19" s="15" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H19" s="16">
         <f>G19/$G$24</f>
@@ -1071,7 +1071,7 @@
       <c r="E20" s="35" t="n"/>
       <c r="F20" s="35" t="n"/>
       <c r="G20" s="22" t="n">
-        <v>260</v>
+        <v>221</v>
       </c>
       <c r="H20" s="23">
         <f>G20/$G$24</f>
@@ -1093,7 +1093,7 @@
       <c r="E21" s="33" t="n"/>
       <c r="F21" s="33" t="n"/>
       <c r="G21" s="15" t="n">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="H21" s="16">
         <f>G21/$G$24</f>
@@ -1115,7 +1115,7 @@
       <c r="E22" s="35" t="n"/>
       <c r="F22" s="35" t="n"/>
       <c r="G22" s="22" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H22" s="23">
         <f>G22/$G$24</f>
@@ -1137,7 +1137,7 @@
       <c r="E23" s="33" t="n"/>
       <c r="F23" s="33" t="n"/>
       <c r="G23" s="15" t="n">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="H23" s="16">
         <f>G23/$G$24</f>
@@ -1214,7 +1214,7 @@
       <c r="E28" s="35" t="n"/>
       <c r="F28" s="35" t="n"/>
       <c r="G28" s="22" t="n">
-        <v>462</v>
+        <v>419</v>
       </c>
       <c r="H28" s="23">
         <f>G28/$G$32</f>
@@ -1236,7 +1236,7 @@
       <c r="E29" s="33" t="n"/>
       <c r="F29" s="33" t="n"/>
       <c r="G29" s="15" t="n">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="H29" s="16">
         <f>G29/$G$32</f>
@@ -1258,7 +1258,7 @@
       <c r="E30" s="35" t="n"/>
       <c r="F30" s="35" t="n"/>
       <c r="G30" s="22" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H30" s="23">
         <f>G30/$G$32</f>
@@ -1280,7 +1280,7 @@
       <c r="E31" s="33" t="n"/>
       <c r="F31" s="33" t="n"/>
       <c r="G31" s="15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H31" s="16">
         <f>G31/$G$32</f>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="G7" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H7" s="39">
         <f>G7/$G$18</f>
@@ -1526,7 +1526,7 @@
         </is>
       </c>
       <c r="G9" s="15" t="n">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="H9" s="39">
         <f>G9/$G$18</f>
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="G10" s="22" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="H10" s="42">
         <f>G10/$G$18</f>
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="H11" s="39">
         <f>G11/$G$18</f>
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="G12" s="22" t="n">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="H12" s="42">
         <f>G12/$G$18</f>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="G13" s="15" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H13" s="39">
         <f>G13/$G$18</f>
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="G14" s="22" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H14" s="42">
         <f>G14/$G$18</f>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H15" s="39">
         <f>G15/$G$18</f>
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="G16" s="22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H16" s="42">
         <f>G16/$G$18</f>
@@ -1854,7 +1854,7 @@
         </is>
       </c>
       <c r="G17" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H17" s="39">
         <f>G17/$G$18</f>
@@ -1928,7 +1928,7 @@
         </is>
       </c>
       <c r="G19" s="15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H19" s="39">
         <f>G19/$G$31</f>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="G32" s="22" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H32" s="42">
         <f>G32/$G$37</f>
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="G35" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H35" s="39">
         <f>G35/$G$37</f>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="J44" s="49" t="inlineStr">
         <is>
-          <t>739 Trámites 100% Mapeados</t>
+          <t>676 Trámites 100% Mapeados</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="H7" s="15" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="54" customHeight="1">
@@ -3138,7 +3138,7 @@
         </is>
       </c>
       <c r="H9" s="15" t="n">
-        <v>87</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" ht="54" customHeight="1">
@@ -3176,7 +3176,7 @@
         </is>
       </c>
       <c r="H10" s="22" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" ht="54" customHeight="1">
@@ -3214,7 +3214,7 @@
         </is>
       </c>
       <c r="H11" s="15" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" ht="54" customHeight="1">
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="H12" s="22" t="n">
-        <v>67</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" ht="54" customHeight="1">
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="H13" s="15" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" ht="54" customHeight="1">
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="H14" s="22" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" ht="54" customHeight="1">
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="H15" s="15" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" ht="54" customHeight="1">
@@ -3404,7 +3404,7 @@
         </is>
       </c>
       <c r="H16" s="22" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1">
@@ -3442,7 +3442,7 @@
         </is>
       </c>
       <c r="H17" s="15" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" ht="54" customHeight="1">
@@ -3480,7 +3480,7 @@
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" ht="54" customHeight="1">
@@ -3936,7 +3936,7 @@
         </is>
       </c>
       <c r="H30" s="22" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" ht="54" customHeight="1">
@@ -4050,7 +4050,7 @@
         </is>
       </c>
       <c r="H33" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" ht="54" customHeight="1">

</xml_diff>

<commit_message>
feat(taxonomy): incorporar textos oficiales ATO para los 4 regimenes de Contribuyentes en excel y frontend
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -3053,7 +3053,7 @@
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Inscribe tu primer NIT en línea, actualiza tus datos de residencia y obtén tu solvencia fiscal sin acudir a una agencia.</t>
+          <t>Gestiones y servicios de identificación tributaria para personas sin actividad comercial.</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
-          <t>Emite tus facturas FEL de pequeño contribuyente, declara el 5% mensual en Declaraguate y consulta tus libros digitales.</t>
+          <t>Información y obligaciones para pequeños negocios y régimen simplificado.</t>
         </is>
       </c>
       <c r="G8" s="21" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Gestiona tus obligaciones en gerencias especializadas, presenta estados financieros auditados y reporta precios de transferencia.</t>
+          <t>Servicios y gestiones tributarias para empresas con atención diferenciada.</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(comercio-exterior): consolidar 6 ramas canonicas, actualizar entregables vivos y registrar skill de auditoria IA
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -778,7 +778,7 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>TOTAL CONTENIDOS
-676 Trámites</t>
+718 Trámites</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -790,7 +790,7 @@
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>COMERCIO EXTERIOR
-204 Trámites</t>
+246 Trámites</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="G11" s="15" t="n">
-        <v>204</v>
+        <v>246</v>
       </c>
       <c r="H11" s="16">
         <f>G11/$G$15</f>
@@ -1049,7 +1049,7 @@
       <c r="E19" s="33" t="n"/>
       <c r="F19" s="33" t="n"/>
       <c r="G19" s="15" t="n">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="H19" s="16">
         <f>G19/$G$24</f>
@@ -1071,7 +1071,7 @@
       <c r="E20" s="35" t="n"/>
       <c r="F20" s="35" t="n"/>
       <c r="G20" s="22" t="n">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="H20" s="23">
         <f>G20/$G$24</f>
@@ -1093,7 +1093,7 @@
       <c r="E21" s="33" t="n"/>
       <c r="F21" s="33" t="n"/>
       <c r="G21" s="15" t="n">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="H21" s="16">
         <f>G21/$G$24</f>
@@ -1115,7 +1115,7 @@
       <c r="E22" s="35" t="n"/>
       <c r="F22" s="35" t="n"/>
       <c r="G22" s="22" t="n">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="H22" s="23">
         <f>G22/$G$24</f>
@@ -1137,7 +1137,7 @@
       <c r="E23" s="33" t="n"/>
       <c r="F23" s="33" t="n"/>
       <c r="G23" s="15" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H23" s="16">
         <f>G23/$G$24</f>
@@ -1214,7 +1214,7 @@
       <c r="E28" s="35" t="n"/>
       <c r="F28" s="35" t="n"/>
       <c r="G28" s="22" t="n">
-        <v>419</v>
+        <v>497</v>
       </c>
       <c r="H28" s="23">
         <f>G28/$G$32</f>
@@ -1236,7 +1236,7 @@
       <c r="E29" s="33" t="n"/>
       <c r="F29" s="33" t="n"/>
       <c r="G29" s="15" t="n">
-        <v>173</v>
+        <v>128</v>
       </c>
       <c r="H29" s="16">
         <f>G29/$G$32</f>
@@ -1258,7 +1258,7 @@
       <c r="E30" s="35" t="n"/>
       <c r="F30" s="35" t="n"/>
       <c r="G30" s="22" t="n">
-        <v>78</v>
+        <v>35</v>
       </c>
       <c r="H30" s="23">
         <f>G30/$G$32</f>
@@ -1280,7 +1280,7 @@
       <c r="E31" s="33" t="n"/>
       <c r="F31" s="33" t="n"/>
       <c r="G31" s="15" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H31" s="16">
         <f>G31/$G$32</f>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="J6" s="9" t="inlineStr">
         <is>
-          <t>Ruta Canónica de Navegación (Miga de Pan)</t>
+          <t>Ruta oficial de Navegación (Miga de Pan)</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
         </is>
       </c>
       <c r="G19" s="15" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H19" s="39">
         <f>G19/$G$31</f>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="G20" s="22" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="H20" s="42">
         <f>G20/$G$31</f>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="G21" s="15" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H21" s="39">
         <f>G21/$G$31</f>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="G22" s="22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H22" s="42">
         <f>G22/$G$31</f>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="G23" s="15" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H23" s="39">
         <f>G23/$G$31</f>
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="G24" s="22" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H24" s="42">
         <f>G24/$G$31</f>
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="G25" s="15" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H25" s="39">
         <f>G25/$G$31</f>
@@ -2215,7 +2215,7 @@
         </is>
       </c>
       <c r="G26" s="22" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H26" s="42">
         <f>G26/$G$31</f>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="G27" s="15" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H27" s="39">
         <f>G27/$G$31</f>
@@ -2297,7 +2297,7 @@
         </is>
       </c>
       <c r="G28" s="22" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H28" s="42">
         <f>G28/$G$31</f>
@@ -2338,7 +2338,7 @@
         </is>
       </c>
       <c r="G29" s="15" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H29" s="39">
         <f>G29/$G$31</f>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="G30" s="22" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H30" s="42">
         <f>G30/$G$31</f>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="J44" s="49" t="inlineStr">
         <is>
-          <t>676 Trámites 100% Mapeados</t>
+          <t>718 Trámites 100% Mapeados</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="54" customHeight="1">
@@ -3518,7 +3518,7 @@
         </is>
       </c>
       <c r="H19" s="15" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" ht="54" customHeight="1">
@@ -3556,7 +3556,7 @@
         </is>
       </c>
       <c r="H20" s="22" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" ht="54" customHeight="1">
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="H21" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" ht="54" customHeight="1">
@@ -3632,7 +3632,7 @@
         </is>
       </c>
       <c r="H22" s="22" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" ht="54" customHeight="1">
@@ -3670,7 +3670,7 @@
         </is>
       </c>
       <c r="H23" s="15" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" ht="54" customHeight="1">
@@ -3708,7 +3708,7 @@
         </is>
       </c>
       <c r="H24" s="22" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="54" customHeight="1">
@@ -3746,7 +3746,7 @@
         </is>
       </c>
       <c r="H25" s="15" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="54" customHeight="1">
@@ -3784,7 +3784,7 @@
         </is>
       </c>
       <c r="H26" s="22" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" ht="54" customHeight="1">
@@ -3822,7 +3822,7 @@
         </is>
       </c>
       <c r="H27" s="15" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" ht="54" customHeight="1">
@@ -3860,7 +3860,7 @@
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" ht="54" customHeight="1">
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="H29" s="15" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="54" customHeight="1">

</xml_diff>

<commit_message>
feat(profesionales): fusionar duplicados, eliminar subcategorias genericas residuales y sincronizar entregables a 716 tramites
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -778,7 +778,7 @@
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>TOTAL CONTENIDOS
-718 Trámites</t>
+716 Trámites</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -796,7 +796,7 @@
       <c r="F6" s="6" t="inlineStr">
         <is>
           <t>PROFESIONALES
-49 Trámites</t>
+47 Trámites</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="G13" s="15" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H13" s="16">
         <f>G13/$G$15</f>
@@ -1071,7 +1071,7 @@
       <c r="E20" s="35" t="n"/>
       <c r="F20" s="35" t="n"/>
       <c r="G20" s="22" t="n">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H20" s="23">
         <f>G20/$G$24</f>
@@ -1214,7 +1214,7 @@
       <c r="E28" s="35" t="n"/>
       <c r="F28" s="35" t="n"/>
       <c r="G28" s="22" t="n">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="H28" s="23">
         <f>G28/$G$32</f>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="G32" s="22" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H32" s="42">
         <f>G32/$G$37</f>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="J44" s="49" t="inlineStr">
         <is>
-          <t>718 Trámites 100% Mapeados</t>
+          <t>716 Trámites 100% Mapeados</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
         </is>
       </c>
       <c r="H30" s="22" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31" ht="54" customHeight="1">

</xml_diff>

<commit_message>
feat(profesionales): auditoria integral de arquitectura de informacion, homogeneizacion de columnas N1-N5 y sincronizacion de entregables excel
</commit_message>
<xml_diff>
--- a/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
+++ b/docs/fuentes-datos/Mapa_de_Navegacion_y_Descripciones_Portal_SAT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fichas por Rol y Categoría" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fichas por Rol y Categoría'!$A$6:$H$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fichas por Rol y Categoría'!$A$6:$H$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -47,7 +47,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -256,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -347,9 +347,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -770,7 +767,7 @@
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ARQUITECTURA DE INFORMACIÓN DEL PORTAL WEB — DEFINICIÓN DE SEGMENTOS, LEAD TEXT, ATO Y BASE JURÍDICA</t>
+          <t>ARQUITECTURA DE INFORMACIÓN DEL PORTAL WEB — DEFINICIÓN DE SEGMENTOS, LEAD TEXT Y BASE JURÍDICA</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1046,7 @@
       <c r="E19" s="33" t="n"/>
       <c r="F19" s="33" t="n"/>
       <c r="G19" s="15" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H19" s="16">
         <f>G19/$G$24</f>
@@ -1071,7 +1068,7 @@
       <c r="E20" s="35" t="n"/>
       <c r="F20" s="35" t="n"/>
       <c r="G20" s="22" t="n">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="H20" s="23">
         <f>G20/$G$24</f>
@@ -1093,7 +1090,7 @@
       <c r="E21" s="33" t="n"/>
       <c r="F21" s="33" t="n"/>
       <c r="G21" s="15" t="n">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="H21" s="16">
         <f>G21/$G$24</f>
@@ -1137,7 +1134,7 @@
       <c r="E23" s="33" t="n"/>
       <c r="F23" s="33" t="n"/>
       <c r="G23" s="15" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="H23" s="16">
         <f>G23/$G$24</f>
@@ -1152,7 +1149,7 @@
       </c>
       <c r="C24" s="26" t="inlineStr">
         <is>
-          <t>100% de contenidos clasificados según ciclo de vida del contribuyente</t>
+          <t>100% de contenidos clasificados según ciclo de vida</t>
         </is>
       </c>
       <c r="D24" s="24" t="n"/>
@@ -1175,25 +1172,25 @@
       </c>
     </row>
     <row r="27" ht="26" customHeight="1">
-      <c r="B27" s="36" t="inlineStr">
+      <c r="B27" s="29" t="inlineStr">
         <is>
           <t>Tipo de Interacción</t>
         </is>
       </c>
-      <c r="C27" s="36" t="inlineStr">
-        <is>
-          <t>Modalidad Operativa</t>
+      <c r="C27" s="29" t="inlineStr">
+        <is>
+          <t>Descripción Técnica</t>
         </is>
       </c>
       <c r="D27" s="30" t="n"/>
       <c r="E27" s="30" t="n"/>
       <c r="F27" s="31" t="n"/>
-      <c r="G27" s="36" t="inlineStr">
+      <c r="G27" s="29" t="inlineStr">
         <is>
           <t>Total Contenidos</t>
         </is>
       </c>
-      <c r="H27" s="36" t="inlineStr">
+      <c r="H27" s="29" t="inlineStr">
         <is>
           <t>% del Portal</t>
         </is>
@@ -1214,7 +1211,7 @@
       <c r="E28" s="35" t="n"/>
       <c r="F28" s="35" t="n"/>
       <c r="G28" s="22" t="n">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="H28" s="23">
         <f>G28/$G$32</f>
@@ -1236,7 +1233,7 @@
       <c r="E29" s="33" t="n"/>
       <c r="F29" s="33" t="n"/>
       <c r="G29" s="15" t="n">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="H29" s="16">
         <f>G29/$G$32</f>
@@ -1258,7 +1255,7 @@
       <c r="E30" s="35" t="n"/>
       <c r="F30" s="35" t="n"/>
       <c r="G30" s="22" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H30" s="23">
         <f>G30/$G$32</f>
@@ -1343,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J44"/>
+  <dimension ref="B2:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -1423,12 +1420,12 @@
       <c r="B7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="37" t="inlineStr">
+      <c r="C7" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D7" s="37" t="inlineStr">
+      <c r="D7" s="36" t="inlineStr">
         <is>
           <t>NIT sin Obligaciones</t>
         </is>
@@ -1438,7 +1435,7 @@
           <t>NIT sin Obligaciones</t>
         </is>
       </c>
-      <c r="F7" s="38" t="inlineStr">
+      <c r="F7" s="37" t="inlineStr">
         <is>
           <t>Inscripción de primer NIT, actualización de datos de residencia y solvencia fiscal para personas sin actividad mercantil.</t>
         </is>
@@ -1446,15 +1443,15 @@
       <c r="G7" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="H7" s="39">
+      <c r="H7" s="38">
         <f>G7/$G$18</f>
         <v/>
       </c>
-      <c r="I7" s="39">
-        <f>G7/$G$44</f>
-        <v/>
-      </c>
-      <c r="J7" s="38" t="inlineStr">
+      <c r="I7" s="38">
+        <f>G7/$G$38</f>
+        <v/>
+      </c>
+      <c r="J7" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; NIT sin Obligaciones &gt; NIT sin Obligaciones</t>
         </is>
@@ -1464,12 +1461,12 @@
       <c r="B8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="C8" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D8" s="40" t="inlineStr">
+      <c r="D8" s="39" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
@@ -1479,7 +1476,7 @@
           <t>Pequeños Contribuyentes</t>
         </is>
       </c>
-      <c r="F8" s="41" t="inlineStr">
+      <c r="F8" s="40" t="inlineStr">
         <is>
           <t>Régimen del 5% definitivo, facturación FEL, régimen electrónico y regímenes especiales del sector primario y agropecuario.</t>
         </is>
@@ -1487,15 +1484,15 @@
       <c r="G8" s="22" t="n">
         <v>22</v>
       </c>
-      <c r="H8" s="42">
+      <c r="H8" s="41">
         <f>G8/$G$18</f>
         <v/>
       </c>
-      <c r="I8" s="42">
-        <f>G8/$G$44</f>
-        <v/>
-      </c>
-      <c r="J8" s="41" t="inlineStr">
+      <c r="I8" s="41">
+        <f>G8/$G$38</f>
+        <v/>
+      </c>
+      <c r="J8" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Pequeños Contribuyentes &gt; Pequeños Contribuyentes</t>
         </is>
@@ -1505,12 +1502,12 @@
       <c r="B9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="37" t="inlineStr">
+      <c r="C9" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D9" s="37" t="inlineStr">
+      <c r="D9" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1520,7 +1517,7 @@
           <t>Declaraciones y Pagos</t>
         </is>
       </c>
-      <c r="F9" s="38" t="inlineStr">
+      <c r="F9" s="37" t="inlineStr">
         <is>
           <t>Declaración y pago de IVA General, pagos trimestrales o mensuales de ISR, liquidación de ISO y formularios electrónicos.</t>
         </is>
@@ -1528,15 +1525,15 @@
       <c r="G9" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="H9" s="39">
+      <c r="H9" s="38">
         <f>G9/$G$18</f>
         <v/>
       </c>
-      <c r="I9" s="39">
-        <f>G9/$G$44</f>
-        <v/>
-      </c>
-      <c r="J9" s="38" t="inlineStr">
+      <c r="I9" s="38">
+        <f>G9/$G$38</f>
+        <v/>
+      </c>
+      <c r="J9" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; Declaraciones y Pagos</t>
         </is>
@@ -1546,12 +1543,12 @@
       <c r="B10" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="40" t="inlineStr">
+      <c r="C10" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D10" s="40" t="inlineStr">
+      <c r="D10" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1561,7 +1558,7 @@
           <t>RTU Digital y Agencia Virtual</t>
         </is>
       </c>
-      <c r="F10" s="41" t="inlineStr">
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>Inscripción y actualización periódica en el RTU, modificación de domicilios, altas de establecimientos y gestión de usuarios.</t>
         </is>
@@ -1569,15 +1566,15 @@
       <c r="G10" s="22" t="n">
         <v>68</v>
       </c>
-      <c r="H10" s="42">
+      <c r="H10" s="41">
         <f>G10/$G$18</f>
         <v/>
       </c>
-      <c r="I10" s="42">
-        <f>G10/$G$44</f>
-        <v/>
-      </c>
-      <c r="J10" s="41" t="inlineStr">
+      <c r="I10" s="41">
+        <f>G10/$G$38</f>
+        <v/>
+      </c>
+      <c r="J10" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; RTU Digital y Agencia Virtual</t>
         </is>
@@ -1587,12 +1584,12 @@
       <c r="B11" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="37" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D11" s="37" t="inlineStr">
+      <c r="D11" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1602,7 +1599,7 @@
           <t>Vehículos</t>
         </is>
       </c>
-      <c r="F11" s="38" t="inlineStr">
+      <c r="F11" s="37" t="inlineStr">
         <is>
           <t>Registro Fiscal de Vehículos (RFV), calcomanía anual ISCV, primeras placas, traspasos y reposición de distintivos.</t>
         </is>
@@ -1610,15 +1607,15 @@
       <c r="G11" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="H11" s="39">
+      <c r="H11" s="38">
         <f>G11/$G$18</f>
         <v/>
       </c>
-      <c r="I11" s="39">
-        <f>G11/$G$44</f>
-        <v/>
-      </c>
-      <c r="J11" s="38" t="inlineStr">
+      <c r="I11" s="38">
+        <f>G11/$G$38</f>
+        <v/>
+      </c>
+      <c r="J11" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; Vehículos</t>
         </is>
@@ -1628,12 +1625,12 @@
       <c r="B12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="C12" s="40" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D12" s="40" t="inlineStr">
+      <c r="D12" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1643,7 +1640,7 @@
           <t>Servicios al Contribuyente</t>
         </is>
       </c>
-      <c r="F12" s="41" t="inlineStr">
+      <c r="F12" s="40" t="inlineStr">
         <is>
           <t>Agendamiento de citas presenciales, solvencia fiscal con código QR, consultas públicas y asistencia tributaria.</t>
         </is>
@@ -1651,15 +1648,15 @@
       <c r="G12" s="22" t="n">
         <v>44</v>
       </c>
-      <c r="H12" s="42">
+      <c r="H12" s="41">
         <f>G12/$G$18</f>
         <v/>
       </c>
-      <c r="I12" s="42">
-        <f>G12/$G$44</f>
-        <v/>
-      </c>
-      <c r="J12" s="41" t="inlineStr">
+      <c r="I12" s="41">
+        <f>G12/$G$38</f>
+        <v/>
+      </c>
+      <c r="J12" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; Servicios al Contribuyente</t>
         </is>
@@ -1669,12 +1666,12 @@
       <c r="B13" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="C13" s="37" t="inlineStr">
+      <c r="C13" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D13" s="37" t="inlineStr">
+      <c r="D13" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1684,7 +1681,7 @@
           <t>Empresas y Sociedades</t>
         </is>
       </c>
-      <c r="F13" s="38" t="inlineStr">
+      <c r="F13" s="37" t="inlineStr">
         <is>
           <t>Inscripción y cese de sociedades mercantiles, habilitación de sucursales, nombramiento de representantes legales y personerías.</t>
         </is>
@@ -1692,15 +1689,15 @@
       <c r="G13" s="15" t="n">
         <v>31</v>
       </c>
-      <c r="H13" s="39">
+      <c r="H13" s="38">
         <f>G13/$G$18</f>
         <v/>
       </c>
-      <c r="I13" s="39">
-        <f>G13/$G$44</f>
-        <v/>
-      </c>
-      <c r="J13" s="38" t="inlineStr">
+      <c r="I13" s="38">
+        <f>G13/$G$38</f>
+        <v/>
+      </c>
+      <c r="J13" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; Empresas y Sociedades</t>
         </is>
@@ -1710,12 +1707,12 @@
       <c r="B14" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="C14" s="40" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D14" s="40" t="inlineStr">
+      <c r="D14" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1725,7 +1722,7 @@
           <t>Facturación Electrónica</t>
         </is>
       </c>
-      <c r="F14" s="41" t="inlineStr">
+      <c r="F14" s="40" t="inlineStr">
         <is>
           <t>Habilitación como emisor FEL, emisión de facturas y notas de crédito en Agencia Virtual, y anulación de DTE.</t>
         </is>
@@ -1733,15 +1730,15 @@
       <c r="G14" s="22" t="n">
         <v>13</v>
       </c>
-      <c r="H14" s="42">
+      <c r="H14" s="41">
         <f>G14/$G$18</f>
         <v/>
       </c>
-      <c r="I14" s="42">
-        <f>G14/$G$44</f>
-        <v/>
-      </c>
-      <c r="J14" s="41" t="inlineStr">
+      <c r="I14" s="41">
+        <f>G14/$G$38</f>
+        <v/>
+      </c>
+      <c r="J14" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; Facturación Electrónica</t>
         </is>
@@ -1751,12 +1748,12 @@
       <c r="B15" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="C15" s="37" t="inlineStr">
+      <c r="C15" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D15" s="37" t="inlineStr">
+      <c r="D15" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1766,7 +1763,7 @@
           <t>Solvencia y Convenios</t>
         </is>
       </c>
-      <c r="F15" s="38" t="inlineStr">
+      <c r="F15" s="37" t="inlineStr">
         <is>
           <t>Suscripción de convenios de pago en cuotas, facilidades crediticias y regularización de omisos y saldos pendientes.</t>
         </is>
@@ -1774,15 +1771,15 @@
       <c r="G15" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="H15" s="39">
+      <c r="H15" s="38">
         <f>G15/$G$18</f>
         <v/>
       </c>
-      <c r="I15" s="39">
-        <f>G15/$G$44</f>
-        <v/>
-      </c>
-      <c r="J15" s="38" t="inlineStr">
+      <c r="I15" s="38">
+        <f>G15/$G$38</f>
+        <v/>
+      </c>
+      <c r="J15" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; Solvencia y Convenios</t>
         </is>
@@ -1792,12 +1789,12 @@
       <c r="B16" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="C16" s="40" t="inlineStr">
+      <c r="C16" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D16" s="40" t="inlineStr">
+      <c r="D16" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -1807,7 +1804,7 @@
           <t>Asalariados</t>
         </is>
       </c>
-      <c r="F16" s="41" t="inlineStr">
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>Rentas del trabajo en relación de dependencia, planilla electrónica del IVA y devolución de retenciones de ISR.</t>
         </is>
@@ -1815,15 +1812,15 @@
       <c r="G16" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="H16" s="42">
+      <c r="H16" s="41">
         <f>G16/$G$18</f>
         <v/>
       </c>
-      <c r="I16" s="42">
-        <f>G16/$G$44</f>
-        <v/>
-      </c>
-      <c r="J16" s="41" t="inlineStr">
+      <c r="I16" s="41">
+        <f>G16/$G$38</f>
+        <v/>
+      </c>
+      <c r="J16" s="40" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyente General &gt; Asalariados</t>
         </is>
@@ -1833,12 +1830,12 @@
       <c r="B17" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="C17" s="37" t="inlineStr">
+      <c r="C17" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="D17" s="37" t="inlineStr">
+      <c r="D17" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes Especiales</t>
         </is>
@@ -1848,7 +1845,7 @@
           <t>Contribuyentes Especiales</t>
         </is>
       </c>
-      <c r="F17" s="38" t="inlineStr">
+      <c r="F17" s="37" t="inlineStr">
         <is>
           <t>Atención en gerencias diferenciadas, presentación de estados financieros auditados y precios de transferencia.</t>
         </is>
@@ -1856,48 +1853,48 @@
       <c r="G17" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="H17" s="39">
+      <c r="H17" s="38">
         <f>G17/$G$18</f>
         <v/>
       </c>
-      <c r="I17" s="39">
-        <f>G17/$G$44</f>
-        <v/>
-      </c>
-      <c r="J17" s="38" t="inlineStr">
+      <c r="I17" s="38">
+        <f>G17/$G$38</f>
+        <v/>
+      </c>
+      <c r="J17" s="37" t="inlineStr">
         <is>
           <t>Contribuyentes &gt; Contribuyentes Especiales &gt; Contribuyentes Especiales</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="B18" s="43" t="inlineStr"/>
-      <c r="C18" s="44" t="inlineStr">
+      <c r="B18" s="42" t="inlineStr"/>
+      <c r="C18" s="43" t="inlineStr">
         <is>
           <t>SUBTOTAL CONTRIBUYENTES</t>
         </is>
       </c>
-      <c r="D18" s="45" t="inlineStr">
+      <c r="D18" s="44" t="inlineStr">
         <is>
           <t>11 Categorías / Actores</t>
         </is>
       </c>
-      <c r="E18" s="43" t="inlineStr"/>
-      <c r="F18" s="43" t="inlineStr"/>
-      <c r="G18" s="46">
+      <c r="E18" s="42" t="inlineStr"/>
+      <c r="F18" s="42" t="inlineStr"/>
+      <c r="G18" s="45">
         <f>SUM(G7:G17)</f>
         <v/>
       </c>
-      <c r="H18" s="46" t="inlineStr">
+      <c r="H18" s="45" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="I18" s="47">
-        <f>G18/$G$44</f>
-        <v/>
-      </c>
-      <c r="J18" s="45" t="inlineStr">
+      <c r="I18" s="46">
+        <f>G18/$G$38</f>
+        <v/>
+      </c>
+      <c r="J18" s="44" t="inlineStr">
         <is>
           <t>Cobertura completa de Contribuyentes</t>
         </is>
@@ -1907,40 +1904,40 @@
       <c r="B19" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="C19" s="37" t="inlineStr">
+      <c r="C19" s="36" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D19" s="37" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="D19" s="36" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
         <is>
-          <t>Importadores y Exportadores (Compartido)</t>
-        </is>
-      </c>
-      <c r="F19" s="38" t="inlineStr">
-        <is>
-          <t>Arancel Integrado Centroamericano (SAC), pagos aduaneros por BancaSAT, DUCAs comunes y solvencia aduanera.</t>
+          <t>Importadores</t>
+        </is>
+      </c>
+      <c r="F19" s="37" t="inlineStr">
+        <is>
+          <t>Inscripción en padrón de importadores, liquidación de DUCA-D, valoración aduanera, despacho y rescate de mercancías.</t>
         </is>
       </c>
       <c r="G19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="39">
-        <f>G19/$G$31</f>
-        <v/>
-      </c>
-      <c r="I19" s="39">
-        <f>G19/$G$44</f>
-        <v/>
-      </c>
-      <c r="J19" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Importadores y Exportadores (Compartido)</t>
+        <v>55</v>
+      </c>
+      <c r="H19" s="38">
+        <f>G19/$G$25</f>
+        <v/>
+      </c>
+      <c r="I19" s="38">
+        <f>G19/$G$38</f>
+        <v/>
+      </c>
+      <c r="J19" s="37" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; Operaciones Aduaneras y Logística &gt; Importadores</t>
         </is>
       </c>
     </row>
@@ -1948,40 +1945,40 @@
       <c r="B20" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="C20" s="40" t="inlineStr">
+      <c r="C20" s="39" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D20" s="40" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="D20" s="39" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="E20" s="35" t="inlineStr">
         <is>
-          <t>Importadores</t>
-        </is>
-      </c>
-      <c r="F20" s="41" t="inlineStr">
-        <is>
-          <t>Inscripción en padrón de importadores, liquidación de DUCA-D, valoración aduanera y rescate de mercancías.</t>
+          <t>Exportadores</t>
+        </is>
+      </c>
+      <c r="F20" s="40" t="inlineStr">
+        <is>
+          <t>Registro de exportadores VUPE, autorización de embarques y devolución de crédito fiscal del IVA para exportadores.</t>
         </is>
       </c>
       <c r="G20" s="22" t="n">
-        <v>55</v>
-      </c>
-      <c r="H20" s="42">
-        <f>G20/$G$31</f>
-        <v/>
-      </c>
-      <c r="I20" s="42">
-        <f>G20/$G$44</f>
-        <v/>
-      </c>
-      <c r="J20" s="41" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Importadores</t>
+        <v>21</v>
+      </c>
+      <c r="H20" s="41">
+        <f>G20/$G$25</f>
+        <v/>
+      </c>
+      <c r="I20" s="41">
+        <f>G20/$G$38</f>
+        <v/>
+      </c>
+      <c r="J20" s="40" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; Operaciones Aduaneras y Logística &gt; Exportadores</t>
         </is>
       </c>
     </row>
@@ -1989,40 +1986,40 @@
       <c r="B21" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="C21" s="37" t="inlineStr">
+      <c r="C21" s="36" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D21" s="37" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="D21" s="36" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="E21" s="33" t="inlineStr">
         <is>
-          <t>Exportadores</t>
-        </is>
-      </c>
-      <c r="F21" s="38" t="inlineStr">
-        <is>
-          <t>Registro de exportadores VUPE, autorización de embarques y devolución de crédito fiscal del IVA para exportadores.</t>
+          <t>Operador Económico Autorizado (OEA)</t>
+        </is>
+      </c>
+      <c r="F21" s="37" t="inlineStr">
+        <is>
+          <t>Certificación en seguridad de la cadena de suministro, carril exprés aduanero y reducción de selectivo rojo.</t>
         </is>
       </c>
       <c r="G21" s="15" t="n">
-        <v>21</v>
-      </c>
-      <c r="H21" s="39">
-        <f>G21/$G$31</f>
-        <v/>
-      </c>
-      <c r="I21" s="39">
-        <f>G21/$G$44</f>
-        <v/>
-      </c>
-      <c r="J21" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Exportadores</t>
+        <v>2</v>
+      </c>
+      <c r="H21" s="38">
+        <f>G21/$G$25</f>
+        <v/>
+      </c>
+      <c r="I21" s="38">
+        <f>G21/$G$38</f>
+        <v/>
+      </c>
+      <c r="J21" s="37" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; Operaciones Aduaneras y Logística &gt; Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
     </row>
@@ -2030,40 +2027,40 @@
       <c r="B22" s="17" t="n">
         <v>15</v>
       </c>
-      <c r="C22" s="40" t="inlineStr">
+      <c r="C22" s="39" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D22" s="40" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="D22" s="39" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="E22" s="35" t="inlineStr">
         <is>
-          <t>Operador Económico Autorizado (OEA)</t>
-        </is>
-      </c>
-      <c r="F22" s="41" t="inlineStr">
-        <is>
-          <t>Certificación en seguridad de la cadena de suministro, carril exprés aduanero y reducción de selectivo rojo.</t>
+          <t>Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        </is>
+      </c>
+      <c r="F22" s="40" t="inlineStr">
+        <is>
+          <t>Agentes aduaneros, apoderados especiales, depósitos aduaneros (DAT, AGD, fiscales), empresas de courier y transportistas aduaneros.</t>
         </is>
       </c>
       <c r="G22" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="H22" s="42">
-        <f>G22/$G$31</f>
-        <v/>
-      </c>
-      <c r="I22" s="42">
-        <f>G22/$G$44</f>
-        <v/>
-      </c>
-      <c r="J22" s="41" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 1. Importadores y Exportadores &gt; Operador Económico Autorizado (OEA)</t>
+        <v>76</v>
+      </c>
+      <c r="H22" s="41">
+        <f>G22/$G$25</f>
+        <v/>
+      </c>
+      <c r="I22" s="41">
+        <f>G22/$G$38</f>
+        <v/>
+      </c>
+      <c r="J22" s="40" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; Operaciones Aduaneras y Logística &gt; Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
     </row>
@@ -2071,40 +2068,40 @@
       <c r="B23" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="C23" s="37" t="inlineStr">
+      <c r="C23" s="36" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D23" s="37" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="D23" s="36" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="E23" s="33" t="inlineStr">
         <is>
-          <t>Depósitos Aduaneros</t>
-        </is>
-      </c>
-      <c r="F23" s="38" t="inlineStr">
-        <is>
-          <t>Almacenes Fiscales, Almacenes Generales de Depósito (AGD) y Depósitos Aduaneros Temporales (DAT).</t>
+          <t>Regímenes Territoriales y Zonas Especiales</t>
+        </is>
+      </c>
+      <c r="F23" s="37" t="inlineStr">
+        <is>
+          <t>Maquilas (Decreto 29-89) y Zonas de Desarrollo Económico Especial Público (ZDEEP) para entidades administradoras y usuarias.</t>
         </is>
       </c>
       <c r="G23" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="39">
-        <f>G23/$G$31</f>
-        <v/>
-      </c>
-      <c r="I23" s="39">
-        <f>G23/$G$44</f>
-        <v/>
-      </c>
-      <c r="J23" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Depósitos Aduaneros</t>
+        <v>42</v>
+      </c>
+      <c r="H23" s="38">
+        <f>G23/$G$25</f>
+        <v/>
+      </c>
+      <c r="I23" s="38">
+        <f>G23/$G$38</f>
+        <v/>
+      </c>
+      <c r="J23" s="37" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; Operaciones Aduaneras y Logística &gt; Regímenes Territoriales y Zonas Especiales</t>
         </is>
       </c>
     </row>
@@ -2112,831 +2109,585 @@
       <c r="B24" s="17" t="n">
         <v>17</v>
       </c>
-      <c r="C24" s="40" t="inlineStr">
+      <c r="C24" s="39" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="D24" s="40" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="D24" s="39" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="E24" s="35" t="inlineStr">
         <is>
-          <t>Agentes Aduaneros</t>
-        </is>
-      </c>
-      <c r="F24" s="41" t="inlineStr">
-        <is>
-          <t>Habilitación de carné oficial, constitución de pólizas de caución y transmisión de DUCAs con firma electrónica.</t>
+          <t>Normativa y Operaciones Aduaneras Generales</t>
+        </is>
+      </c>
+      <c r="F24" s="40" t="inlineStr">
+        <is>
+          <t>Arancel Centroamericano (SAC), permisos no arancelarios, acuerdos comerciales, prevención del contrabando y modernización aduanera.</t>
         </is>
       </c>
       <c r="G24" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="42">
-        <f>G24/$G$31</f>
-        <v/>
-      </c>
-      <c r="I24" s="42">
-        <f>G24/$G$44</f>
-        <v/>
-      </c>
-      <c r="J24" s="41" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Agentes Aduaneros</t>
+        <v>50</v>
+      </c>
+      <c r="H24" s="41">
+        <f>G24/$G$25</f>
+        <v/>
+      </c>
+      <c r="I24" s="41">
+        <f>G24/$G$38</f>
+        <v/>
+      </c>
+      <c r="J24" s="40" t="inlineStr">
+        <is>
+          <t>Operadores de Comercio Exterior &gt; Operaciones Aduaneras y Logística &gt; Normativa y Operaciones Aduaneras Generales</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="B25" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="C25" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D25" s="37" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
-        </is>
-      </c>
-      <c r="E25" s="33" t="inlineStr">
-        <is>
-          <t>Apoderados Especiales Aduaneros</t>
-        </is>
-      </c>
-      <c r="F25" s="38" t="inlineStr">
-        <is>
-          <t>Representación exclusiva de personas jurídicas en despachos aduaneros propios, carné y renovación de fianza.</t>
-        </is>
-      </c>
-      <c r="G25" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="39">
-        <f>G25/$G$31</f>
-        <v/>
-      </c>
-      <c r="I25" s="39">
-        <f>G25/$G$44</f>
-        <v/>
-      </c>
-      <c r="J25" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Apoderados Especiales Aduaneros</t>
+      <c r="B25" s="42" t="inlineStr"/>
+      <c r="C25" s="43" t="inlineStr">
+        <is>
+          <t>SUBTOTAL OPERADORES DE COMERCIO EXTERIOR</t>
+        </is>
+      </c>
+      <c r="D25" s="44" t="inlineStr">
+        <is>
+          <t>6 Categorías / Actores</t>
+        </is>
+      </c>
+      <c r="E25" s="42" t="inlineStr"/>
+      <c r="F25" s="42" t="inlineStr"/>
+      <c r="G25" s="45">
+        <f>SUM(G19:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="45" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="I25" s="46">
+        <f>G25/$G$38</f>
+        <v/>
+      </c>
+      <c r="J25" s="44" t="inlineStr">
+        <is>
+          <t>Cobertura completa de Operadores de Comercio Exterior</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="B26" s="17" t="n">
-        <v>19</v>
-      </c>
-      <c r="C26" s="40" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D26" s="40" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        <v>18</v>
+      </c>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D26" s="39" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="E26" s="35" t="inlineStr">
         <is>
-          <t>Transportistas Aduaneros</t>
-        </is>
-      </c>
-      <c r="F26" s="41" t="inlineStr">
-        <is>
-          <t>Registro de unidades y conductores, transmisión de DUCA-T y colocación de marchamo electrónico RFID.</t>
+          <t>Abogados y Notarios</t>
+        </is>
+      </c>
+      <c r="F26" s="40" t="inlineStr">
+        <is>
+          <t>Compra de papel sellado de protocolo (SAT-7130), timbres fiscales, razón electrónica, avisos notariales y traspasos vehiculares electrónicos (TEV).</t>
         </is>
       </c>
       <c r="G26" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="42">
+        <v>18</v>
+      </c>
+      <c r="H26" s="41">
         <f>G26/$G$31</f>
         <v/>
       </c>
-      <c r="I26" s="42">
-        <f>G26/$G$44</f>
-        <v/>
-      </c>
-      <c r="J26" s="41" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Transportistas Aduaneros</t>
+      <c r="I26" s="41">
+        <f>G26/$G$38</f>
+        <v/>
+      </c>
+      <c r="J26" s="40" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Auxiliares &gt; Abogados y Notarios</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="B27" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="C27" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D27" s="37" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        <v>19</v>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D27" s="36" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="E27" s="33" t="inlineStr">
         <is>
-          <t>Empresas de Entrega Rápida o Courier</t>
-        </is>
-      </c>
-      <c r="F27" s="38" t="inlineStr">
-        <is>
-          <t>Despacho simplificado de paquetería urgente, manifiestos courier y recintos desconsolidadores de encomiendas.</t>
+          <t>Peritos Contadores</t>
+        </is>
+      </c>
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>Inscripción y actualización en el Registro de Contadores, autorización del LET, Factura Electrónica FEL, retenciones y declaraciones.</t>
         </is>
       </c>
       <c r="G27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="39">
+        <v>11</v>
+      </c>
+      <c r="H27" s="38">
         <f>G27/$G$31</f>
         <v/>
       </c>
-      <c r="I27" s="39">
-        <f>G27/$G$44</f>
-        <v/>
-      </c>
-      <c r="J27" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Empresas de Entrega Rápida o Courier</t>
+      <c r="I27" s="38">
+        <f>G27/$G$38</f>
+        <v/>
+      </c>
+      <c r="J27" s="37" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Auxiliares &gt; Peritos Contadores</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="B28" s="17" t="n">
-        <v>21</v>
-      </c>
-      <c r="C28" s="40" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D28" s="40" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+        <v>20</v>
+      </c>
+      <c r="C28" s="39" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D28" s="39" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="E28" s="35" t="inlineStr">
         <is>
-          <t>Consolidadores y Desconsolidadores de Carga</t>
-        </is>
-      </c>
-      <c r="F28" s="41" t="inlineStr">
-        <is>
-          <t>Transmisión de manifiesto electrónico CUSCAR, desconsolidación de conocimientos de embarque y guías hijas.</t>
+          <t>Auditores</t>
+        </is>
+      </c>
+      <c r="F28" s="40" t="inlineStr">
+        <is>
+          <t>Inscripción de CPA, actualización registral de colegiado y emisión de dictámenes de crédito fiscal para exportadores.</t>
         </is>
       </c>
       <c r="G28" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="42">
+        <v>4</v>
+      </c>
+      <c r="H28" s="41">
         <f>G28/$G$31</f>
         <v/>
       </c>
-      <c r="I28" s="42">
-        <f>G28/$G$44</f>
-        <v/>
-      </c>
-      <c r="J28" s="41" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 2. Auxiliares de la Función Pública Aduanera (AFPA) &gt; Consolidadores y Desconsolidadores de Carga</t>
+      <c r="I28" s="41">
+        <f>G28/$G$38</f>
+        <v/>
+      </c>
+      <c r="J28" s="40" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Auxiliares &gt; Auditores</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="B29" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="C29" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D29" s="37" t="inlineStr">
-        <is>
-          <t>3. Regímenes Territoriales y Zonas Especiales</t>
+        <v>21</v>
+      </c>
+      <c r="C29" s="36" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D29" s="36" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="E29" s="33" t="inlineStr">
         <is>
-          <t>ZDEEP - Entidades Administradoras</t>
-        </is>
-      </c>
-      <c r="F29" s="38" t="inlineStr">
-        <is>
-          <t>Habilitación de polígonos industriales ZDEEP, supervisión perimetral, garitas de control y recintos aduaneros.</t>
+          <t>Gestores Tributarios</t>
+        </is>
+      </c>
+      <c r="F29" s="37" t="inlineStr">
+        <is>
+          <t>Acreditación oficial, expedición y renovación anual de gafetes, reposición de credencial y padrón activo de gestores y auxiliares.</t>
         </is>
       </c>
       <c r="G29" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="39">
+        <v>8</v>
+      </c>
+      <c r="H29" s="38">
         <f>G29/$G$31</f>
         <v/>
       </c>
-      <c r="I29" s="39">
-        <f>G29/$G$44</f>
-        <v/>
-      </c>
-      <c r="J29" s="38" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 3. Regímenes Territoriales y Zonas Especiales &gt; ZDEEP - Entidades Administradoras</t>
+      <c r="I29" s="38">
+        <f>G29/$G$38</f>
+        <v/>
+      </c>
+      <c r="J29" s="37" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Auxiliares &gt; Gestores Tributarios</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="B30" s="17" t="n">
-        <v>23</v>
-      </c>
-      <c r="C30" s="40" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="D30" s="40" t="inlineStr">
-        <is>
-          <t>3. Regímenes Territoriales y Zonas Especiales</t>
+        <v>22</v>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="D30" s="39" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="E30" s="35" t="inlineStr">
         <is>
-          <t>ZDEEP - Empresas Usuarias</t>
-        </is>
-      </c>
-      <c r="F30" s="41" t="inlineStr">
-        <is>
-          <t>Ingreso de insumos con suspensión arancelaria, descargos de transformación y exenciones tributarias de fomento.</t>
+          <t>Servicios Profesionales</t>
+        </is>
+      </c>
+      <c r="F30" s="40" t="inlineStr">
+        <is>
+          <t>Facturación FEL por honorarios, catálogo general de Declaraguate, consultas jurídico-tributarias vinculantes y retenciones hospitalarias.</t>
         </is>
       </c>
       <c r="G30" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="42">
+        <v>6</v>
+      </c>
+      <c r="H30" s="41">
         <f>G30/$G$31</f>
         <v/>
       </c>
-      <c r="I30" s="42">
-        <f>G30/$G$44</f>
-        <v/>
-      </c>
-      <c r="J30" s="41" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior &gt; 3. Regímenes Territoriales y Zonas Especiales &gt; ZDEEP - Empresas Usuarias</t>
+      <c r="I30" s="41">
+        <f>G30/$G$38</f>
+        <v/>
+      </c>
+      <c r="J30" s="40" t="inlineStr">
+        <is>
+          <t>Profesionales &gt; Servicios Profesionales y Auxiliares &gt; Servicios Profesionales</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="B31" s="43" t="inlineStr"/>
-      <c r="C31" s="44" t="inlineStr">
-        <is>
-          <t>SUBTOTAL OPERADORES DE COMERCIO EXTERIOR</t>
-        </is>
-      </c>
-      <c r="D31" s="45" t="inlineStr">
-        <is>
-          <t>12 Categorías / Actores</t>
-        </is>
-      </c>
-      <c r="E31" s="43" t="inlineStr"/>
-      <c r="F31" s="43" t="inlineStr"/>
-      <c r="G31" s="46">
-        <f>SUM(G19:G30)</f>
-        <v/>
-      </c>
-      <c r="H31" s="46" t="inlineStr">
+      <c r="B31" s="42" t="inlineStr"/>
+      <c r="C31" s="43" t="inlineStr">
+        <is>
+          <t>SUBTOTAL PROFESIONALES</t>
+        </is>
+      </c>
+      <c r="D31" s="44" t="inlineStr">
+        <is>
+          <t>5 Categorías / Actores</t>
+        </is>
+      </c>
+      <c r="E31" s="42" t="inlineStr"/>
+      <c r="F31" s="42" t="inlineStr"/>
+      <c r="G31" s="45">
+        <f>SUM(G26:G30)</f>
+        <v/>
+      </c>
+      <c r="H31" s="45" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="I31" s="47">
-        <f>G31/$G$44</f>
-        <v/>
-      </c>
-      <c r="J31" s="45" t="inlineStr">
-        <is>
-          <t>Cobertura completa de Operadores de Comercio Exterior</t>
+      <c r="I31" s="46">
+        <f>G31/$G$38</f>
+        <v/>
+      </c>
+      <c r="J31" s="44" t="inlineStr">
+        <is>
+          <t>Cobertura completa de Profesionales</t>
         </is>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="B32" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="C32" s="40" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="D32" s="40" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+        <v>23</v>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D32" s="39" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="E32" s="35" t="inlineStr">
         <is>
-          <t>Abogados y Notarios</t>
-        </is>
-      </c>
-      <c r="F32" s="41" t="inlineStr">
-        <is>
-          <t>Compra de papel sellado de protocolo (SAT-7130), timbres fiscales y traspasos electrónicos vehiculares (TEV).</t>
+          <t>Constitucionales</t>
+        </is>
+      </c>
+      <c r="F32" s="40" t="inlineStr">
+        <is>
+          <t>Exención constitucional de impuestos para universidades, colegios, iglesias y misiones diplomáticas.</t>
         </is>
       </c>
       <c r="G32" s="22" t="n">
         <v>18</v>
       </c>
-      <c r="H32" s="42">
+      <c r="H32" s="41">
         <f>G32/$G$37</f>
         <v/>
       </c>
-      <c r="I32" s="42">
-        <f>G32/$G$44</f>
-        <v/>
-      </c>
-      <c r="J32" s="41" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Abogados y Notarios</t>
+      <c r="I32" s="41">
+        <f>G32/$G$38</f>
+        <v/>
+      </c>
+      <c r="J32" s="40" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; Constitucionales</t>
         </is>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="B33" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="D33" s="37" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+        <v>24</v>
+      </c>
+      <c r="C33" s="36" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D33" s="36" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="E33" s="33" t="inlineStr">
         <is>
-          <t>Peritos Contadores</t>
-        </is>
-      </c>
-      <c r="F33" s="38" t="inlineStr">
-        <is>
-          <t>Inscripción en el Registro de Contadores, autorización de libros contables digitales y firma de balances.</t>
+          <t>Decreto</t>
+        </is>
+      </c>
+      <c r="F33" s="37" t="inlineStr">
+        <is>
+          <t>Entidades con incentivos y exenciones especiales otorgadas por leyes ordinarias de fomento sectorial.</t>
         </is>
       </c>
       <c r="G33" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="H33" s="39">
+        <v>16</v>
+      </c>
+      <c r="H33" s="38">
         <f>G33/$G$37</f>
         <v/>
       </c>
-      <c r="I33" s="39">
-        <f>G33/$G$44</f>
-        <v/>
-      </c>
-      <c r="J33" s="38" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Peritos Contadores</t>
+      <c r="I33" s="38">
+        <f>G33/$G$38</f>
+        <v/>
+      </c>
+      <c r="J33" s="37" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; Decreto</t>
         </is>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="B34" s="17" t="n">
-        <v>26</v>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="D34" s="40" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+        <v>25</v>
+      </c>
+      <c r="C34" s="39" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D34" s="39" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="E34" s="35" t="inlineStr">
         <is>
-          <t>Gestores Tributarios</t>
-        </is>
-      </c>
-      <c r="F34" s="41" t="inlineStr">
-        <is>
-          <t>Acreditación oficial ante SAT, renovación de gafetes, registro biométrico y representación presencial autorizada.</t>
+          <t>No Lucrativos</t>
+        </is>
+      </c>
+      <c r="F34" s="40" t="inlineStr">
+        <is>
+          <t>Resoluciones de exención de ISR e IVA para ONGs, fundaciones benéficas, asociaciones y cooperativas.</t>
         </is>
       </c>
       <c r="G34" s="22" t="n">
-        <v>8</v>
-      </c>
-      <c r="H34" s="42">
+        <v>14</v>
+      </c>
+      <c r="H34" s="41">
         <f>G34/$G$37</f>
         <v/>
       </c>
-      <c r="I34" s="42">
-        <f>G34/$G$44</f>
-        <v/>
-      </c>
-      <c r="J34" s="41" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Gestores Tributarios</t>
+      <c r="I34" s="41">
+        <f>G34/$G$38</f>
+        <v/>
+      </c>
+      <c r="J34" s="40" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; No Lucrativos</t>
         </is>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="B35" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="D35" s="37" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+        <v>26</v>
+      </c>
+      <c r="C35" s="36" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D35" s="36" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
         </is>
       </c>
       <c r="E35" s="33" t="inlineStr">
         <is>
-          <t>Servicios Profesionales</t>
-        </is>
-      </c>
-      <c r="F35" s="38" t="inlineStr">
-        <is>
-          <t>Facturación FEL por honorarios profesionales, retenciones de ISR y actualización de constancia de colegiado activo.</t>
+          <t>Entidades del Estado</t>
+        </is>
+      </c>
+      <c r="F35" s="37" t="inlineStr">
+        <is>
+          <t>Ministerios, secretarías, organismos del Estado, compras públicas y emisión de constancias de retención.</t>
         </is>
       </c>
       <c r="G35" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="H35" s="39">
+        <v>26</v>
+      </c>
+      <c r="H35" s="38">
         <f>G35/$G$37</f>
         <v/>
       </c>
-      <c r="I35" s="39">
-        <f>G35/$G$44</f>
-        <v/>
-      </c>
-      <c r="J35" s="38" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Servicios Profesionales</t>
+      <c r="I35" s="38">
+        <f>G35/$G$38</f>
+        <v/>
+      </c>
+      <c r="J35" s="37" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Sector Público y Entidades del Estado &gt; Entidades del Estado</t>
         </is>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="B36" s="17" t="n">
-        <v>28</v>
-      </c>
-      <c r="C36" s="40" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="D36" s="40" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+        <v>27</v>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="D36" s="39" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
         </is>
       </c>
       <c r="E36" s="35" t="inlineStr">
         <is>
-          <t>Auditores</t>
-        </is>
-      </c>
-      <c r="F36" s="41" t="inlineStr">
-        <is>
-          <t>Dictámenes de crédito fiscal para exportadores, dictámenes de estados financieros e informes tributarios.</t>
+          <t>Municipalidades</t>
+        </is>
+      </c>
+      <c r="F36" s="40" t="inlineStr">
+        <is>
+          <t>Autonomía municipal, inscripción de corporaciones y flotillas vehiculares municipales exentas del ISCV.</t>
         </is>
       </c>
       <c r="G36" s="22" t="n">
-        <v>4</v>
-      </c>
-      <c r="H36" s="42">
+        <v>5</v>
+      </c>
+      <c r="H36" s="41">
         <f>G36/$G$37</f>
         <v/>
       </c>
-      <c r="I36" s="42">
-        <f>G36/$G$44</f>
-        <v/>
-      </c>
-      <c r="J36" s="41" t="inlineStr">
-        <is>
-          <t>Profesionales &gt; Servicios Profesionales y Terceras Personas &gt; Auditores</t>
+      <c r="I36" s="41">
+        <f>G36/$G$38</f>
+        <v/>
+      </c>
+      <c r="J36" s="40" t="inlineStr">
+        <is>
+          <t>Entes Exentos &gt; Sector Público y Entidades del Estado &gt; Municipalidades</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
-      <c r="B37" s="43" t="inlineStr"/>
-      <c r="C37" s="44" t="inlineStr">
-        <is>
-          <t>SUBTOTAL PROFESIONALES</t>
-        </is>
-      </c>
-      <c r="D37" s="45" t="inlineStr">
+      <c r="B37" s="42" t="inlineStr"/>
+      <c r="C37" s="43" t="inlineStr">
+        <is>
+          <t>SUBTOTAL ENTES EXENTOS</t>
+        </is>
+      </c>
+      <c r="D37" s="44" t="inlineStr">
         <is>
           <t>5 Categorías / Actores</t>
         </is>
       </c>
-      <c r="E37" s="43" t="inlineStr"/>
-      <c r="F37" s="43" t="inlineStr"/>
-      <c r="G37" s="46">
+      <c r="E37" s="42" t="inlineStr"/>
+      <c r="F37" s="42" t="inlineStr"/>
+      <c r="G37" s="45">
         <f>SUM(G32:G36)</f>
         <v/>
       </c>
-      <c r="H37" s="46" t="inlineStr">
+      <c r="H37" s="45" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="I37" s="47">
-        <f>G37/$G$44</f>
-        <v/>
-      </c>
-      <c r="J37" s="45" t="inlineStr">
-        <is>
-          <t>Cobertura completa de Profesionales</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="B38" s="17" t="n">
-        <v>29</v>
-      </c>
-      <c r="C38" s="40" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D38" s="40" t="inlineStr">
-        <is>
-          <t>Organizaciones No Lucrativas (Exentas)</t>
-        </is>
-      </c>
-      <c r="E38" s="35" t="inlineStr">
-        <is>
-          <t>Constitucionales</t>
-        </is>
-      </c>
-      <c r="F38" s="41" t="inlineStr">
-        <is>
-          <t>Exención constitucional de impuestos para universidades, colegios, iglesias y misiones diplomáticas.</t>
-        </is>
-      </c>
-      <c r="G38" s="22" t="n">
-        <v>18</v>
-      </c>
-      <c r="H38" s="42">
-        <f>G38/$G$43</f>
-        <v/>
-      </c>
-      <c r="I38" s="42">
-        <f>G38/$G$44</f>
-        <v/>
-      </c>
-      <c r="J38" s="41" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; Constitucionales</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="B39" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="C39" s="37" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D39" s="37" t="inlineStr">
-        <is>
-          <t>Organizaciones No Lucrativas (Exentas)</t>
-        </is>
-      </c>
-      <c r="E39" s="33" t="inlineStr">
-        <is>
-          <t>Decreto</t>
-        </is>
-      </c>
-      <c r="F39" s="38" t="inlineStr">
-        <is>
-          <t>Entidades con incentivos y exenciones especiales otorgadas por leyes ordinarias de fomento sectorial.</t>
-        </is>
-      </c>
-      <c r="G39" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="H39" s="39">
-        <f>G39/$G$43</f>
-        <v/>
-      </c>
-      <c r="I39" s="39">
-        <f>G39/$G$44</f>
-        <v/>
-      </c>
-      <c r="J39" s="38" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; Decreto</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="B40" s="17" t="n">
-        <v>31</v>
-      </c>
-      <c r="C40" s="40" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D40" s="40" t="inlineStr">
-        <is>
-          <t>Organizaciones No Lucrativas (Exentas)</t>
-        </is>
-      </c>
-      <c r="E40" s="35" t="inlineStr">
-        <is>
-          <t>No Lucrativos</t>
-        </is>
-      </c>
-      <c r="F40" s="41" t="inlineStr">
-        <is>
-          <t>Resoluciones de exención de ISR e IVA para ONGs, fundaciones benéficas, asociaciones y cooperativas.</t>
-        </is>
-      </c>
-      <c r="G40" s="22" t="n">
-        <v>14</v>
-      </c>
-      <c r="H40" s="42">
-        <f>G40/$G$43</f>
-        <v/>
-      </c>
-      <c r="I40" s="42">
-        <f>G40/$G$44</f>
-        <v/>
-      </c>
-      <c r="J40" s="41" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Organizaciones No Lucrativas (Exentas) &gt; No Lucrativos</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="24" customHeight="1">
-      <c r="B41" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="C41" s="37" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D41" s="37" t="inlineStr">
-        <is>
-          <t>Sector Público y Entidades del Estado</t>
-        </is>
-      </c>
-      <c r="E41" s="33" t="inlineStr">
-        <is>
-          <t>Entidades del Estado</t>
-        </is>
-      </c>
-      <c r="F41" s="38" t="inlineStr">
-        <is>
-          <t>Ministerios, secretarías, organismos del Estado, compras públicas y emisión de constancias de retención.</t>
-        </is>
-      </c>
-      <c r="G41" s="15" t="n">
-        <v>26</v>
-      </c>
-      <c r="H41" s="39">
-        <f>G41/$G$43</f>
-        <v/>
-      </c>
-      <c r="I41" s="39">
-        <f>G41/$G$44</f>
-        <v/>
-      </c>
-      <c r="J41" s="38" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Sector Público y Entidades del Estado &gt; Entidades del Estado</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="B42" s="17" t="n">
-        <v>33</v>
-      </c>
-      <c r="C42" s="40" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="D42" s="40" t="inlineStr">
-        <is>
-          <t>Sector Público y Entidades del Estado</t>
-        </is>
-      </c>
-      <c r="E42" s="35" t="inlineStr">
-        <is>
-          <t>Municipalidades</t>
-        </is>
-      </c>
-      <c r="F42" s="41" t="inlineStr">
-        <is>
-          <t>Autonomía municipal, inscripción de corporaciones y flotillas vehiculares municipales exentas del ISCV.</t>
-        </is>
-      </c>
-      <c r="G42" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="H42" s="42">
-        <f>G42/$G$43</f>
-        <v/>
-      </c>
-      <c r="I42" s="42">
-        <f>G42/$G$44</f>
-        <v/>
-      </c>
-      <c r="J42" s="41" t="inlineStr">
-        <is>
-          <t>Entes Exentos &gt; Sector Público y Entidades del Estado &gt; Municipalidades</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="24" customHeight="1">
-      <c r="B43" s="43" t="inlineStr"/>
-      <c r="C43" s="44" t="inlineStr">
-        <is>
-          <t>SUBTOTAL ENTES EXENTOS</t>
-        </is>
-      </c>
-      <c r="D43" s="45" t="inlineStr">
-        <is>
-          <t>5 Categorías / Actores</t>
-        </is>
-      </c>
-      <c r="E43" s="43" t="inlineStr"/>
-      <c r="F43" s="43" t="inlineStr"/>
-      <c r="G43" s="46">
-        <f>SUM(G38:G42)</f>
-        <v/>
-      </c>
-      <c r="H43" s="46" t="inlineStr">
+      <c r="I37" s="46">
+        <f>G37/$G$38</f>
+        <v/>
+      </c>
+      <c r="J37" s="44" t="inlineStr">
+        <is>
+          <t>Cobertura completa de Entes Exentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="B38" s="47" t="inlineStr"/>
+      <c r="C38" s="48" t="inlineStr">
+        <is>
+          <t>TOTAL PORTAL WEB SAT</t>
+        </is>
+      </c>
+      <c r="D38" s="49" t="inlineStr">
+        <is>
+          <t>4 Segmentos y 27 Categorías</t>
+        </is>
+      </c>
+      <c r="E38" s="47" t="inlineStr"/>
+      <c r="F38" s="48" t="inlineStr">
+        <is>
+          <t>Universo Total de Fichas Oficiales</t>
+        </is>
+      </c>
+      <c r="G38" s="50">
+        <f>G18+G25+G31+G37</f>
+        <v/>
+      </c>
+      <c r="H38" s="51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="52" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="I43" s="47">
-        <f>G43/$G$44</f>
-        <v/>
-      </c>
-      <c r="J43" s="45" t="inlineStr">
-        <is>
-          <t>Cobertura completa de Entes Exentos</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="28" customHeight="1">
-      <c r="B44" s="48" t="inlineStr"/>
-      <c r="C44" s="49" t="inlineStr">
-        <is>
-          <t>TOTAL PORTAL WEB SAT</t>
-        </is>
-      </c>
-      <c r="D44" s="50" t="inlineStr">
-        <is>
-          <t>4 Segmentos y 33 Categorías</t>
-        </is>
-      </c>
-      <c r="E44" s="48" t="inlineStr"/>
-      <c r="F44" s="49" t="inlineStr">
-        <is>
-          <t>Universo Total de Fichas Oficiales</t>
-        </is>
-      </c>
-      <c r="G44" s="51">
-        <f>G18+G31+G37+G43</f>
-        <v/>
-      </c>
-      <c r="H44" s="52" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I44" s="53" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="J44" s="49" t="inlineStr">
+      <c r="J38" s="48" t="inlineStr">
         <is>
           <t>716 Trámites 100% Mapeados</t>
         </is>
@@ -2957,7 +2708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:H40"/>
+  <dimension ref="A2:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2981,7 +2732,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MATRIZ COMPLETA DE LAS 33 CATEGORÍAS DEL PORTAL CON SUS TEXTOS ORIENTADORES Y MARCO NORMATIVO OFICIAL</t>
+          <t>MATRIZ COMPLETA DE LAS 27 CATEGORÍAS DEL PORTAL CON SUS TEXTOS ORIENTADORES Y MARCO NORMATIVO OFICIAL</t>
         </is>
       </c>
     </row>
@@ -3031,12 +2782,12 @@
       <c r="A7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="37" t="inlineStr">
+      <c r="B7" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C7" s="37" t="inlineStr">
+      <c r="C7" s="36" t="inlineStr">
         <is>
           <t>NIT sin Obligaciones</t>
         </is>
@@ -3069,12 +2820,12 @@
       <c r="A8" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C8" s="40" t="inlineStr">
+      <c r="C8" s="39" t="inlineStr">
         <is>
           <t>Pequeños Contribuyentes</t>
         </is>
@@ -3107,12 +2858,12 @@
       <c r="A9" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C9" s="37" t="inlineStr">
+      <c r="C9" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3145,12 +2896,12 @@
       <c r="A10" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="40" t="inlineStr">
+      <c r="B10" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C10" s="40" t="inlineStr">
+      <c r="C10" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3183,12 +2934,12 @@
       <c r="A11" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C11" s="37" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3221,12 +2972,12 @@
       <c r="A12" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B12" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C12" s="40" t="inlineStr">
+      <c r="C12" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3259,12 +3010,12 @@
       <c r="A13" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="37" t="inlineStr">
+      <c r="B13" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C13" s="37" t="inlineStr">
+      <c r="C13" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3297,12 +3048,12 @@
       <c r="A14" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="40" t="inlineStr">
+      <c r="B14" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C14" s="40" t="inlineStr">
+      <c r="C14" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3335,12 +3086,12 @@
       <c r="A15" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="37" t="inlineStr">
+      <c r="B15" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C15" s="37" t="inlineStr">
+      <c r="C15" s="36" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3373,12 +3124,12 @@
       <c r="A16" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B16" s="39" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C16" s="40" t="inlineStr">
+      <c r="C16" s="39" t="inlineStr">
         <is>
           <t>Contribuyente General</t>
         </is>
@@ -3411,12 +3162,12 @@
       <c r="A17" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="37" t="inlineStr">
+      <c r="B17" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes</t>
         </is>
       </c>
-      <c r="C17" s="37" t="inlineStr">
+      <c r="C17" s="36" t="inlineStr">
         <is>
           <t>Contribuyentes Especiales</t>
         </is>
@@ -3449,869 +3200,641 @@
       <c r="A18" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="40" t="inlineStr">
+      <c r="B18" s="39" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C18" s="40" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="D18" s="35" t="inlineStr">
         <is>
-          <t>Importadores y Exportadores (Compartido)</t>
+          <t>Importadores</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>Operadores comerciales que realizan indistintamente gestiones transversales de entrada y salida de mercancías, consultas arancelarias y pagos tributarios aduaneros en las aduanas de la República.</t>
+          <t>Personas individuales o jurídicas autorizadas en el padrón aduanero de la SAT para introducir legalmente mercancías extranjeras al territorio aduanero nacional para su consumo, uso o transformación.</t>
         </is>
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>Consulta el Arancel Integrado Centroamericano (SAC), realiza pagos por BancaSAT y tramita solvencias aduaneras unificadas.</t>
+          <t>Inscríbete en el padrón de importadores, liquida tus declaraciones aduaneras DUCA-D, consulta aranceles y rescata mercancías en aduana.</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Convenio sobre el Régimen Arancelario y Aduanero Centroamericano, CAUCA IV (Resolución 223-2008 COMIECO) y RECAUCA IV (Resolución 224-2008 COMIECO).</t>
+          <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Acuerdo de Valoración de la OMC.</t>
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" ht="54" customHeight="1">
       <c r="A19" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="37" t="inlineStr">
+      <c r="B19" s="36" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C19" s="37" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="C19" s="36" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="D19" s="33" t="inlineStr">
         <is>
-          <t>Importadores</t>
+          <t>Exportadores</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Personas individuales o jurídicas autorizadas en el padrón aduanero de la SAT para introducir legalmente mercancías extranjeras al territorio aduanero nacional para su consumo, uso o transformación.</t>
+          <t>Personas individuales o jurídicas inscritas en el Registro de Exportadores de la SAT que despachan mercancías de origen nacional o nacionalizadas hacia mercados del exterior.</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Inscríbete en el padrón de importadores, liquida tus declaraciones aduaneras DUCA-D, consulta aranceles y rescata mercancías en aduana.</t>
+          <t>Registra tus exportaciones con código VUPE, emite facturas con régimen especial y gestiona la devolución de crédito fiscal del IVA.</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>CAUCA IV (Arts. 21 y 77), RECAUCA IV (Arts. 317 al 330) y Acuerdo Relativo a la Aplicación del Artículo VII del GATT (Valoración OMC).</t>
+          <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Ley de Fomento y Maquila (Decreto 29-89) y CAUCA/RECAUCA IV.</t>
         </is>
       </c>
       <c r="H19" s="15" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
     </row>
     <row r="20" ht="54" customHeight="1">
       <c r="A20" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="40" t="inlineStr">
+      <c r="B20" s="39" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C20" s="40" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="D20" s="35" t="inlineStr">
         <is>
-          <t>Exportadores</t>
+          <t>Operador Económico Autorizado (OEA)</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
         <is>
-          <t>Personas individuales o jurídicas inscritas en el Registro de Exportadores de la SAT que despachan mercancías de origen nacional o nacionalizadas hacia mercados del exterior.</t>
+          <t>Operadores de la cadena logística internacional certificados por la Intendencia de Aduanas por mantener rigurosos estándares de seguridad y confiabilidad en sus operaciones transfronterizas.</t>
         </is>
       </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
-          <t>Registra tus exportaciones con código VUPE, emite facturas con régimen especial y gestiona la devolución de crédito fiscal del IVA.</t>
+          <t>Accede a carriles exprés preferenciales, prioridad en contingencias y despacho ágil con selectivo rojo reducido.</t>
         </is>
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>Ley del IVA (Decreto 27-92, Arts. 23 al 25 bis), Ley de Fomento y Maquila (Decreto 29-89) y CAUCA/RECAUCA IV.</t>
+          <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio de la SAT sobre el Programa OEA-Guatemala.</t>
         </is>
       </c>
       <c r="H20" s="22" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" ht="54" customHeight="1">
       <c r="A21" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="B21" s="37" t="inlineStr">
+      <c r="B21" s="36" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C21" s="37" t="inlineStr">
-        <is>
-          <t>1. Importadores y Exportadores</t>
+      <c r="C21" s="36" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>Operador Económico Autorizado (OEA)</t>
+          <t>Auxiliares de la Función Pública Aduanera (AFPA)</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Operadores de la cadena logística internacional certificados por la Intendencia de Aduanas por mantener rigurosos estándares de seguridad y confiabilidad en sus operaciones transfronterizas.</t>
+          <t>Personas naturales o jurídicas autorizadas por la SAT para actuar en nombre propio o de terceros ante el Servicio Aduanero en el desaduanamiento, transporte, custodia o desconsolidación de mercancías.</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Accede a carriles exprés preferenciales, prioridad en contingencias y despacho ágil con selectivo rojo reducido.</t>
+          <t>Gestiona carnés oficiales, pólizas de garantía operativa, marchamos electrónicos y despachos logísticos autorizados.</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>Marco Normativo SAFE de la OMA, CAUCA IV y Resoluciones de Directorio de la SAT sobre el Programa OEA-Guatemala.</t>
+          <t>CAUCA IV (Arts. 18 al 28), RECAUCA IV (Arts. 74 al 136) y Ley Nacional de Aduanas.</t>
         </is>
       </c>
       <c r="H21" s="15" t="n">
-        <v>2</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" ht="54" customHeight="1">
       <c r="A22" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="B22" s="40" t="inlineStr">
+      <c r="B22" s="39" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C22" s="40" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="D22" s="35" t="inlineStr">
         <is>
-          <t>Depósitos Aduaneros</t>
+          <t>Regímenes Territoriales y Zonas Especiales</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
-          <t>Recintos públicos o privados autorizados para custodiar mercancías con suspensión de tributos aduaneros, emisión de certificados de depósito y bonos de prenda (AGD) y actas de recepción DAT.</t>
+          <t>Empresas y polígonos industriales delimitados que operan bajo regímenes aduaneros liberatorios o de fomento económico con suspensión y exención arancelaria y fiscal.</t>
         </is>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
-          <t>Controla inventarios de custodia, gestiona actas de recepción, emite certificados de depósito (AGD) y tramita prórrogas de permanencia.</t>
+          <t>Administra polígonos ZDEEP, ingresa insumos con suspensión de aranceles y liquida cuentas corrientes bajo el Decreto 29-89.</t>
         </is>
       </c>
       <c r="G22" s="21" t="inlineStr">
         <is>
-          <t>Decreto 1236 (Ley de Almacenes Generales de Depósito), CAUCA IV y RECAUCA IV (Arts. 119 al 129 - Régimen de Depósito Aduanero).</t>
+          <t>Decreto 29-89 (Ley de Maquilas), Decreto 22-73 (Ley Orgánica de ZOLIC reformada) y Resoluciones SAT-ZDEEP.</t>
         </is>
       </c>
       <c r="H22" s="22" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" ht="54" customHeight="1">
       <c r="A23" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="B23" s="37" t="inlineStr">
+      <c r="B23" s="36" t="inlineStr">
         <is>
           <t>Operadores de Comercio Exterior</t>
         </is>
       </c>
-      <c r="C23" s="37" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="C23" s="36" t="inlineStr">
+        <is>
+          <t>Operaciones Aduaneras y Logística</t>
         </is>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
-          <t>Agentes Aduaneros</t>
+          <t>Normativa y Operaciones Aduaneras Generales</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Profesionales auxiliares de la función pública aduanera autorizados para actuar por cuenta de terceros en los trámites y operaciones de desaduanamiento ante la SAT.</t>
+          <t>Servicios transversales de consulta técnica arancelaria, resoluciones anticipadas, facilitación comercial y herramientas de control del despacho aduanero general.</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Gestiona tu carné y habilitación oficial, presenta pólizas de seguro de caución y transmite declaraciones con firma electrónica.</t>
+          <t>Consulta el Sistema Arancelario Centroamericano (SAC), tramita resoluciones anticipadas y reporta incidentes de contrabando.</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>CAUCA IV (Arts. 22 al 28), RECAUCA IV (Arts. 74 al 85) y Ley Nacional de Aduanas.</t>
+          <t>Convenio sobre el Régimen Arancelario y Aduanero Centroamericano, Acuerdos Comerciales de la OMC y CAUCA/RECAUCA IV.</t>
         </is>
       </c>
       <c r="H23" s="15" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" ht="54" customHeight="1">
       <c r="A24" s="17" t="n">
         <v>18</v>
       </c>
-      <c r="B24" s="40" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="C24" s="40" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="D24" s="35" t="inlineStr">
         <is>
-          <t>Apoderados Especiales Aduaneros</t>
+          <t>Abogados y Notarios</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>Personas individuales mandatarias designadas exclusivamente por una persona jurídica para representarla formalmente en sus despachos aduaneros propios.</t>
+          <t>Profesionales del derecho colegiados activos autorizados para ejercer la fe pública notarial, autorizar traspasos electrónicos de vehículos y emitir razones tributarias ante la SAT.</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
-          <t>Registra tu mandato legal, actualiza tu carné de apoderado y tramita declaraciones DUCA corporativas.</t>
+          <t>Compra papel sellado para protocolos, emite razones electrónicas de timbres fiscales, autoriza traspasos vehiculares (TEV) y presenta avisos notariales.</t>
         </is>
       </c>
       <c r="G24" s="21" t="inlineStr">
         <is>
-          <t>CAUCA IV (Art. 21), RECAUCA IV (Arts. 86 al 90) y Código de Notariado.</t>
+          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales (Decreto 37-92), Ley del ISCV (Decreto 70-94) y Acuerdo de Directorio SAT 08-2020.</t>
         </is>
       </c>
       <c r="H24" s="22" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" ht="54" customHeight="1">
       <c r="A25" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="C25" s="37" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="B25" s="36" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="C25" s="36" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
-          <t>Transportistas Aduaneros</t>
+          <t>Peritos Contadores</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Empresas y conductores autorizados para realizar el traslado de mercancías bajo control aduanero dentro del territorio nacional o en tránsito internacional centroamericano.</t>
+          <t>Técnicos y profesionales contables inscritos ante la SAT facultados para llevar y certificar registros contables, libros tributarios electrónicos y declaraciones juradas de contribuyentes.</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Registra medios de transporte, activa marchamos electrónicos RFID y transmite declaraciones de tránsito DUCA-T.</t>
+          <t>Inscríbete en el Registro de Contadores, habilita el Libro Electrónico Tributario (LET), administra facturación FEL y concilia retenciones tributarias.</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>CAUCA IV (Arts. 18 al 20), RECAUCA IV (Tránsito Aduanero Internacional Terrestre) y Reglamentos de Transporte Centroamericano.</t>
+          <t>Decreto 2450 (Normas de la Profesión Contable), Código de Comercio (Decreto 2-70, Arts. 368 al 381) y Código Tributario (Arts. 112 y 120).</t>
         </is>
       </c>
       <c r="H25" s="15" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" ht="54" customHeight="1">
       <c r="A26" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="40" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="C26" s="40" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="B26" s="39" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="D26" s="35" t="inlineStr">
         <is>
-          <t>Empresas de Entrega Rápida o Courier</t>
+          <t>Auditores</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>Empresas de mensajería y paquetería urgente autorizadas para transportar y desaduanar envíos postales exprés y encomiendas internacionales no comerciales.</t>
+          <t>Contadores Públicos y Auditores (CPA) colegiados activos autorizados para emitir dictámenes periciales de devolución de crédito fiscal, auditorías tributarias y certificar estados financieros.</t>
         </is>
       </c>
       <c r="F26" s="20" t="inlineStr">
         <is>
-          <t>Transmite manifiestos courier, aplica franquicias simplificadas y habilita recintos desconsolidadores de paquetería.</t>
+          <t>Inscribe tu firma de CPA, acredita tu colegiado activo y emite dictámenes vinculantes para la devolución de crédito fiscal bajo el régimen optativo.</t>
         </is>
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>CAUCA IV y RECAUCA IV (Arts. 574 al 596 - Régimen de Envíos de Entrega Rápida o Courier).</t>
+          <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001), Ley del IVA (Decreto 27-92, Art. 25 bis) y Acuerdo de Directorio SAT 07-2007.</t>
         </is>
       </c>
       <c r="H26" s="22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" ht="54" customHeight="1">
       <c r="A27" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B27" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="C27" s="37" t="inlineStr">
-        <is>
-          <t>2. Auxiliares de la Función Pública Aduanera (AFPA)</t>
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="C27" s="36" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>Consolidadores y Desconsolidadores de Carga</t>
+          <t>Gestores Tributarios</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Operadores logísticos autorizados para agrupar o separar mercancías pertenecientes a distintos consignatarios bajo un solo documento matriz de transporte.</t>
+          <t>Personas individuales acreditadas formalmente ante la SAT para representar a terceros en la tramitación presencial de gestiones administrativas tributarias y aduaneras.</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
-          <t>Transmite manifiestos CUSCAR, emite guías hijas y reporta inconsistencias o averías de carga ante la aduana.</t>
+          <t>Tramita y renueva tu gafete oficial de gestor tributario, consulta el padrón activo institucional y gestiona expedientes autorizados en agencias.</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>CAUCA IV y RECAUCA IV (Arts. 102 al 109 - Auxiliares Consolidador y Desconsolidador de Carga).</t>
+          <t>Código Tributario (Decreto 6-91, Art. 22 - Representación) y Normativa Institucional de Acreditación de Gestores de la SAT.</t>
         </is>
       </c>
       <c r="H27" s="15" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" ht="54" customHeight="1">
       <c r="A28" s="17" t="n">
         <v>22</v>
       </c>
-      <c r="B28" s="40" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="C28" s="40" t="inlineStr">
-        <is>
-          <t>3. Regímenes Territoriales y Zonas Especiales</t>
+      <c r="B28" s="39" t="inlineStr">
+        <is>
+          <t>Profesionales</t>
+        </is>
+      </c>
+      <c r="C28" s="39" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales y Auxiliares</t>
         </is>
       </c>
       <c r="D28" s="35" t="inlineStr">
         <is>
-          <t>ZDEEP - Entidades Administradoras</t>
+          <t>Servicios Profesionales</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>Personas jurídicas públicas o privadas autorizadas por ZOLIC y SAT para desarrollar, operar y vigilar la infraestructura de polígonos industriales y logísticos ZDEEP.</t>
+          <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de salud por honorarios, sujetos a regímenes de retención y actualización registral.</t>
         </is>
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Delimita polígonos aduaneros, administra garitas de control y supervisa el perímetro de seguridad de la zona especial.</t>
+          <t>Genera formularios oficiales en Declaraguate, actualiza tu actividad profesional en el RTU, presenta consultas técnicas vinculantes y gestiona retenciones.</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
         <is>
-          <t>Decreto 22-73 (Ley Orgánica de ZOLIC reformada), CAUCA IV, RECAUCA IV y Resoluciones Conjuntas SAT-ZOLIC.</t>
+          <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Código Tributario (Decreto 6-91, Arts. 102 al 105).</t>
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" ht="54" customHeight="1">
       <c r="A29" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="B29" s="37" t="inlineStr">
-        <is>
-          <t>Operadores de Comercio Exterior</t>
-        </is>
-      </c>
-      <c r="C29" s="37" t="inlineStr">
-        <is>
-          <t>3. Regímenes Territoriales y Zonas Especiales</t>
+      <c r="B29" s="36" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="C29" s="36" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
-          <t>ZDEEP - Empresas Usuarias</t>
+          <t>Constitucionales</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Empresas industriales, comerciales o de servicios instaladas y operando dentro de los recintos calificados como ZDEEP para producir o transformar con beneficios fiscales.</t>
+          <t>Instituciones educativas, universidades, comunidades religiosas, misiones diplomáticas y cuerpos consulares que gozan de exención de impuestos por mandato directo de la Carta Magna.</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Ingresa materias primas con suspensión de DAI e IVA, realiza descargos de producción y goza de exenciones tributarias.</t>
+          <t>Inscribe tu personería jurídica exenta en el RTU, emite constancias electrónicas de exención de IVA y timbres, y acredita representación legal.</t>
         </is>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>Decreto 22-73 (Régimen Fiscal ZDEEP), Ley de Actualización Tributaria (Decreto 10-2012) y CAUCA/RECAUCA IV.</t>
+          <t>Constitución Política de la República de Guatemala (Arts. 37, 73, 88), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
         </is>
       </c>
       <c r="H29" s="15" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" ht="54" customHeight="1">
       <c r="A30" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="B30" s="40" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="C30" s="40" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+      <c r="B30" s="39" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="D30" s="35" t="inlineStr">
         <is>
-          <t>Abogados y Notarios</t>
+          <t>Decreto</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>Profesionales del derecho colegiados activos autorizados para ejercer la fe pública notarial, redactar instrumentos públicos y autorizar traspasos electrónicos de vehículos ante la SAT.</t>
+          <t>Personas o entidades beneficiarias de leyes de fomento económico y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso.</t>
         </is>
       </c>
       <c r="F30" s="20" t="inlineStr">
         <is>
-          <t>Compra papel sellado especial para protocolos, adquiere timbres fiscales, realiza traspasos vehiculares electrónicos (TEV) y presenta avisos notariales.</t>
+          <t>Acredita resoluciones ministeriales de calificación de fomento, gestiona exenciones arancelarias temporales y presenta reportes periódicos de cumplimiento.</t>
         </is>
       </c>
       <c r="G30" s="21" t="inlineStr">
         <is>
-          <t>Código de Notariado (Decreto 314), Ley de Timbres Fiscales y de Papel Sellado Especial para Protocolos (Decreto 37-92) y Código Tributario.</t>
+          <t>Decretos específicos de fomento (Decreto 29-89 de Maquilas, Decreto 65-89 de Zonas Francas, Ley de Incentivos para Energías Renovables) y Código Tributario.</t>
         </is>
       </c>
       <c r="H30" s="22" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" ht="54" customHeight="1">
       <c r="A31" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="B31" s="37" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="C31" s="37" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+      <c r="B31" s="36" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="C31" s="36" t="inlineStr">
+        <is>
+          <t>Organizaciones No Lucrativas (Exentas)</t>
         </is>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
-          <t>Peritos Contadores</t>
+          <t>No Lucrativos</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Técnicos y profesionales contables inscritos y autorizados ante la SAT para llevar y firmar registros contables de contribuyentes, certificar estados financieros y realizar gestiones tributarias.</t>
+          <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas, asociaciones civiles sin fines de lucro y cooperativas que solicitan reconocimiento administrativo de exención de ISR e IVA.</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>Inscríbete y actualiza tus datos en el Registro de Contadores, autoriza libros contables computarizados y asocia contribuyentes a tu perfil.</t>
+          <t>Solicita tu resolución formal de exención de ISR, actualiza estatutos y junta directiva en el RTU y emite constancias de retención y exención.</t>
         </is>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>Decreto 2450 (Normas que Regulan el Ejercicio de la Profesión de Contador), Código de Comercio (Decreto 2-70) y Código Tributario (Arts. 112 y 120).</t>
+          <t>Decreto 02-2003 (Ley de ONGs para el Desarrollo), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
         </is>
       </c>
       <c r="H31" s="15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" ht="54" customHeight="1">
       <c r="A32" s="17" t="n">
         <v>26</v>
       </c>
-      <c r="B32" s="40" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="C32" s="40" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+      <c r="B32" s="39" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
         </is>
       </c>
       <c r="D32" s="35" t="inlineStr">
         <is>
-          <t>Gestores Tributarios</t>
+          <t>Entidades del Estado</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>Personas individuales autorizadas y acreditadas formalmente ante la SAT para representar a terceros en la tramitación presencial de gestiones administrativas tributarias y aduaneras.</t>
+          <t>Ministerios de Estado, secretarías, organismos de los poderes Ejecutivo, Legislativo y Judicial, y entidades públicas descentralizadas que operan como agentes de retención del IVA e ISR.</t>
         </is>
       </c>
       <c r="F32" s="20" t="inlineStr">
         <is>
-          <t>Tramita y renueva tu carné oficial de gestor tributario, registra tus datos biométricos y gestiona expedientes autorizados en agencias tributarias.</t>
+          <t>Habilita unidades ejecutoras en el RTU, emite constancias de retención en compras públicas y administra el parque vehicular oficial del Estado.</t>
         </is>
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
-          <t>Acuerdos de Directorio de la SAT sobre Regulación y Acreditación de Gestores Tributarios y Código Tributario.</t>
+          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
         </is>
       </c>
       <c r="H32" s="22" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" ht="54" customHeight="1">
       <c r="A33" s="10" t="n">
         <v>27</v>
       </c>
-      <c r="B33" s="37" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
+      <c r="B33" s="36" t="inlineStr">
+        <is>
+          <t>Entes Exentos</t>
+        </is>
+      </c>
+      <c r="C33" s="36" t="inlineStr">
+        <is>
+          <t>Sector Público y Entidades del Estado</t>
         </is>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
-          <t>Servicios Profesionales</t>
+          <t>Municipalidades</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Profesionales liberales e independientes que prestan servicios técnicos, científicos, jurídicos o de consultoría por honorarios profesionales.</t>
+          <t>Las 340 corporaciones municipales autónomas de la República de Guatemala, mancomunidades y empresas municipales públicas prestadoras de servicios comunitarios.</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr">
         <is>
-          <t>Emite facturas electrónicas FEL por honorarios, liquida retenciones de ISR, actualiza tu colegiado activo y consulta tu solvencia fiscal.</t>
+          <t>Registra autoridades y tesoreros en el RTU, gestiona la exención del impuesto de circulación para flotillas municipales y tramita solvencias institucionales.</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>Ley de Actualización Tributaria (Decreto 10-2012, Libro I) y Ley del IVA (Decreto 27-92).</t>
+          <t>Constitución Política de la República (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
         </is>
       </c>
       <c r="H33" s="15" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="34" ht="54" customHeight="1">
-      <c r="A34" s="17" t="n">
-        <v>28</v>
-      </c>
-      <c r="B34" s="40" t="inlineStr">
-        <is>
-          <t>Profesionales</t>
-        </is>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
-        <is>
-          <t>Servicios Profesionales y Terceras Personas</t>
-        </is>
-      </c>
-      <c r="D34" s="35" t="inlineStr">
-        <is>
-          <t>Auditores</t>
-        </is>
-      </c>
-      <c r="E34" s="19" t="inlineStr">
-        <is>
-          <t>Contadores Públicos y Auditores (CPA) colegiados activos y firmas de auditoría facultados para emitir dictámenes sobre estados financieros, devolución de crédito fiscal e informes de precios de transferencia.</t>
-        </is>
-      </c>
-      <c r="F34" s="20" t="inlineStr">
-        <is>
-          <t>Emite dictámenes de crédito fiscal para exportadores, dictámenes de estados financieros para licitaciones y presenta informes tributarios requeridos por SAT.</t>
-        </is>
-      </c>
-      <c r="G34" s="21" t="inlineStr">
-        <is>
-          <t>Ley de Colegiación Profesional Obligatoria (Decreto 72-2001), Ley del IVA (Decreto 27-92, Art. 23 bis) y Ley de Actualización Tributaria (Decreto 10-2012).</t>
-        </is>
-      </c>
-      <c r="H34" s="22" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" ht="54" customHeight="1">
-      <c r="A35" s="10" t="n">
-        <v>29</v>
-      </c>
-      <c r="B35" s="37" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>Organizaciones No Lucrativas (Exentas)</t>
-        </is>
-      </c>
-      <c r="D35" s="33" t="inlineStr">
-        <is>
-          <t>Constitucionales</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>Instituciones educativas, universidades, comunidades religiosas, misiones diplomáticas y cuerpos consulares que gozan de exención de impuestos por mandato directo de la Carta Magna.</t>
-        </is>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>Inscribe tu personería jurídica exenta en el RTU, emite constancias electrónicas de exención de IVA y timbres, y acredita representación legal.</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="inlineStr">
-        <is>
-          <t>Constitución Política de la República de Guatemala (Arts. 37, 73, 88), Ley del IVA (Art. 8) y Código Tributario (Art. 62).</t>
-        </is>
-      </c>
-      <c r="H35" s="15" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="36" ht="54" customHeight="1">
-      <c r="A36" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="B36" s="40" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="C36" s="40" t="inlineStr">
-        <is>
-          <t>Organizaciones No Lucrativas (Exentas)</t>
-        </is>
-      </c>
-      <c r="D36" s="35" t="inlineStr">
-        <is>
-          <t>Decreto</t>
-        </is>
-      </c>
-      <c r="E36" s="19" t="inlineStr">
-        <is>
-          <t>Personas o entidades beneficiarias de leyes de fomento económico y exenciones tributarias específicas aprobadas mediante decretos legislativos ordinarios del Congreso.</t>
-        </is>
-      </c>
-      <c r="F36" s="20" t="inlineStr">
-        <is>
-          <t>Acredita resoluciones ministeriales de calificación de fomento, gestiona exenciones arancelarias temporales y presenta reportes periódicos de cumplimiento.</t>
-        </is>
-      </c>
-      <c r="G36" s="21" t="inlineStr">
-        <is>
-          <t>Decretos específicos de fomento (Decreto 29-89 de Maquilas, Decreto 65-89 de Zonas Francas, Ley de Incentivos para Energías Renovables) y Código Tributario.</t>
-        </is>
-      </c>
-      <c r="H36" s="22" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" ht="54" customHeight="1">
-      <c r="A37" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="B37" s="37" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="C37" s="37" t="inlineStr">
-        <is>
-          <t>Organizaciones No Lucrativas (Exentas)</t>
-        </is>
-      </c>
-      <c r="D37" s="33" t="inlineStr">
-        <is>
-          <t>No Lucrativos</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>Organizaciones No Gubernamentales (ONGs), fundaciones benéficas, asociaciones civiles sin fines de lucro y cooperativas que solicitan reconocimiento administrativo de exención de ISR e IVA.</t>
-        </is>
-      </c>
-      <c r="F37" s="13" t="inlineStr">
-        <is>
-          <t>Solicita tu resolución formal de exención de ISR, actualiza estatutos y junta directiva en el RTU y emite constancias de retención y exención.</t>
-        </is>
-      </c>
-      <c r="G37" s="14" t="inlineStr">
-        <is>
-          <t>Decreto 02-2003 (Ley de ONGs para el Desarrollo), Ley de Actualización Tributaria (Decreto 10-2012, Art. 11) y Ley del IVA.</t>
-        </is>
-      </c>
-      <c r="H37" s="15" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" ht="54" customHeight="1">
-      <c r="A38" s="17" t="n">
-        <v>32</v>
-      </c>
-      <c r="B38" s="40" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="C38" s="40" t="inlineStr">
-        <is>
-          <t>Sector Público y Entidades del Estado</t>
-        </is>
-      </c>
-      <c r="D38" s="35" t="inlineStr">
-        <is>
-          <t>Entidades del Estado</t>
-        </is>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>Ministerios de Estado, secretarías, organismos de los poderes Ejecutivo, Legislativo y Judicial, y entidades públicas descentralizadas que operan como agentes de retención del IVA e ISR.</t>
-        </is>
-      </c>
-      <c r="F38" s="20" t="inlineStr">
-        <is>
-          <t>Habilita unidades ejecutoras en el RTU, emite constancias de retención en compras públicas y administra el parque vehicular oficial del Estado.</t>
-        </is>
-      </c>
-      <c r="G38" s="21" t="inlineStr">
-        <is>
-          <t>Ley Orgánica del Presupuesto (Decreto 101-97), Ley del IVA, Ley de Contrataciones del Estado (Decreto 57-92) y Código Tributario.</t>
-        </is>
-      </c>
-      <c r="H38" s="22" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="39" ht="54" customHeight="1">
-      <c r="A39" s="10" t="n">
-        <v>33</v>
-      </c>
-      <c r="B39" s="37" t="inlineStr">
-        <is>
-          <t>Entes Exentos</t>
-        </is>
-      </c>
-      <c r="C39" s="37" t="inlineStr">
-        <is>
-          <t>Sector Público y Entidades del Estado</t>
-        </is>
-      </c>
-      <c r="D39" s="33" t="inlineStr">
-        <is>
-          <t>Municipalidades</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="inlineStr">
-        <is>
-          <t>Las 340 corporaciones municipales autónomas de la República de Guatemala, mancomunidades y empresas municipales públicas prestadoras de servicios comunitarios.</t>
-        </is>
-      </c>
-      <c r="F39" s="13" t="inlineStr">
-        <is>
-          <t>Registra autoridades y tesoreros en el RTU, gestiona la exención del impuesto de circulación para flotillas municipales y tramita solvencias institucionales.</t>
-        </is>
-      </c>
-      <c r="G39" s="14" t="inlineStr">
-        <is>
-          <t>Constitución Política de la República (Art. 257), Código Municipal (Decreto 12-2002) y Ley del ISCV (Decreto 70-94).</t>
-        </is>
-      </c>
-      <c r="H39" s="15" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="48" t="inlineStr"/>
-      <c r="B40" s="49" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="47" t="inlineStr"/>
+      <c r="B34" s="48" t="inlineStr">
         <is>
           <t>TOTAL PORTAL WEB SAT</t>
         </is>
       </c>
-      <c r="C40" s="50" t="inlineStr">
+      <c r="C34" s="49" t="inlineStr">
         <is>
           <t>4 Segmentos Oficiales</t>
         </is>
       </c>
-      <c r="D40" s="50" t="inlineStr">
-        <is>
-          <t>33 Categorías</t>
-        </is>
-      </c>
-      <c r="E40" s="50" t="inlineStr">
+      <c r="D34" s="49" t="inlineStr">
+        <is>
+          <t>27 Categorías</t>
+        </is>
+      </c>
+      <c r="E34" s="49" t="inlineStr">
         <is>
           <t>100% de la arquitectura de información clasificada</t>
         </is>
       </c>
-      <c r="F40" s="48" t="inlineStr"/>
-      <c r="G40" s="48" t="inlineStr"/>
-      <c r="H40" s="53">
-        <f>SUM(H7:H39)</f>
+      <c r="F34" s="47" t="inlineStr"/>
+      <c r="G34" s="47" t="inlineStr"/>
+      <c r="H34" s="52">
+        <f>SUM(H7:H33)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:H39"/>
+  <autoFilter ref="A6:H33"/>
   <mergeCells count="2">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A2:H3"/>

</xml_diff>